<commit_message>
Update dashboards - 2026-09-07
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1060,8 +1060,8 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C5" s="51" t="n">
-        <v>46023</v>
+      <c r="C5" s="52" t="n">
+        <v>46113</v>
       </c>
       <c r="D5" s="45" t="inlineStr">
         <is>
@@ -1074,19 +1074,19 @@
         </is>
       </c>
       <c r="F5" s="24" t="n">
+        <v>8121516.5</v>
+      </c>
+      <c r="G5" s="24" t="n">
         <v>7966430.3</v>
       </c>
-      <c r="G5" s="24" t="n">
+      <c r="H5" s="24" t="n">
         <v>7855631.5</v>
       </c>
-      <c r="H5" s="24" t="n">
+      <c r="I5" s="24" t="n">
         <v>7774506.8</v>
       </c>
-      <c r="I5" s="24" t="n">
+      <c r="J5" s="24" t="n">
         <v>7621432.3</v>
-      </c>
-      <c r="J5" s="24" t="n">
-        <v>7510528.3</v>
       </c>
       <c r="K5" s="46" t="n"/>
       <c r="L5" s="28" t="inlineStr">
@@ -1135,8 +1135,8 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C6" s="51" t="n">
-        <v>46023</v>
+      <c r="C6" s="52" t="n">
+        <v>46113</v>
       </c>
       <c r="D6" s="45" t="inlineStr">
         <is>
@@ -1149,19 +1149,19 @@
         </is>
       </c>
       <c r="F6" s="25" t="n">
+        <v>0.01946746461837501</v>
+      </c>
+      <c r="G6" s="25" t="n">
         <v>0.01410437849585988</v>
       </c>
-      <c r="G6" s="25" t="n">
+      <c r="H6" s="25" t="n">
         <v>0.0104347069321491</v>
       </c>
-      <c r="H6" s="25" t="n">
+      <c r="I6" s="25" t="n">
         <v>0.02008474181421249</v>
       </c>
-      <c r="I6" s="25" t="n">
+      <c r="J6" s="25" t="n">
         <v>0.0147664712214719</v>
-      </c>
-      <c r="J6" s="25" t="n">
-        <v>0.007273424182290045</v>
       </c>
       <c r="K6" s="46" t="n"/>
       <c r="L6" s="28" t="inlineStr">

</xml_diff>

<commit_message>
Update dashboards - 2026-09-08
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1293,7 +1293,7 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="52" t="n">
+      <c r="C8" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D8" s="45" t="inlineStr">
@@ -1486,7 +1486,7 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="52" t="n">
+      <c r="N10" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O10" s="45" t="inlineStr">
@@ -1565,7 +1565,7 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="52" t="n">
+      <c r="N11" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O11" s="45" t="inlineStr">
@@ -1640,7 +1640,7 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="52" t="n">
+      <c r="N12" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O12" s="45" t="inlineStr">
@@ -3680,7 +3680,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="52" t="n">
+      <c r="N39" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O39" s="45" t="inlineStr">
@@ -3755,7 +3755,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="52" t="n">
+      <c r="N40" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O40" s="45" t="inlineStr">

</xml_diff>

<commit_message>
Update dashboards - 2026-09-09
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1099,7 +1099,7 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="52" t="n">
+      <c r="N5" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O5" s="45" t="inlineStr">
@@ -2500,8 +2500,8 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="51" t="n">
-        <v>46174</v>
+      <c r="C24" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D24" s="45" t="inlineStr">
         <is>
@@ -2514,19 +2514,19 @@
         </is>
       </c>
       <c r="F24" s="38" t="n">
-        <v>0.005013854980292054</v>
+        <v>0.002069337953391592</v>
       </c>
       <c r="G24" s="38" t="n">
-        <v>-0.00392895391127901</v>
+        <v>0.004986963805690525</v>
       </c>
       <c r="H24" s="38" t="n">
-        <v>0.008723867563298793</v>
+        <v>-0.001636032119741393</v>
       </c>
       <c r="I24" s="38" t="n">
-        <v>0.008102056603516816</v>
+        <v>0.008761168564920929</v>
       </c>
       <c r="J24" s="38" t="n">
-        <v>0.0008464850167981819</v>
+        <v>0.008334847450631955</v>
       </c>
       <c r="K24" s="46" t="n"/>
       <c r="L24" s="28" t="inlineStr">
@@ -2579,8 +2579,8 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="51" t="n">
-        <v>46174</v>
+      <c r="C25" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D25" s="45" t="inlineStr">
         <is>
@@ -2593,19 +2593,19 @@
         </is>
       </c>
       <c r="F25" s="38" t="n">
-        <v>0.001951572292765213</v>
+        <v>0.004001237090364151</v>
       </c>
       <c r="G25" s="38" t="n">
-        <v>0.001109630592487365</v>
+        <v>0.002058428469037255</v>
       </c>
       <c r="H25" s="38" t="n">
-        <v>0.002171973058996635</v>
+        <v>0.001101254055870582</v>
       </c>
       <c r="I25" s="38" t="n">
-        <v>0.003192546663167928</v>
+        <v>0.002229132702467274</v>
       </c>
       <c r="J25" s="38" t="n">
-        <v>0.001614188463588073</v>
+        <v>0.002637510626163131</v>
       </c>
       <c r="K25" s="46" t="n"/>
       <c r="L25" s="28" t="n"/>
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46269</v>
+        <v>46273</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,7 +2936,7 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
-        <v>2.33</v>
+        <v>2.34</v>
       </c>
       <c r="R29" s="45" t="n">
         <v>2.33</v>
@@ -2948,7 +2948,7 @@
         <v>2.33</v>
       </c>
       <c r="U29" s="21" t="n">
-        <v>2.31</v>
+        <v>2.33</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46269</v>
+        <v>46273</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,19 +3015,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
-        <v>2.35</v>
+        <v>2.37</v>
       </c>
       <c r="R30" s="45" t="n">
         <v>2.35</v>
       </c>
       <c r="S30" s="45" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="T30" s="45" t="n">
         <v>2.34</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.35</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.31</v>
       </c>
     </row>
     <row r="31">
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,16 +4361,16 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.37</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.34</v>
-      </c>
-      <c r="R48" s="45" t="n">
-        <v>4.39</v>
       </c>
       <c r="S48" s="45" t="n">
         <v>4.39</v>
       </c>
       <c r="T48" s="45" t="n">
-        <v>4.34</v>
+        <v>4.39</v>
       </c>
       <c r="U48" s="21" t="n">
         <v>4.34</v>
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.54</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.52</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.54</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.55</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.49</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.48</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.77</v>
-      </c>
-      <c r="R50" s="45" t="n">
-        <v>4.79</v>
       </c>
       <c r="S50" s="45" t="n">
         <v>4.79</v>
       </c>
       <c r="T50" s="45" t="n">
+        <v>4.79</v>
+      </c>
+      <c r="U50" s="21" t="n">
         <v>4.75</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.73</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46268</v>
+        <v>46273</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,19 +4641,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.37</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.34</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
+        <v>6.34</v>
+      </c>
+      <c r="T52" s="9" t="n">
         <v>6.37</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.37</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>6.34</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.27</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-09-10
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1228,7 +1228,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>4.7487</v>
+        <v>4.4164</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.54</v>
@@ -1720,7 +1720,7 @@
         </is>
       </c>
       <c r="N13" s="52" t="n">
-        <v>46258</v>
+        <v>46265</v>
       </c>
       <c r="O13" s="45" t="inlineStr">
         <is>
@@ -1736,16 +1736,16 @@
         <v>206000</v>
       </c>
       <c r="R13" s="24" t="n">
+        <v>207000</v>
+      </c>
+      <c r="S13" s="24" t="n">
         <v>204000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>207000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>212000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>200000</v>
       </c>
     </row>
     <row r="14">
@@ -1795,7 +1795,7 @@
         </is>
       </c>
       <c r="N14" s="52" t="n">
-        <v>46251</v>
+        <v>46258</v>
       </c>
       <c r="O14" s="45" t="inlineStr">
         <is>
@@ -1808,19 +1808,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1779000</v>
+        <v>1774000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1775000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1771000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1796000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1781000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1799000</v>
       </c>
     </row>
     <row r="15">
@@ -2390,8 +2390,8 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="51" t="n">
-        <v>46204</v>
+      <c r="N22" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O22" s="45" t="inlineStr">
         <is>
@@ -2404,19 +2404,19 @@
         </is>
       </c>
       <c r="Q22" s="38" t="n">
-        <v>-0.0002809580670085632</v>
+        <v>0.003999132564547425</v>
       </c>
       <c r="R22" s="38" t="n">
-        <v>-0.001122570686872826</v>
+        <v>0.0007468069216873818</v>
       </c>
       <c r="S22" s="38" t="n">
-        <v>0.004529844434762564</v>
+        <v>-0.001255864953080388</v>
       </c>
       <c r="T22" s="38" t="n">
-        <v>0.01090075327249296</v>
+        <v>0.005145423904755253</v>
       </c>
       <c r="U22" s="23" t="n">
-        <v>0.007760893971436644</v>
+        <v>0.01080359860874536</v>
       </c>
     </row>
     <row r="23">
@@ -2460,8 +2460,8 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="51" t="n">
-        <v>46204</v>
+      <c r="N23" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O23" s="45" t="inlineStr">
         <is>
@@ -2474,19 +2474,19 @@
         </is>
       </c>
       <c r="Q23" s="38" t="n">
-        <v>0.04656510491520538</v>
+        <v>0.05413622452737953</v>
       </c>
       <c r="R23" s="38" t="n">
-        <v>0.05535301530395638</v>
+        <v>0.0480424072675253</v>
       </c>
       <c r="S23" s="38" t="n">
-        <v>0.05825059229310237</v>
+        <v>0.05575734704467192</v>
       </c>
       <c r="T23" s="38" t="n">
-        <v>0.05703159391825534</v>
+        <v>0.05879732438762639</v>
       </c>
       <c r="U23" s="23" t="n">
-        <v>0.04280841579142882</v>
+        <v>0.05693000575666253</v>
       </c>
     </row>
     <row r="24">
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,10 +2936,10 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.34</v>
-      </c>
-      <c r="R29" s="45" t="n">
-        <v>2.33</v>
       </c>
       <c r="S29" s="45" t="n">
         <v>2.33</v>
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,16 +3018,16 @@
         <v>2.37</v>
       </c>
       <c r="R30" s="45" t="n">
-        <v>2.35</v>
+        <v>2.37</v>
       </c>
       <c r="S30" s="45" t="n">
         <v>2.35</v>
       </c>
       <c r="T30" s="45" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="U30" s="21" t="n">
         <v>2.34</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.35</v>
       </c>
     </row>
     <row r="31">
@@ -3871,7 +3871,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="D42" s="45" t="inlineStr">
         <is>
@@ -3884,19 +3884,19 @@
         </is>
       </c>
       <c r="F42" s="39" t="n">
+        <v>3980000</v>
+      </c>
+      <c r="G42" s="39" t="n">
         <v>4060000</v>
       </c>
-      <c r="G42" s="39" t="n">
+      <c r="H42" s="39" t="n">
         <v>4130000</v>
       </c>
-      <c r="H42" s="39" t="n">
+      <c r="I42" s="39" t="n">
         <v>4190000</v>
       </c>
-      <c r="I42" s="39" t="n">
+      <c r="J42" s="39" t="n">
         <v>4040000</v>
-      </c>
-      <c r="J42" s="39" t="n">
-        <v>4010000</v>
       </c>
       <c r="K42" s="7" t="n"/>
       <c r="L42" s="28" t="n"/>
@@ -3942,7 +3942,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="D43" s="45" t="inlineStr">
         <is>
@@ -3955,7 +3955,7 @@
         </is>
       </c>
       <c r="F43" s="38" t="n">
-        <v>0.007444168734491315</v>
+        <v>-0.01240694789081886</v>
       </c>
       <c r="G43" s="38" t="n">
         <v/>
@@ -4142,7 +4142,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="52" t="n">
+      <c r="C46" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D46" s="45" t="inlineStr">
@@ -4229,7 +4229,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="52" t="n">
+      <c r="C47" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D47" s="45" t="inlineStr">
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4308,7 +4308,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="52" t="n">
+      <c r="C48" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D48" s="45" t="inlineStr">
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46269</v>
+        <v>46273</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,19 +4361,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.37</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.34</v>
-      </c>
-      <c r="S48" s="45" t="n">
-        <v>4.39</v>
       </c>
       <c r="T48" s="45" t="n">
         <v>4.39</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>4.34</v>
+        <v>4.39</v>
       </c>
     </row>
     <row r="49">
@@ -4383,7 +4383,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="52" t="n">
+      <c r="C49" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D49" s="45" t="inlineStr">
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46269</v>
+        <v>46273</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.54</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.52</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.54</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.55</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.49</v>
       </c>
     </row>
     <row r="50">
@@ -4462,7 +4462,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="52" t="n">
+      <c r="C50" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D50" s="45" t="inlineStr">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46269</v>
+        <v>46273</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.78</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.77</v>
-      </c>
-      <c r="S50" s="45" t="n">
-        <v>4.79</v>
       </c>
       <c r="T50" s="45" t="n">
         <v>4.79</v>
       </c>
       <c r="U50" s="21" t="n">
-        <v>4.75</v>
+        <v>4.79</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4537,7 +4537,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="52" t="n">
+      <c r="C51" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D51" s="45" t="inlineStr">
@@ -4577,7 +4577,7 @@
         </is>
       </c>
       <c r="N51" s="52" t="n">
-        <v>46265</v>
+        <v>46272</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
         <is>
@@ -4590,19 +4590,19 @@
         </is>
       </c>
       <c r="Q51" s="45" t="n">
+        <v>6.76</v>
+      </c>
+      <c r="R51" s="45" t="n">
         <v>6.71</v>
       </c>
-      <c r="R51" s="45" t="n">
+      <c r="S51" s="45" t="n">
         <v>6.66</v>
       </c>
-      <c r="S51" s="45" t="n">
+      <c r="T51" s="45" t="n">
         <v>6.65</v>
       </c>
-      <c r="T51" s="45" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.67</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.69</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,16 +4641,16 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.37</v>
-      </c>
-      <c r="R52" s="9" t="n">
-        <v>6.34</v>
       </c>
       <c r="S52" s="9" t="n">
         <v>6.34</v>
       </c>
       <c r="T52" s="9" t="n">
-        <v>6.37</v>
+        <v>6.34</v>
       </c>
       <c r="U52" s="22" t="n">
         <v>6.37</v>

</xml_diff>

<commit_message>
Update dashboards - 2026-09-11
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -949,7 +949,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="52" t="n">
+      <c r="N3" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O3" s="45" t="inlineStr">
@@ -1020,7 +1020,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="52" t="n">
+      <c r="N4" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O4" s="45" t="inlineStr">
@@ -1174,7 +1174,7 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="52" t="n">
+      <c r="N6" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O6" s="45" t="inlineStr">
@@ -1253,7 +1253,7 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="52" t="n">
+      <c r="N7" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O7" s="45" t="inlineStr">
@@ -1332,7 +1332,7 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="52" t="n">
+      <c r="N8" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O8" s="45" t="inlineStr">
@@ -1411,7 +1411,7 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="52" t="n">
+      <c r="N9" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O9" s="45" t="inlineStr">
@@ -1873,7 +1873,7 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="52" t="n">
+      <c r="N15" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O15" s="45" t="inlineStr">
@@ -2086,8 +2086,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="51" t="n">
-        <v>46204</v>
+      <c r="N18" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O18" s="45" t="inlineStr">
         <is>
@@ -2100,19 +2100,19 @@
         </is>
       </c>
       <c r="Q18" s="38" t="n">
+        <v>0.003960181843858157</v>
+      </c>
+      <c r="R18" s="38" t="n">
         <v>0.0007366914435544825</v>
       </c>
-      <c r="R18" s="38" t="n">
+      <c r="S18" s="38" t="n">
         <v>-0.004224816530380648</v>
       </c>
-      <c r="S18" s="38" t="n">
+      <c r="T18" s="38" t="n">
         <v>0.004729142286413968</v>
       </c>
-      <c r="T18" s="38" t="n">
+      <c r="U18" s="23" t="n">
         <v>0.006400377846336402</v>
-      </c>
-      <c r="U18" s="23" t="n">
-        <v>0.008651438343614481</v>
       </c>
     </row>
     <row r="19" ht="31.5" customHeight="1">
@@ -2161,8 +2161,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="51" t="n">
-        <v>46204</v>
+      <c r="N19" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O19" s="45" t="inlineStr">
         <is>
@@ -2175,19 +2175,19 @@
         </is>
       </c>
       <c r="Q19" s="38" t="n">
+        <v>0.03353016322755652</v>
+      </c>
+      <c r="R19" s="38" t="n">
         <v>0.03303856050706308</v>
       </c>
-      <c r="R19" s="38" t="n">
+      <c r="S19" s="38" t="n">
         <v>0.03463530729385406</v>
       </c>
-      <c r="S19" s="38" t="n">
+      <c r="T19" s="38" t="n">
         <v>0.04166614684049648</v>
       </c>
-      <c r="T19" s="38" t="n">
+      <c r="U19" s="23" t="n">
         <v>0.03779245836741563</v>
-      </c>
-      <c r="U19" s="23" t="n">
-        <v>0.03285957752865201</v>
       </c>
     </row>
     <row r="20">
@@ -2236,8 +2236,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="51" t="n">
-        <v>46204</v>
+      <c r="N20" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O20" s="45" t="inlineStr">
         <is>
@@ -2250,19 +2250,19 @@
         </is>
       </c>
       <c r="Q20" s="38" t="n">
+        <v>0.002897956881014574</v>
+      </c>
+      <c r="R20" s="38" t="n">
         <v>0.002154345141564873</v>
       </c>
-      <c r="R20" s="38" t="n">
+      <c r="S20" s="38" t="n">
         <v>-0.0001666066684318235</v>
       </c>
-      <c r="S20" s="38" t="n">
+      <c r="T20" s="38" t="n">
         <v>0.002080954496262777</v>
       </c>
-      <c r="T20" s="38" t="n">
+      <c r="U20" s="23" t="n">
         <v>0.00376460730477457</v>
-      </c>
-      <c r="U20" s="23" t="n">
-        <v>0.001957950538511444</v>
       </c>
     </row>
     <row r="21">
@@ -2311,8 +2311,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="51" t="n">
-        <v>46204</v>
+      <c r="N21" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O21" s="45" t="inlineStr">
         <is>
@@ -2325,19 +2325,19 @@
         </is>
       </c>
       <c r="Q21" s="38" t="n">
+        <v>0.02446163178647254</v>
+      </c>
+      <c r="R21" s="38" t="n">
         <v>0.0246651778923092</v>
       </c>
-      <c r="R21" s="38" t="n">
+      <c r="S21" s="38" t="n">
         <v>0.02565785056369746</v>
       </c>
-      <c r="S21" s="38" t="n">
+      <c r="T21" s="38" t="n">
         <v>0.02822942063611032</v>
       </c>
-      <c r="T21" s="38" t="n">
+      <c r="U21" s="23" t="n">
         <v>0.02743309430968526</v>
-      </c>
-      <c r="U21" s="23" t="n">
-        <v>0.0260216770548682</v>
       </c>
     </row>
     <row r="22">
@@ -2351,7 +2351,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="52" t="n">
+      <c r="C22" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D22" s="45" t="inlineStr">
@@ -2426,7 +2426,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="52" t="n">
+      <c r="C23" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D23" s="45" t="inlineStr">
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,13 +2936,13 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.34</v>
-      </c>
-      <c r="S29" s="45" t="n">
-        <v>2.33</v>
       </c>
       <c r="T29" s="45" t="n">
         <v>2.33</v>
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,19 +3015,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
-        <v>2.37</v>
+        <v>2.4</v>
       </c>
       <c r="R30" s="45" t="n">
         <v>2.37</v>
       </c>
       <c r="S30" s="45" t="n">
-        <v>2.35</v>
+        <v>2.37</v>
       </c>
       <c r="T30" s="45" t="n">
         <v>2.35</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.34</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="31">
@@ -3226,7 +3226,7 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="52" t="n">
+      <c r="N33" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O33" s="45" t="inlineStr">
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,16 +4361,16 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.39</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.37</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.34</v>
-      </c>
-      <c r="T48" s="45" t="n">
-        <v>4.39</v>
       </c>
       <c r="U48" s="21" t="n">
         <v>4.39</v>
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.61</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.57</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.54</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.52</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.54</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.55</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,16 +4515,16 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.83</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.8</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.78</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.77</v>
-      </c>
-      <c r="T50" s="45" t="n">
-        <v>4.79</v>
       </c>
       <c r="U50" s="21" t="n">
         <v>4.79</v>
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,19 +4641,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.38</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.37</v>
-      </c>
-      <c r="S52" s="9" t="n">
-        <v>6.34</v>
       </c>
       <c r="T52" s="9" t="n">
         <v>6.34</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>6.37</v>
+        <v>6.34</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-09-12
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,16 +2936,16 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.34</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.34</v>
-      </c>
-      <c r="T29" s="45" t="n">
-        <v>2.33</v>
       </c>
       <c r="U29" s="21" t="n">
         <v>2.33</v>
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,16 +3015,16 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.4</v>
-      </c>
-      <c r="R30" s="45" t="n">
-        <v>2.37</v>
       </c>
       <c r="S30" s="45" t="n">
         <v>2.37</v>
       </c>
       <c r="T30" s="45" t="n">
-        <v>2.35</v>
+        <v>2.37</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.35</v>
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,19 +4361,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.43</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.39</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.37</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.34</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.39</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.61</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.57</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.54</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.52</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.54</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.95</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.83</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.8</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.78</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.77</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.79</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-09-14
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1060,7 +1060,7 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C5" s="52" t="n">
+      <c r="C5" s="51" t="n">
         <v>46113</v>
       </c>
       <c r="D5" s="45" t="inlineStr">
@@ -1135,7 +1135,7 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C6" s="52" t="n">
+      <c r="C6" s="51" t="n">
         <v>46113</v>
       </c>
       <c r="D6" s="45" t="inlineStr">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,13 +4644,13 @@
         <v>6.46</v>
       </c>
       <c r="R52" s="9" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="S52" s="9" t="n">
         <v>6.38</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.37</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>6.34</v>
       </c>
       <c r="U52" s="22" t="n">
         <v>6.34</v>

</xml_diff>

<commit_message>
Update dashboards - 2026-09-15
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1293,8 +1293,10 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="51" t="n">
-        <v>46204</v>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'RECPROUSM156N' not found in values file."</t>
+        </is>
       </c>
       <c r="D8" s="45" t="inlineStr">
         <is>
@@ -1307,19 +1309,19 @@
         </is>
       </c>
       <c r="F8" s="45" t="n">
-        <v>0.76</v>
+        <v>1</v>
       </c>
       <c r="G8" s="45" t="n">
-        <v>0.5600000000000001</v>
+        <v>1</v>
       </c>
       <c r="H8" s="45" t="n">
-        <v>0.54</v>
+        <v>1</v>
       </c>
       <c r="I8" s="45" t="n">
-        <v>0.46</v>
+        <v>1</v>
       </c>
       <c r="J8" s="45" t="n">
-        <v>0.54</v>
+        <v>1</v>
       </c>
       <c r="K8" s="46" t="n"/>
       <c r="L8" s="28" t="inlineStr">
@@ -1411,8 +1413,10 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="51" t="n">
-        <v>46235</v>
+      <c r="N9" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'EMRATIO' not found in values file."</t>
+        </is>
       </c>
       <c r="O9" s="45" t="inlineStr">
         <is>
@@ -1425,19 +1429,19 @@
         </is>
       </c>
       <c r="Q9" s="45" t="n">
-        <v>59.1</v>
+        <v>1</v>
       </c>
       <c r="R9" s="45" t="n">
-        <v>58.9</v>
+        <v>1</v>
       </c>
       <c r="S9" s="45" t="n">
-        <v>59</v>
+        <v>1</v>
       </c>
       <c r="T9" s="45" t="n">
-        <v>59.2</v>
+        <v>1</v>
       </c>
       <c r="U9" s="21" t="n">
-        <v>59.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1526,8 +1530,10 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="51" t="n">
-        <v>46204</v>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCEDGC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D11" s="45" t="inlineStr">
         <is>
@@ -1540,19 +1546,19 @@
         </is>
       </c>
       <c r="F11" s="25" t="n">
-        <v>-0.01390979158115568</v>
+        <v>1</v>
       </c>
       <c r="G11" s="25" t="n">
-        <v>0.00767463235294108</v>
+        <v>1</v>
       </c>
       <c r="H11" s="25" t="n">
-        <v>0.01091753774680604</v>
+        <v>1</v>
       </c>
       <c r="I11" s="25" t="n">
-        <v>-0.01148105625717566</v>
+        <v>1</v>
       </c>
       <c r="J11" s="25" t="n">
-        <v>0.01363932594730488</v>
+        <v>1</v>
       </c>
       <c r="K11" s="46" t="n"/>
       <c r="L11" s="28" t="inlineStr">
@@ -1601,8 +1607,10 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="51" t="n">
-        <v>46204</v>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCEDGC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D12" s="45" t="inlineStr">
         <is>
@@ -1615,19 +1623,19 @@
         </is>
       </c>
       <c r="F12" s="25" t="n">
-        <v>0.009618976466193458</v>
+        <v>1</v>
       </c>
       <c r="G12" s="25" t="n">
-        <v>0.03727707081697323</v>
+        <v>1</v>
       </c>
       <c r="H12" s="25" t="n">
-        <v>0.02752986730887292</v>
+        <v>1</v>
       </c>
       <c r="I12" s="25" t="n">
-        <v>-0.005773672055427252</v>
+        <v>1</v>
       </c>
       <c r="J12" s="25" t="n">
-        <v>-0.000734248084071364</v>
+        <v>1</v>
       </c>
       <c r="K12" s="46" t="n"/>
       <c r="L12" s="28" t="inlineStr">
@@ -2500,7 +2508,7 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="52" t="n">
+      <c r="C24" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D24" s="45" t="inlineStr">
@@ -2579,7 +2587,7 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="52" t="n">
+      <c r="C25" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D25" s="45" t="inlineStr">
@@ -2923,7 +2931,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,19 +2944,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.32</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.34</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.34</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.33</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3010,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,19 +3023,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.36</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.4</v>
-      </c>
-      <c r="S30" s="45" t="n">
-        <v>2.37</v>
       </c>
       <c r="T30" s="45" t="n">
         <v>2.37</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.35</v>
+        <v>2.37</v>
       </c>
     </row>
     <row r="31">
@@ -4269,7 +4277,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4356,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,19 +4369,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.63</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.56</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.43</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.39</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.37</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.34</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4431,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4444,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.75</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.61</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.57</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.54</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.52</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4510,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4523,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.96</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.95</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.83</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.8</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.78</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.77</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4628,7 +4636,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,19 +4649,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>6.46</v>
+        <v>6.44</v>
       </c>
       <c r="R52" s="9" t="n">
         <v>6.46</v>
       </c>
       <c r="S52" s="9" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="T52" s="9" t="n">
         <v>6.38</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.37</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.34</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-09-16
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1228,7 +1228,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>4.4164</v>
+        <v>5.1028</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.54</v>
@@ -1293,10 +1293,8 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'RECPROUSM156N' not found in values file."</t>
-        </is>
+      <c r="C8" s="51" t="n">
+        <v>46204</v>
       </c>
       <c r="D8" s="45" t="inlineStr">
         <is>
@@ -1309,19 +1307,19 @@
         </is>
       </c>
       <c r="F8" s="45" t="n">
-        <v>1</v>
+        <v>0.76</v>
       </c>
       <c r="G8" s="45" t="n">
-        <v>1</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H8" s="45" t="n">
-        <v>1</v>
+        <v>0.54</v>
       </c>
       <c r="I8" s="45" t="n">
-        <v>1</v>
+        <v>0.46</v>
       </c>
       <c r="J8" s="45" t="n">
-        <v>1</v>
+        <v>0.54</v>
       </c>
       <c r="K8" s="46" t="n"/>
       <c r="L8" s="28" t="inlineStr">
@@ -1413,10 +1411,8 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'EMRATIO' not found in values file."</t>
-        </is>
+      <c r="N9" s="51" t="n">
+        <v>46235</v>
       </c>
       <c r="O9" s="45" t="inlineStr">
         <is>
@@ -1429,19 +1425,19 @@
         </is>
       </c>
       <c r="Q9" s="45" t="n">
-        <v>1</v>
+        <v>59.1</v>
       </c>
       <c r="R9" s="45" t="n">
-        <v>1</v>
+        <v>58.9</v>
       </c>
       <c r="S9" s="45" t="n">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="T9" s="45" t="n">
-        <v>1</v>
+        <v>59.2</v>
       </c>
       <c r="U9" s="21" t="n">
-        <v>1</v>
+        <v>59.1</v>
       </c>
     </row>
     <row r="10">
@@ -1530,10 +1526,8 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCEDGC96' not found in values file."</t>
-        </is>
+      <c r="C11" s="51" t="n">
+        <v>46204</v>
       </c>
       <c r="D11" s="45" t="inlineStr">
         <is>
@@ -1546,19 +1540,19 @@
         </is>
       </c>
       <c r="F11" s="25" t="n">
-        <v>1</v>
+        <v>-0.01390979158115568</v>
       </c>
       <c r="G11" s="25" t="n">
-        <v>1</v>
+        <v>0.00767463235294108</v>
       </c>
       <c r="H11" s="25" t="n">
-        <v>1</v>
+        <v>0.01091753774680604</v>
       </c>
       <c r="I11" s="25" t="n">
-        <v>1</v>
+        <v>-0.01148105625717566</v>
       </c>
       <c r="J11" s="25" t="n">
-        <v>1</v>
+        <v>0.01363932594730488</v>
       </c>
       <c r="K11" s="46" t="n"/>
       <c r="L11" s="28" t="inlineStr">
@@ -1607,10 +1601,8 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCEDGC96' not found in values file."</t>
-        </is>
+      <c r="C12" s="51" t="n">
+        <v>46204</v>
       </c>
       <c r="D12" s="45" t="inlineStr">
         <is>
@@ -1623,19 +1615,19 @@
         </is>
       </c>
       <c r="F12" s="25" t="n">
-        <v>1</v>
+        <v>0.009618976466193458</v>
       </c>
       <c r="G12" s="25" t="n">
-        <v>1</v>
+        <v>0.03727707081697323</v>
       </c>
       <c r="H12" s="25" t="n">
-        <v>1</v>
+        <v>0.02752986730887292</v>
       </c>
       <c r="I12" s="25" t="n">
-        <v>1</v>
+        <v>-0.005773672055427252</v>
       </c>
       <c r="J12" s="25" t="n">
-        <v>1</v>
+        <v>-0.000734248084071364</v>
       </c>
       <c r="K12" s="46" t="n"/>
       <c r="L12" s="28" t="inlineStr">
@@ -1968,8 +1960,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="51" t="n">
-        <v>46204</v>
+      <c r="C17" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D17" s="45" t="inlineStr">
         <is>
@@ -1982,19 +1974,19 @@
         </is>
       </c>
       <c r="F17" s="25" t="n">
-        <v>-0.005819766896853373</v>
+        <v>0.01240741855056227</v>
       </c>
       <c r="G17" s="25" t="n">
-        <v>0.002453693069100149</v>
+        <v>-0.005366991635299634</v>
       </c>
       <c r="H17" s="25" t="n">
+        <v>0.00312584835132701</v>
+      </c>
+      <c r="I17" s="25" t="n">
         <v>0.009346631589902232</v>
       </c>
-      <c r="I17" s="25" t="n">
+      <c r="J17" s="25" t="n">
         <v>0.006742589318751824</v>
-      </c>
-      <c r="J17" s="25" t="n">
-        <v>0.01717978949867671</v>
       </c>
       <c r="K17" s="46" t="n"/>
       <c r="L17" s="29" t="inlineStr">
@@ -2055,8 +2047,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="51" t="n">
-        <v>46204</v>
+      <c r="C18" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D18" s="45" t="inlineStr">
         <is>
@@ -2069,19 +2061,19 @@
         </is>
       </c>
       <c r="F18" s="25" t="n">
-        <v>0.05009241229083468</v>
+        <v>0.06014763635267802</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>0.06753173107393633</v>
+        <v>0.05032033271185719</v>
       </c>
       <c r="H18" s="25" t="n">
+        <v>0.06824752183509293</v>
+      </c>
+      <c r="I18" s="25" t="n">
         <v>0.0723275853623377</v>
       </c>
-      <c r="I18" s="25" t="n">
+      <c r="J18" s="25" t="n">
         <v>0.05073763706982706</v>
-      </c>
-      <c r="J18" s="25" t="n">
-        <v>0.04240611939906461</v>
       </c>
       <c r="K18" s="46" t="n"/>
       <c r="L18" s="28" t="inlineStr">
@@ -2931,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2944,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.34</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.32</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.34</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.33</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.34</v>
       </c>
     </row>
     <row r="30">
@@ -3010,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3023,16 +3015,16 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.37</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.36</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.4</v>
-      </c>
-      <c r="T30" s="45" t="n">
-        <v>2.37</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.37</v>
@@ -3838,8 +3830,8 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="51" t="n">
-        <v>46204</v>
+      <c r="N41" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O41" s="45" t="inlineStr">
         <is>
@@ -3852,19 +3844,19 @@
         </is>
       </c>
       <c r="Q41" s="38" t="n">
-        <v>-0.01312649164677793</v>
+        <v>0.006053268765133124</v>
       </c>
       <c r="R41" s="38" t="n">
+        <v>-0.01431980906921249</v>
+      </c>
+      <c r="S41" s="38" t="n">
         <v>-0.007109004739336622</v>
       </c>
-      <c r="S41" s="38" t="n">
+      <c r="T41" s="38" t="n">
         <v>0.01199040767386084</v>
       </c>
-      <c r="T41" s="38" t="n">
+      <c r="U41" s="23" t="n">
         <v>0.03538175046554937</v>
-      </c>
-      <c r="U41" s="23" t="n">
-        <v>0.01704545454545436</v>
       </c>
     </row>
     <row r="42">
@@ -3913,8 +3905,8 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="51" t="n">
-        <v>46204</v>
+      <c r="N42" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O42" s="45" t="inlineStr">
         <is>
@@ -3927,19 +3919,19 @@
         </is>
       </c>
       <c r="Q42" s="38" t="n">
-        <v>0.08246073298429316</v>
+        <v>0.0862745098039215</v>
       </c>
       <c r="R42" s="38" t="n">
+        <v>0.08115183246073283</v>
+      </c>
+      <c r="S42" s="38" t="n">
         <v>0.1004596191726854</v>
       </c>
-      <c r="S42" s="38" t="n">
+      <c r="T42" s="38" t="n">
         <v>0.1134564643799473</v>
       </c>
-      <c r="T42" s="38" t="n">
+      <c r="U42" s="23" t="n">
         <v>0.09305373525557023</v>
-      </c>
-      <c r="U42" s="23" t="n">
-        <v>0.05639344262295078</v>
       </c>
     </row>
     <row r="43">
@@ -3988,8 +3980,8 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="51" t="n">
-        <v>46204</v>
+      <c r="N43" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O43" s="45" t="inlineStr">
         <is>
@@ -4002,19 +3994,19 @@
         </is>
       </c>
       <c r="Q43" s="38" t="n">
-        <v>-0.003994673768308865</v>
+        <v>0.006675567423231055</v>
       </c>
       <c r="R43" s="38" t="n">
-        <v>-0.002656042496679945</v>
+        <v>-0.003326679973386537</v>
       </c>
       <c r="S43" s="38" t="n">
-        <v>0.01688048615800142</v>
+        <v>-0.002654280026542666</v>
       </c>
       <c r="T43" s="38" t="n">
+        <v>0.0175557056043214</v>
+      </c>
+      <c r="U43" s="23" t="n">
         <v>0.02279005524861866</v>
-      </c>
-      <c r="U43" s="23" t="n">
-        <v>0.009059233449477455</v>
       </c>
     </row>
     <row r="44">
@@ -4063,8 +4055,8 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="51" t="n">
-        <v>46204</v>
+      <c r="N44" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O44" s="45" t="inlineStr">
         <is>
@@ -4077,19 +4069,19 @@
         </is>
       </c>
       <c r="Q44" s="38" t="n">
-        <v>0.05949008498583574</v>
+        <v>0.06950354609929087</v>
       </c>
       <c r="R44" s="38" t="n">
-        <v>0.06676136363636347</v>
+        <v>0.06090651558073671</v>
       </c>
       <c r="S44" s="38" t="n">
-        <v>0.06808510638297868</v>
+        <v>0.0674715909090909</v>
       </c>
       <c r="T44" s="38" t="n">
+        <v>0.06879432624113467</v>
+      </c>
+      <c r="U44" s="23" t="n">
         <v>0.04516584333098099</v>
-      </c>
-      <c r="U44" s="23" t="n">
-        <v>0.0225988700564973</v>
       </c>
     </row>
     <row r="45">
@@ -4277,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4356,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4369,19 +4361,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.63</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.56</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.43</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.39</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.37</v>
       </c>
     </row>
     <row r="49">
@@ -4431,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4444,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.78</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.75</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.61</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.57</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.54</v>
       </c>
     </row>
     <row r="50">
@@ -4510,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4523,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.97</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.96</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.95</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.83</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.8</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.78</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4636,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4649,19 +4641,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.48</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.44</v>
-      </c>
-      <c r="R52" s="9" t="n">
-        <v>6.46</v>
       </c>
       <c r="S52" s="9" t="n">
         <v>6.46</v>
       </c>
       <c r="T52" s="9" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="U52" s="22" t="n">
         <v>6.38</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.37</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-09-17
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1228,7 +1228,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>5.1028</v>
+        <v>5.0796</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.54</v>
@@ -1720,7 +1720,7 @@
         </is>
       </c>
       <c r="N13" s="52" t="n">
-        <v>46265</v>
+        <v>46272</v>
       </c>
       <c r="O13" s="45" t="inlineStr">
         <is>
@@ -1733,19 +1733,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
+        <v>196000</v>
+      </c>
+      <c r="R13" s="24" t="n">
         <v>206000</v>
       </c>
-      <c r="R13" s="24" t="n">
+      <c r="S13" s="24" t="n">
         <v>207000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>204000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>207000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>212000</v>
       </c>
     </row>
     <row r="14">
@@ -1795,7 +1795,7 @@
         </is>
       </c>
       <c r="N14" s="52" t="n">
-        <v>46258</v>
+        <v>46265</v>
       </c>
       <c r="O14" s="45" t="inlineStr">
         <is>
@@ -1808,19 +1808,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1774000</v>
+        <v>1730000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1769000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1775000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1771000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1796000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1781000</v>
       </c>
     </row>
     <row r="15">
@@ -2126,8 +2126,10 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="51" t="n">
-        <v>46204</v>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DSPIC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D19" s="45" t="inlineStr">
         <is>
@@ -2140,19 +2142,19 @@
         </is>
       </c>
       <c r="F19" s="25" t="n">
-        <v>0.003744135940935589</v>
+        <v>1</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>0.003044427530958238</v>
+        <v>1</v>
       </c>
       <c r="H19" s="25" t="n">
-        <v>0.002394596009377858</v>
+        <v>1</v>
       </c>
       <c r="I19" s="25" t="n">
-        <v>-0.004070879897950741</v>
+        <v>1</v>
       </c>
       <c r="J19" s="25" t="n">
-        <v>-0.001185470781469022</v>
+        <v>1</v>
       </c>
       <c r="K19" s="46" t="n"/>
       <c r="L19" s="28" t="n"/>
@@ -2197,8 +2199,10 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="51" t="n">
-        <v>46204</v>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DSPIC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D20" s="45" t="inlineStr">
         <is>
@@ -2211,19 +2215,19 @@
         </is>
       </c>
       <c r="F20" s="25" t="n">
-        <v>0.004523055945102436</v>
+        <v>1</v>
       </c>
       <c r="G20" s="25" t="n">
-        <v>0.005166433768880193</v>
+        <v>1</v>
       </c>
       <c r="H20" s="25" t="n">
-        <v>0.001067799720814703</v>
+        <v>1</v>
       </c>
       <c r="I20" s="25" t="n">
-        <v>-0.009695084625184218</v>
+        <v>1</v>
       </c>
       <c r="J20" s="25" t="n">
-        <v>7.7652239989875e-05</v>
+        <v>1</v>
       </c>
       <c r="K20" s="46" t="n"/>
       <c r="L20" s="28" t="inlineStr">
@@ -2390,7 +2394,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="52" t="n">
+      <c r="N22" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O22" s="45" t="inlineStr">
@@ -2460,7 +2464,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="52" t="n">
+      <c r="N23" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O23" s="45" t="inlineStr">
@@ -2923,7 +2927,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,19 +2940,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.35</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.34</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.32</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.34</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.33</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3006,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,19 +3019,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.38</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.37</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.36</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.4</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.37</v>
       </c>
     </row>
     <row r="31">
@@ -3420,8 +3424,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="51" t="n">
-        <v>46204</v>
+      <c r="C36" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D36" s="45" t="inlineStr">
         <is>
@@ -3434,19 +3438,19 @@
         </is>
       </c>
       <c r="F36" s="24" t="n">
-        <v>1239</v>
+        <v>1275</v>
       </c>
       <c r="G36" s="24" t="n">
-        <v>1415</v>
+        <v>1309</v>
       </c>
       <c r="H36" s="24" t="n">
+        <v>1439</v>
+      </c>
+      <c r="I36" s="24" t="n">
         <v>1182</v>
       </c>
-      <c r="I36" s="24" t="n">
+      <c r="J36" s="24" t="n">
         <v>1414</v>
-      </c>
-      <c r="J36" s="24" t="n">
-        <v>1522</v>
       </c>
       <c r="K36" s="46" t="n"/>
       <c r="L36" s="28" t="n"/>
@@ -3491,8 +3495,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="51" t="n">
-        <v>46204</v>
+      <c r="C37" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D37" s="45" t="inlineStr">
         <is>
@@ -3505,19 +3509,19 @@
         </is>
       </c>
       <c r="F37" s="25" t="n">
-        <v>-0.1347765363128492</v>
+        <v>-0.01239349341595662</v>
       </c>
       <c r="G37" s="25" t="n">
-        <v>0.02610587382160986</v>
+        <v>-0.08589385474860335</v>
       </c>
       <c r="H37" s="25" t="n">
+        <v>0.04350978970268311</v>
+      </c>
+      <c r="I37" s="25" t="n">
         <v>-0.08301008533747091</v>
       </c>
-      <c r="I37" s="25" t="n">
+      <c r="J37" s="25" t="n">
         <v>0.01</v>
-      </c>
-      <c r="J37" s="25" t="n">
-        <v>0.1307578008915305</v>
       </c>
       <c r="K37" s="46" t="n"/>
       <c r="L37" s="28" t="inlineStr">
@@ -3570,8 +3574,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="51" t="n">
-        <v>46204</v>
+      <c r="C38" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D38" s="45" t="inlineStr">
         <is>
@@ -3584,19 +3588,19 @@
         </is>
       </c>
       <c r="F38" s="24" t="n">
+        <v>1394</v>
+      </c>
+      <c r="G38" s="24" t="n">
         <v>1433</v>
       </c>
-      <c r="G38" s="24" t="n">
+      <c r="H38" s="24" t="n">
         <v>1374</v>
       </c>
-      <c r="H38" s="24" t="n">
+      <c r="I38" s="24" t="n">
         <v>1410</v>
       </c>
-      <c r="I38" s="24" t="n">
+      <c r="J38" s="24" t="n">
         <v>1423</v>
-      </c>
-      <c r="J38" s="24" t="n">
-        <v>1363</v>
       </c>
       <c r="K38" s="46" t="n"/>
       <c r="L38" s="28" t="n"/>
@@ -3641,8 +3645,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="51" t="n">
-        <v>46204</v>
+      <c r="C39" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D39" s="45" t="inlineStr">
         <is>
@@ -3655,19 +3659,19 @@
         </is>
       </c>
       <c r="F39" s="38" t="n">
+        <v>0.03489235337787677</v>
+      </c>
+      <c r="G39" s="38" t="n">
         <v>0.02357142857142857</v>
       </c>
-      <c r="G39" s="38" t="n">
+      <c r="H39" s="38" t="n">
         <v>-0.0178699070764832</v>
       </c>
-      <c r="H39" s="38" t="n">
+      <c r="I39" s="38" t="n">
         <v>-0.00423728813559322</v>
       </c>
-      <c r="I39" s="38" t="n">
+      <c r="J39" s="38" t="n">
         <v>-0.01522491349480969</v>
-      </c>
-      <c r="J39" s="38" t="n">
-        <v>-0.08646112600536193</v>
       </c>
       <c r="K39" s="46" t="n"/>
       <c r="L39" s="28" t="inlineStr">
@@ -4269,7 +4273,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4352,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,19 +4365,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.65</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.63</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.56</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.43</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.39</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4427,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4440,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.83</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.8</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.78</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.75</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.61</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.57</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4506,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4519,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.97</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.96</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.95</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.83</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.8</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4577,7 +4581,7 @@
         </is>
       </c>
       <c r="N51" s="52" t="n">
-        <v>46272</v>
+        <v>46279</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
         <is>
@@ -4590,19 +4594,19 @@
         </is>
       </c>
       <c r="Q51" s="45" t="n">
+        <v>6.95</v>
+      </c>
+      <c r="R51" s="45" t="n">
         <v>6.76</v>
       </c>
-      <c r="R51" s="45" t="n">
+      <c r="S51" s="45" t="n">
         <v>6.71</v>
       </c>
-      <c r="S51" s="45" t="n">
+      <c r="T51" s="45" t="n">
         <v>6.66</v>
       </c>
-      <c r="T51" s="45" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.65</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.67</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4628,7 +4632,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,19 +4645,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.44</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.48</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.44</v>
-      </c>
-      <c r="S52" s="9" t="n">
-        <v>6.46</v>
       </c>
       <c r="T52" s="9" t="n">
         <v>6.46</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>6.38</v>
+        <v>6.46</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-09-18
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2086,7 +2086,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="52" t="n">
+      <c r="N18" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O18" s="45" t="inlineStr">
@@ -2126,10 +2126,8 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DSPIC96' not found in values file."</t>
-        </is>
+      <c r="C19" s="51" t="n">
+        <v>46204</v>
       </c>
       <c r="D19" s="45" t="inlineStr">
         <is>
@@ -2142,19 +2140,19 @@
         </is>
       </c>
       <c r="F19" s="25" t="n">
-        <v>1</v>
+        <v>0.003744135940935589</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>1</v>
+        <v>0.003044427530958238</v>
       </c>
       <c r="H19" s="25" t="n">
-        <v>1</v>
+        <v>0.002394596009377858</v>
       </c>
       <c r="I19" s="25" t="n">
-        <v>1</v>
+        <v>-0.004070879897950741</v>
       </c>
       <c r="J19" s="25" t="n">
-        <v>1</v>
+        <v>-0.001185470781469022</v>
       </c>
       <c r="K19" s="46" t="n"/>
       <c r="L19" s="28" t="n"/>
@@ -2163,7 +2161,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="52" t="n">
+      <c r="N19" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O19" s="45" t="inlineStr">
@@ -2199,10 +2197,8 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DSPIC96' not found in values file."</t>
-        </is>
+      <c r="C20" s="51" t="n">
+        <v>46204</v>
       </c>
       <c r="D20" s="45" t="inlineStr">
         <is>
@@ -2215,19 +2211,19 @@
         </is>
       </c>
       <c r="F20" s="25" t="n">
-        <v>1</v>
+        <v>0.004523055945102436</v>
       </c>
       <c r="G20" s="25" t="n">
-        <v>1</v>
+        <v>0.005166433768880193</v>
       </c>
       <c r="H20" s="25" t="n">
-        <v>1</v>
+        <v>0.001067799720814703</v>
       </c>
       <c r="I20" s="25" t="n">
-        <v>1</v>
+        <v>-0.009695084625184218</v>
       </c>
       <c r="J20" s="25" t="n">
-        <v>1</v>
+        <v>7.7652239989875e-05</v>
       </c>
       <c r="K20" s="46" t="n"/>
       <c r="L20" s="28" t="inlineStr">
@@ -2240,7 +2236,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="52" t="n">
+      <c r="N20" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O20" s="45" t="inlineStr">
@@ -2315,7 +2311,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="52" t="n">
+      <c r="N21" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O21" s="45" t="inlineStr">
@@ -2927,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2940,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.31</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.35</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.34</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.32</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.34</v>
       </c>
     </row>
     <row r="30">
@@ -3006,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3022,16 +3018,16 @@
         <v>2.33</v>
       </c>
       <c r="R30" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="S30" s="45" t="n">
         <v>2.38</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.37</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.36</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.4</v>
       </c>
     </row>
     <row r="31">
@@ -3120,8 +3116,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="51" t="n">
-        <v>46204</v>
+      <c r="C32" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D32" s="45" t="inlineStr">
         <is>
@@ -3134,19 +3130,19 @@
         </is>
       </c>
       <c r="F32" s="25" t="n">
-        <v>0.002014850155856562</v>
+        <v>0.0002212616963008784</v>
       </c>
       <c r="G32" s="25" t="n">
-        <v>0.002701202518000656</v>
+        <v>0.001977791174811783</v>
       </c>
       <c r="H32" s="25" t="n">
-        <v>-9.656671199120836e-05</v>
+        <v>0.001971948448746819</v>
       </c>
       <c r="I32" s="25" t="n">
-        <v>0.00752302359703716</v>
+        <v>0.0005975922782888166</v>
       </c>
       <c r="J32" s="25" t="n">
-        <v>-0.001481767876646223</v>
+        <v>0.008303058183333656</v>
       </c>
       <c r="K32" s="46" t="n"/>
       <c r="L32" s="28" t="n"/>
@@ -3191,8 +3187,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="51" t="n">
-        <v>46204</v>
+      <c r="C33" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D33" s="45" t="inlineStr">
         <is>
@@ -3205,19 +3201,19 @@
         </is>
       </c>
       <c r="F33" s="25" t="n">
-        <v>0.01079455120026685</v>
+        <v>0.0142042239731089</v>
       </c>
       <c r="G33" s="25" t="n">
-        <v>0.01289238607192659</v>
+        <v>0.01129997840893473</v>
       </c>
       <c r="H33" s="25" t="n">
-        <v>0.01529631408748529</v>
+        <v>0.01343634365900168</v>
       </c>
       <c r="I33" s="25" t="n">
-        <v>0.01376375856712151</v>
+        <v>0.01658091130138508</v>
       </c>
       <c r="J33" s="25" t="n">
-        <v>0.00706549063542895</v>
+        <v>0.01434223394335294</v>
       </c>
       <c r="K33" s="46" t="n"/>
       <c r="L33" s="28" t="inlineStr">
@@ -3270,8 +3266,8 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="51" t="n">
-        <v>46204</v>
+      <c r="C34" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D34" s="45" t="inlineStr">
         <is>
@@ -3284,19 +3280,19 @@
         </is>
       </c>
       <c r="F34" s="24" t="n">
-        <v>76.2878</v>
+        <v>76.2717</v>
       </c>
       <c r="G34" s="24" t="n">
-        <v>76.2029</v>
+        <v>76.3259</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>76.0642</v>
+        <v>76.24379999999999</v>
       </c>
       <c r="I34" s="24" t="n">
-        <v>76.1369</v>
+        <v>76.1605</v>
       </c>
       <c r="J34" s="24" t="n">
-        <v>75.6332</v>
+        <v>76.1803</v>
       </c>
       <c r="K34" s="46" t="n"/>
       <c r="L34" s="28" t="n"/>
@@ -4273,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4352,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4365,19 +4361,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.67</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.65</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.63</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.56</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.43</v>
       </c>
     </row>
     <row r="49">
@@ -4427,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4440,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.86</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.83</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.8</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.78</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.75</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.61</v>
       </c>
     </row>
     <row r="50">
@@ -4506,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4519,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5.01</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.97</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.96</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.95</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.83</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4632,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4645,16 +4641,16 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.44</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.48</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.44</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>6.46</v>
       </c>
       <c r="U52" s="22" t="n">
         <v>6.46</v>

</xml_diff>

<commit_message>
Update dashboards - 2026-09-19
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.34</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.31</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.35</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.34</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.32</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3021,13 +3021,13 @@
         <v>2.33</v>
       </c>
       <c r="S30" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="T30" s="45" t="n">
         <v>2.38</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.37</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.36</v>
       </c>
     </row>
     <row r="31">
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4282,7 +4282,7 @@
         </is>
       </c>
       <c r="Q47" s="45" t="n">
-        <v>3.63</v>
+        <v>3.88</v>
       </c>
       <c r="R47" s="45" t="n">
         <v>3.63</v>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,19 +4361,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.74</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.67</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.65</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.63</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.56</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.86</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.83</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.8</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.78</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.75</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.94</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>5.01</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.97</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.96</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.95</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-09-21
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,19 +4641,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.41</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.38</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.44</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.48</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.44</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.46</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-09-22
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2500,8 +2500,10 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="51" t="n">
-        <v>46204</v>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'REVOLSL' not found in values file."</t>
+        </is>
       </c>
       <c r="D24" s="45" t="inlineStr">
         <is>
@@ -2514,19 +2516,19 @@
         </is>
       </c>
       <c r="F24" s="38" t="n">
-        <v>0.002069337953391592</v>
+        <v>1</v>
       </c>
       <c r="G24" s="38" t="n">
-        <v>0.004986963805690525</v>
+        <v>1</v>
       </c>
       <c r="H24" s="38" t="n">
-        <v>-0.001636032119741393</v>
+        <v>1</v>
       </c>
       <c r="I24" s="38" t="n">
-        <v>0.008761168564920929</v>
+        <v>1</v>
       </c>
       <c r="J24" s="38" t="n">
-        <v>0.008334847450631955</v>
+        <v>1</v>
       </c>
       <c r="K24" s="46" t="n"/>
       <c r="L24" s="28" t="inlineStr">
@@ -2923,7 +2925,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,16 +2941,16 @@
         <v>2.35</v>
       </c>
       <c r="R29" s="45" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="S29" s="45" t="n">
         <v>2.34</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.31</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.35</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.34</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3004,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,7 +3017,7 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
-        <v>2.33</v>
+        <v>2.34</v>
       </c>
       <c r="R30" s="45" t="n">
         <v>2.33</v>
@@ -3024,10 +3026,10 @@
         <v>2.33</v>
       </c>
       <c r="T30" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="U30" s="21" t="n">
         <v>2.38</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.37</v>
       </c>
     </row>
     <row r="31">
@@ -4269,7 +4271,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4285,7 +4287,7 @@
         <v>3.88</v>
       </c>
       <c r="R47" s="45" t="n">
-        <v>3.63</v>
+        <v>3.88</v>
       </c>
       <c r="S47" s="45" t="n">
         <v>3.63</v>
@@ -4348,7 +4350,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,19 +4363,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.67</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.74</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.67</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.65</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.63</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4425,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4438,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.86</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.78</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.86</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.83</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.8</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.78</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4504,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4517,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5.01</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.94</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>5.01</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.97</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.96</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4628,7 +4630,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,19 +4643,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.41</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.38</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.44</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.48</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.44</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-09-23
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1960,7 +1960,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="52" t="n">
+      <c r="C17" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="45" t="inlineStr">
@@ -2047,7 +2047,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="52" t="n">
+      <c r="C18" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="45" t="inlineStr">
@@ -2500,10 +2500,8 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'REVOLSL' not found in values file."</t>
-        </is>
+      <c r="C24" s="51" t="n">
+        <v>46204</v>
       </c>
       <c r="D24" s="45" t="inlineStr">
         <is>
@@ -2516,19 +2514,19 @@
         </is>
       </c>
       <c r="F24" s="38" t="n">
-        <v>1</v>
+        <v>0.002069337953391592</v>
       </c>
       <c r="G24" s="38" t="n">
-        <v>1</v>
+        <v>0.004986963805690525</v>
       </c>
       <c r="H24" s="38" t="n">
-        <v>1</v>
+        <v>-0.001636032119741393</v>
       </c>
       <c r="I24" s="38" t="n">
-        <v>1</v>
+        <v>0.008761168564920929</v>
       </c>
       <c r="J24" s="38" t="n">
-        <v>1</v>
+        <v>0.008334847450631955</v>
       </c>
       <c r="K24" s="46" t="n"/>
       <c r="L24" s="28" t="inlineStr">
@@ -2925,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2938,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
-        <v>2.35</v>
+        <v>2.34</v>
       </c>
       <c r="R29" s="45" t="n">
         <v>2.35</v>
       </c>
       <c r="S29" s="45" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="T29" s="45" t="n">
         <v>2.34</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.31</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.35</v>
       </c>
     </row>
     <row r="30">
@@ -3004,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3017,10 +3015,10 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.34</v>
-      </c>
-      <c r="R30" s="45" t="n">
-        <v>2.33</v>
       </c>
       <c r="S30" s="45" t="n">
         <v>2.33</v>
@@ -3029,7 +3027,7 @@
         <v>2.33</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.38</v>
+        <v>2.33</v>
       </c>
     </row>
     <row r="31">
@@ -3832,7 +3830,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="52" t="n">
+      <c r="N41" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O41" s="45" t="inlineStr">
@@ -3907,7 +3905,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="52" t="n">
+      <c r="N42" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O42" s="45" t="inlineStr">
@@ -3982,7 +3980,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="52" t="n">
+      <c r="N43" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O43" s="45" t="inlineStr">
@@ -4057,7 +4055,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="52" t="n">
+      <c r="N44" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O44" s="45" t="inlineStr">
@@ -4271,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4290,13 +4288,13 @@
         <v>3.88</v>
       </c>
       <c r="S47" s="45" t="n">
-        <v>3.63</v>
+        <v>3.88</v>
       </c>
       <c r="T47" s="45" t="n">
-        <v>3.63</v>
+        <v>3.88</v>
       </c>
       <c r="U47" s="21" t="n">
-        <v>3.63</v>
+        <v>3.88</v>
       </c>
     </row>
     <row r="48">
@@ -4350,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4366,16 +4364,16 @@
         <v>4.76</v>
       </c>
       <c r="R48" s="45" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="S48" s="45" t="n">
         <v>4.67</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.74</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.67</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.65</v>
       </c>
     </row>
     <row r="49">
@@ -4425,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4438,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.83</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.86</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.78</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.86</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.83</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.8</v>
       </c>
     </row>
     <row r="50">
@@ -4504,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4517,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.96</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>5.01</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.94</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>5.01</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>5</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.97</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4630,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4646,16 +4644,16 @@
         <v>6.38</v>
       </c>
       <c r="R52" s="9" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="S52" s="9" t="n">
         <v>6.41</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.38</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.44</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.48</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-09-24
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1720,7 +1720,7 @@
         </is>
       </c>
       <c r="N13" s="52" t="n">
-        <v>46272</v>
+        <v>46279</v>
       </c>
       <c r="O13" s="45" t="inlineStr">
         <is>
@@ -1733,19 +1733,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>196000</v>
+        <v>197000</v>
       </c>
       <c r="R13" s="24" t="n">
-        <v>206000</v>
+        <v>198000</v>
       </c>
       <c r="S13" s="24" t="n">
         <v>207000</v>
       </c>
       <c r="T13" s="24" t="n">
+        <v>207000</v>
+      </c>
+      <c r="U13" s="26" t="n">
         <v>204000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>207000</v>
       </c>
     </row>
     <row r="14">
@@ -1795,7 +1795,7 @@
         </is>
       </c>
       <c r="N14" s="52" t="n">
-        <v>46265</v>
+        <v>46272</v>
       </c>
       <c r="O14" s="45" t="inlineStr">
         <is>
@@ -1808,19 +1808,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1730000</v>
+        <v>1719000</v>
       </c>
       <c r="R14" s="24" t="n">
-        <v>1769000</v>
+        <v>1717000</v>
       </c>
       <c r="S14" s="24" t="n">
+        <v>1765000</v>
+      </c>
+      <c r="T14" s="24" t="n">
         <v>1775000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1771000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1796000</v>
       </c>
     </row>
     <row r="15">
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.34</v>
-      </c>
-      <c r="R29" s="45" t="n">
-        <v>2.35</v>
       </c>
       <c r="S29" s="45" t="n">
         <v>2.35</v>
       </c>
       <c r="T29" s="45" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="U29" s="21" t="n">
         <v>2.34</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.31</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,13 +3015,13 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.34</v>
-      </c>
-      <c r="S30" s="45" t="n">
-        <v>2.33</v>
       </c>
       <c r="T30" s="45" t="n">
         <v>2.33</v>
@@ -3420,7 +3420,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="52" t="n">
+      <c r="C36" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D36" s="45" t="inlineStr">
@@ -3491,7 +3491,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="52" t="n">
+      <c r="C37" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D37" s="45" t="inlineStr">
@@ -3570,7 +3570,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="52" t="n">
+      <c r="C38" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D38" s="45" t="inlineStr">
@@ -3584,7 +3584,7 @@
         </is>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1394</v>
+        <v>1403</v>
       </c>
       <c r="G38" s="24" t="n">
         <v>1433</v>
@@ -3641,7 +3641,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="52" t="n">
+      <c r="C39" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D39" s="45" t="inlineStr">
@@ -3655,7 +3655,7 @@
         </is>
       </c>
       <c r="F39" s="38" t="n">
-        <v>0.03489235337787677</v>
+        <v>0.04157386785449146</v>
       </c>
       <c r="G39" s="38" t="n">
         <v>0.02357142857142857</v>
@@ -3720,8 +3720,8 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="51" t="n">
-        <v>46204</v>
+      <c r="C40" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D40" s="45" t="inlineStr">
         <is>
@@ -3734,19 +3734,19 @@
         </is>
       </c>
       <c r="F40" s="24" t="n">
-        <v>607</v>
+        <v>684</v>
       </c>
       <c r="G40" s="24" t="n">
-        <v>678</v>
+        <v>643</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>630</v>
+        <v>672</v>
       </c>
       <c r="I40" s="24" t="n">
+        <v>636</v>
+      </c>
+      <c r="J40" s="24" t="n">
         <v>641</v>
-      </c>
-      <c r="J40" s="24" t="n">
-        <v>659</v>
       </c>
       <c r="K40" s="46" t="n"/>
       <c r="L40" s="28" t="n"/>
@@ -3791,8 +3791,8 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="51" t="n">
-        <v>46204</v>
+      <c r="C41" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D41" s="45" t="inlineStr">
         <is>
@@ -3805,19 +3805,19 @@
         </is>
       </c>
       <c r="F41" s="38" t="n">
-        <v>-0.06327160493827161</v>
+        <v>-0.02005730659025788</v>
       </c>
       <c r="G41" s="38" t="n">
-        <v>0.01954887218045113</v>
+        <v>-0.007716049382716049</v>
       </c>
       <c r="H41" s="38" t="n">
-        <v>0.01286173633440514</v>
+        <v>0.01052631578947368</v>
       </c>
       <c r="I41" s="38" t="n">
+        <v>0.022508038585209</v>
+      </c>
+      <c r="J41" s="38" t="n">
         <v>-0.08559201141226819</v>
-      </c>
-      <c r="J41" s="38" t="n">
-        <v>0.004573170731707317</v>
       </c>
       <c r="K41" s="46" t="n"/>
       <c r="L41" s="28" t="inlineStr">
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,19 +4361,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
-        <v>4.76</v>
+        <v>4.71</v>
       </c>
       <c r="R48" s="45" t="n">
         <v>4.76</v>
       </c>
       <c r="S48" s="45" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="T48" s="45" t="n">
         <v>4.67</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.74</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.67</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4439,16 +4439,16 @@
         <v>4.83</v>
       </c>
       <c r="R49" s="45" t="n">
+        <v>4.83</v>
+      </c>
+      <c r="S49" s="45" t="n">
         <v>4.86</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.78</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.86</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.83</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,16 +4518,16 @@
         <v>4.96</v>
       </c>
       <c r="R50" s="45" t="n">
+        <v>4.96</v>
+      </c>
+      <c r="S50" s="45" t="n">
         <v>5.01</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.94</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>5.01</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4577,7 +4577,7 @@
         </is>
       </c>
       <c r="N51" s="52" t="n">
-        <v>46279</v>
+        <v>46286</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
         <is>
@@ -4590,19 +4590,19 @@
         </is>
       </c>
       <c r="Q51" s="45" t="n">
+        <v>7.03</v>
+      </c>
+      <c r="R51" s="45" t="n">
         <v>6.95</v>
       </c>
-      <c r="R51" s="45" t="n">
+      <c r="S51" s="45" t="n">
         <v>6.76</v>
       </c>
-      <c r="S51" s="45" t="n">
+      <c r="T51" s="45" t="n">
         <v>6.71</v>
       </c>
-      <c r="T51" s="45" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.66</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.65</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,19 +4641,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>6.38</v>
+        <v>6.5</v>
       </c>
       <c r="R52" s="9" t="n">
         <v>6.38</v>
       </c>
       <c r="S52" s="9" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="T52" s="9" t="n">
         <v>6.41</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.38</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.44</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-09-25
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1228,7 +1228,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>5.0796</v>
+        <v>5.0163</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.54</v>
@@ -2808,8 +2808,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="51" t="n">
-        <v>46204</v>
+      <c r="C28" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D28" s="45" t="inlineStr">
         <is>
@@ -2822,19 +2822,19 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>0.01076005348756182</v>
+        <v>-0.0001712622024319099</v>
       </c>
       <c r="G28" s="25" t="n">
+        <v>0.008586004485092946</v>
+      </c>
+      <c r="H28" s="25" t="n">
         <v>0.005802145925317914</v>
       </c>
-      <c r="H28" s="25" t="n">
+      <c r="I28" s="25" t="n">
         <v>-0.04004117699494203</v>
       </c>
-      <c r="I28" s="25" t="n">
+      <c r="J28" s="25" t="n">
         <v>0.08512722904348102</v>
-      </c>
-      <c r="J28" s="25" t="n">
-        <v>0.01344578206575542</v>
       </c>
       <c r="K28" s="46" t="n"/>
       <c r="L28" s="28" t="inlineStr">
@@ -2848,7 +2848,7 @@
         </is>
       </c>
       <c r="N28" s="51" t="n">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="O28" s="45" t="inlineStr">
         <is>
@@ -2861,19 +2861,19 @@
         </is>
       </c>
       <c r="Q28" s="45" t="n">
+        <v>4</v>
+      </c>
+      <c r="R28" s="45" t="n">
         <v>4.2</v>
       </c>
-      <c r="R28" s="45" t="n">
+      <c r="S28" s="45" t="n">
         <v>4.6</v>
       </c>
-      <c r="S28" s="45" t="n">
+      <c r="T28" s="45" t="n">
         <v>4.8</v>
       </c>
-      <c r="T28" s="45" t="n">
+      <c r="U28" s="21" t="n">
         <v>4.7</v>
-      </c>
-      <c r="U28" s="21" t="n">
-        <v>3.8</v>
       </c>
     </row>
     <row r="29">
@@ -2883,8 +2883,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="51" t="n">
-        <v>46204</v>
+      <c r="C29" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D29" s="45" t="inlineStr">
         <is>
@@ -2897,19 +2897,19 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>0.1199873280709628</v>
+        <v>0.08478942006420237</v>
       </c>
       <c r="G29" s="25" t="n">
+        <v>0.1175783415612873</v>
+      </c>
+      <c r="H29" s="25" t="n">
         <v>0.07703978368044752</v>
       </c>
-      <c r="H29" s="25" t="n">
+      <c r="I29" s="25" t="n">
         <v>-0.02972368914374733</v>
       </c>
-      <c r="I29" s="25" t="n">
+      <c r="J29" s="25" t="n">
         <v>0.1779567725392831</v>
-      </c>
-      <c r="J29" s="25" t="n">
-        <v>0.01350347073984473</v>
       </c>
       <c r="K29" s="46" t="n"/>
       <c r="L29" s="28" t="inlineStr">
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.36</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.34</v>
-      </c>
-      <c r="S29" s="45" t="n">
-        <v>2.35</v>
       </c>
       <c r="T29" s="45" t="n">
         <v>2.35</v>
       </c>
       <c r="U29" s="21" t="n">
-        <v>2.34</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="30">
@@ -2962,8 +2962,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="51" t="n">
-        <v>46204</v>
+      <c r="C30" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D30" s="45" t="inlineStr">
         <is>
@@ -2976,19 +2976,19 @@
         </is>
       </c>
       <c r="F30" s="25" t="n">
-        <v>0.01294210214449687</v>
+        <v>0.0005108458969496077</v>
       </c>
       <c r="G30" s="25" t="n">
+        <v>0.0141466210331016</v>
+      </c>
+      <c r="H30" s="25" t="n">
         <v>0.003538609511678281</v>
       </c>
-      <c r="H30" s="25" t="n">
+      <c r="I30" s="25" t="n">
         <v>-0.04261964610139124</v>
       </c>
-      <c r="I30" s="25" t="n">
+      <c r="J30" s="25" t="n">
         <v>0.08475262626842106</v>
-      </c>
-      <c r="J30" s="25" t="n">
-        <v>-0.002709178900039744</v>
       </c>
       <c r="K30" s="46" t="n"/>
       <c r="L30" s="28" t="inlineStr">
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,16 +3015,16 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.35</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.34</v>
-      </c>
-      <c r="T30" s="45" t="n">
-        <v>2.33</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.33</v>
@@ -3037,8 +3037,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="51" t="n">
-        <v>46204</v>
+      <c r="C31" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D31" s="45" t="inlineStr">
         <is>
@@ -3051,19 +3051,19 @@
         </is>
       </c>
       <c r="F31" s="25" t="n">
-        <v>0.09763619840916188</v>
+        <v>0.0789205492280784</v>
       </c>
       <c r="G31" s="25" t="n">
+        <v>0.0989414295087489</v>
+      </c>
+      <c r="H31" s="25" t="n">
         <v>0.05755592766471823</v>
       </c>
-      <c r="H31" s="25" t="n">
+      <c r="I31" s="25" t="n">
         <v>-0.04567753459150702</v>
       </c>
-      <c r="I31" s="25" t="n">
+      <c r="J31" s="25" t="n">
         <v>0.1533794281326583</v>
-      </c>
-      <c r="J31" s="25" t="n">
-        <v>-0.0182024802287403</v>
       </c>
       <c r="K31" s="46" t="n"/>
       <c r="L31" s="28" t="inlineStr">
@@ -3116,7 +3116,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="52" t="n">
+      <c r="C32" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D32" s="45" t="inlineStr">
@@ -3187,7 +3187,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="52" t="n">
+      <c r="C33" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D33" s="45" t="inlineStr">
@@ -3266,7 +3266,7 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="52" t="n">
+      <c r="C34" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D34" s="45" t="inlineStr">
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,19 +4361,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.71</v>
-      </c>
-      <c r="R48" s="45" t="n">
-        <v>4.76</v>
       </c>
       <c r="S48" s="45" t="n">
         <v>4.76</v>
       </c>
       <c r="T48" s="45" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="U48" s="21" t="n">
         <v>4.67</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.74</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
-        <v>4.83</v>
+        <v>4.99</v>
       </c>
       <c r="R49" s="45" t="n">
         <v>4.83</v>
       </c>
       <c r="S49" s="45" t="n">
+        <v>4.83</v>
+      </c>
+      <c r="T49" s="45" t="n">
         <v>4.86</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.78</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.86</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
-        <v>4.96</v>
+        <v>5.11</v>
       </c>
       <c r="R50" s="45" t="n">
         <v>4.96</v>
       </c>
       <c r="S50" s="45" t="n">
+        <v>4.96</v>
+      </c>
+      <c r="T50" s="45" t="n">
         <v>5.01</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.94</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>5.01</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,19 +4641,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.5</v>
-      </c>
-      <c r="R52" s="9" t="n">
-        <v>6.38</v>
       </c>
       <c r="S52" s="9" t="n">
         <v>6.38</v>
       </c>
       <c r="T52" s="9" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="U52" s="22" t="n">
         <v>6.41</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.38</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-09-26
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,16 +2936,16 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.36</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.34</v>
-      </c>
-      <c r="T29" s="45" t="n">
-        <v>2.35</v>
       </c>
       <c r="U29" s="21" t="n">
         <v>2.35</v>
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,19 +3015,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.35</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.34</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.33</v>
       </c>
     </row>
     <row r="31">
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,19 +4361,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.87</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.85</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.71</v>
-      </c>
-      <c r="S48" s="45" t="n">
-        <v>4.76</v>
       </c>
       <c r="T48" s="45" t="n">
         <v>4.76</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>4.67</v>
+        <v>4.76</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>5.03</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.99</v>
-      </c>
-      <c r="R49" s="45" t="n">
-        <v>4.83</v>
       </c>
       <c r="S49" s="45" t="n">
         <v>4.83</v>
       </c>
       <c r="T49" s="45" t="n">
+        <v>4.83</v>
+      </c>
+      <c r="U49" s="21" t="n">
         <v>4.86</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.78</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>5.11</v>
-      </c>
-      <c r="R50" s="45" t="n">
-        <v>4.96</v>
       </c>
       <c r="S50" s="45" t="n">
         <v>4.96</v>
       </c>
       <c r="T50" s="45" t="n">
+        <v>4.96</v>
+      </c>
+      <c r="U50" s="21" t="n">
         <v>5.01</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.94</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-09-28
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,16 +4361,16 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.81</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.87</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.85</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.71</v>
-      </c>
-      <c r="T48" s="45" t="n">
-        <v>4.76</v>
       </c>
       <c r="U48" s="21" t="n">
         <v>4.76</v>
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>5.03</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.99</v>
-      </c>
-      <c r="S49" s="45" t="n">
-        <v>4.83</v>
       </c>
       <c r="T49" s="45" t="n">
         <v>4.83</v>
       </c>
       <c r="U49" s="21" t="n">
-        <v>4.86</v>
+        <v>4.83</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5.17</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>5.18</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>5.11</v>
-      </c>
-      <c r="S50" s="45" t="n">
-        <v>4.96</v>
       </c>
       <c r="T50" s="45" t="n">
         <v>4.96</v>
       </c>
       <c r="U50" s="21" t="n">
-        <v>5.01</v>
+        <v>4.96</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,19 +4641,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.63</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.57</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.5</v>
-      </c>
-      <c r="S52" s="9" t="n">
-        <v>6.38</v>
       </c>
       <c r="T52" s="9" t="n">
         <v>6.38</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>6.41</v>
+        <v>6.38</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-09-29
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1486,8 +1486,8 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="51" t="n">
-        <v>46204</v>
+      <c r="N10" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O10" s="45" t="inlineStr">
         <is>
@@ -1500,19 +1500,19 @@
         </is>
       </c>
       <c r="Q10" s="45" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="R10" s="45" t="n">
         <v>4.4</v>
       </c>
-      <c r="R10" s="45" t="n">
+      <c r="S10" s="45" t="n">
         <v>4.3</v>
       </c>
-      <c r="S10" s="45" t="n">
+      <c r="T10" s="45" t="n">
         <v>4.5</v>
       </c>
-      <c r="T10" s="45" t="n">
+      <c r="U10" s="21" t="n">
         <v>4.6</v>
-      </c>
-      <c r="U10" s="21" t="n">
-        <v>4.2</v>
       </c>
     </row>
     <row r="11">
@@ -1565,8 +1565,8 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="51" t="n">
-        <v>46204</v>
+      <c r="N11" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O11" s="45" t="inlineStr">
         <is>
@@ -1579,19 +1579,19 @@
         </is>
       </c>
       <c r="Q11" s="45" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="R11" s="45" t="n">
         <v>3.2</v>
       </c>
-      <c r="R11" s="45" t="n">
+      <c r="S11" s="45" t="n">
         <v>3.4</v>
-      </c>
-      <c r="S11" s="45" t="n">
-        <v>3.3</v>
       </c>
       <c r="T11" s="45" t="n">
         <v>3.3</v>
       </c>
       <c r="U11" s="21" t="n">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="12">
@@ -1640,8 +1640,8 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="51" t="n">
-        <v>46204</v>
+      <c r="N12" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O12" s="45" t="inlineStr">
         <is>
@@ -1657,16 +1657,16 @@
         <v>3.2</v>
       </c>
       <c r="R12" s="45" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="S12" s="45" t="n">
         <v>3.4</v>
       </c>
-      <c r="S12" s="45" t="n">
+      <c r="T12" s="45" t="n">
         <v>3.3</v>
       </c>
-      <c r="T12" s="45" t="n">
+      <c r="U12" s="21" t="n">
         <v>3.2</v>
-      </c>
-      <c r="U12" s="21" t="n">
-        <v>3.4</v>
       </c>
     </row>
     <row r="13">
@@ -1974,19 +1974,19 @@
         </is>
       </c>
       <c r="F17" s="25" t="n">
-        <v>0.01240741855056227</v>
+        <v>0.01127425850332675</v>
       </c>
       <c r="G17" s="25" t="n">
-        <v>-0.005366991635299634</v>
+        <v>-0.004584539731313231</v>
       </c>
       <c r="H17" s="25" t="n">
-        <v>0.00312584835132701</v>
+        <v>0.002027576683551802</v>
       </c>
       <c r="I17" s="25" t="n">
-        <v>0.009346631589902232</v>
+        <v>0.01035195829379165</v>
       </c>
       <c r="J17" s="25" t="n">
-        <v>0.006742589318751824</v>
+        <v>0.005864943726552774</v>
       </c>
       <c r="K17" s="46" t="n"/>
       <c r="L17" s="29" t="inlineStr">
@@ -2061,19 +2061,19 @@
         </is>
       </c>
       <c r="F18" s="25" t="n">
-        <v>0.06014763635267802</v>
+        <v>0.05361901579222471</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>0.05032033271185719</v>
+        <v>0.04476427794008134</v>
       </c>
       <c r="H18" s="25" t="n">
-        <v>0.06824752183509293</v>
+        <v>0.0592802540313897</v>
       </c>
       <c r="I18" s="25" t="n">
-        <v>0.0723275853623377</v>
+        <v>0.06699898466493943</v>
       </c>
       <c r="J18" s="25" t="n">
-        <v>0.05073763706982706</v>
+        <v>0.04091800582057446</v>
       </c>
       <c r="K18" s="46" t="n"/>
       <c r="L18" s="28" t="inlineStr">
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.34</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.36</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.34</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.35</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,16 +3018,16 @@
         <v>2.34</v>
       </c>
       <c r="R30" s="45" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="S30" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.35</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.33</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.34</v>
       </c>
     </row>
     <row r="31">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,16 +4641,16 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.63</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.57</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.5</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>6.38</v>
       </c>
       <c r="U52" s="22" t="n">
         <v>6.38</v>

</xml_diff>

<commit_message>
Update dashboards - 2026-09-30
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -223,7 +223,7 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -378,7 +378,13 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -924,19 +930,19 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
-        <v>24269.613</v>
+        <v>24408.011</v>
       </c>
       <c r="G3" s="24" t="n">
-        <v>24180.419</v>
+        <v>24274.383</v>
       </c>
       <c r="H3" s="24" t="n">
-        <v>24055.749</v>
+        <v>24125.479</v>
       </c>
       <c r="I3" s="24" t="n">
-        <v>24026.834</v>
+        <v>24112.966</v>
       </c>
       <c r="J3" s="24" t="n">
-        <v>23770.976</v>
+        <v>23884.563</v>
       </c>
       <c r="K3" s="46" t="n"/>
       <c r="L3" s="28" t="inlineStr">
@@ -999,19 +1005,19 @@
         </is>
       </c>
       <c r="F4" s="25" t="n">
-        <v>0.003688687114975053</v>
+        <v>0.005504897899979433</v>
       </c>
       <c r="G4" s="25" t="n">
-        <v>0.00518254492928083</v>
+        <v>0.006172063982646803</v>
       </c>
       <c r="H4" s="25" t="n">
-        <v>0.001203446113624551</v>
+        <v>0.0005189324283043639</v>
       </c>
       <c r="I4" s="25" t="n">
-        <v>0.0107634621312982</v>
+        <v>0.009562787479092671</v>
       </c>
       <c r="J4" s="25" t="n">
-        <v>0.009459997171759493</v>
+        <v>0.009909001665228123</v>
       </c>
       <c r="K4" s="46" t="n"/>
       <c r="L4" s="28" t="n"/>
@@ -1099,8 +1105,8 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="51" t="n">
-        <v>46235</v>
+      <c r="N5" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O5" s="45" t="inlineStr">
         <is>
@@ -1113,19 +1119,19 @@
         </is>
       </c>
       <c r="Q5" s="24" t="n">
-        <v>38000</v>
+        <v>90000</v>
       </c>
       <c r="R5" s="24" t="n">
-        <v>46000</v>
+        <v>36000</v>
       </c>
       <c r="S5" s="24" t="n">
+        <v>44000</v>
+      </c>
+      <c r="T5" s="24" t="n">
         <v>95000</v>
       </c>
-      <c r="T5" s="24" t="n">
+      <c r="U5" s="26" t="n">
         <v>122000</v>
-      </c>
-      <c r="U5" s="26" t="n">
-        <v>105000</v>
       </c>
     </row>
     <row r="6">
@@ -1228,7 +1234,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>5.0163</v>
+        <v>3.7372</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.54</v>
@@ -1386,19 +1392,19 @@
         </is>
       </c>
       <c r="F9" s="24" t="n">
-        <v>16829.681</v>
+        <v>16788.685</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>16687.728</v>
+        <v>16634.157</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>16665.219</v>
+        <v>16604.582</v>
       </c>
       <c r="I9" s="24" t="n">
-        <v>16585.878</v>
+        <v>16526.176</v>
       </c>
       <c r="J9" s="24" t="n">
-        <v>16445.685</v>
+        <v>16378.319</v>
       </c>
       <c r="K9" s="46" t="n"/>
       <c r="L9" s="28" t="inlineStr">
@@ -1461,19 +1467,19 @@
         </is>
       </c>
       <c r="F10" s="25" t="n">
-        <v>0.008506430593787417</v>
+        <v>0.009289800499057588</v>
       </c>
       <c r="G10" s="25" t="n">
-        <v>0.001350657318094584</v>
+        <v>0.001781134869881074</v>
       </c>
       <c r="H10" s="25" t="n">
-        <v>0.004783647872002916</v>
+        <v>0.004744352232482596</v>
       </c>
       <c r="I10" s="25" t="n">
-        <v>0.008524606910566446</v>
+        <v>0.00902760533605429</v>
       </c>
       <c r="J10" s="25" t="n">
-        <v>0.006111174905983452</v>
+        <v>0.005218157797150624</v>
       </c>
       <c r="K10" s="46" t="n"/>
       <c r="L10" s="28" t="inlineStr">
@@ -1526,8 +1532,8 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="51" t="n">
-        <v>46204</v>
+      <c r="C11" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D11" s="45" t="inlineStr">
         <is>
@@ -1540,19 +1546,19 @@
         </is>
       </c>
       <c r="F11" s="25" t="n">
-        <v>-0.01390979158115568</v>
+        <v>0.01928463198493957</v>
       </c>
       <c r="G11" s="25" t="n">
-        <v>0.00767463235294108</v>
+        <v>-0.01085475520029067</v>
       </c>
       <c r="H11" s="25" t="n">
-        <v>0.01091753774680604</v>
+        <v>0.01023170451938515</v>
       </c>
       <c r="I11" s="25" t="n">
-        <v>-0.01148105625717566</v>
+        <v>0.007535133136094663</v>
       </c>
       <c r="J11" s="25" t="n">
-        <v>0.01363932594730488</v>
+        <v>-0.003363280350149767</v>
       </c>
       <c r="K11" s="46" t="n"/>
       <c r="L11" s="28" t="inlineStr">
@@ -1601,8 +1607,8 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="51" t="n">
-        <v>46204</v>
+      <c r="C12" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D12" s="45" t="inlineStr">
         <is>
@@ -1615,19 +1621,19 @@
         </is>
       </c>
       <c r="F12" s="25" t="n">
-        <v>0.009618976466193458</v>
+        <v>0.04613572101790768</v>
       </c>
       <c r="G12" s="25" t="n">
-        <v>0.03727707081697323</v>
+        <v>0.02706908747936812</v>
       </c>
       <c r="H12" s="25" t="n">
-        <v>0.02752986730887292</v>
+        <v>0.04882579907588244</v>
       </c>
       <c r="I12" s="25" t="n">
-        <v>-0.005773672055427252</v>
+        <v>0.03805486759382744</v>
       </c>
       <c r="J12" s="25" t="n">
-        <v>-0.000734248084071364</v>
+        <v>0.009190576160485103</v>
       </c>
       <c r="K12" s="46" t="n"/>
       <c r="L12" s="28" t="inlineStr">
@@ -1680,8 +1686,8 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="51" t="n">
-        <v>46204</v>
+      <c r="C13" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D13" s="45" t="inlineStr">
         <is>
@@ -1694,19 +1700,19 @@
         </is>
       </c>
       <c r="F13" s="25" t="n">
-        <v>-0.002005291742097182</v>
+        <v>0.01016111828439903</v>
       </c>
       <c r="G13" s="25" t="n">
-        <v>0.004925970500153865</v>
+        <v>-0.001261528973115378</v>
       </c>
       <c r="H13" s="25" t="n">
-        <v>-0.001648597295182741</v>
+        <v>0.003996735061499113</v>
       </c>
       <c r="I13" s="25" t="n">
-        <v>0.003702041732106975</v>
+        <v>-0.001629808637985675</v>
       </c>
       <c r="J13" s="25" t="n">
-        <v>0.005754259280153384</v>
+        <v>0.003524899892842992</v>
       </c>
       <c r="K13" s="46" t="n"/>
       <c r="L13" s="28" t="inlineStr">
@@ -1755,8 +1761,8 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="51" t="n">
-        <v>46204</v>
+      <c r="C14" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D14" s="45" t="inlineStr">
         <is>
@@ -1769,19 +1775,19 @@
         </is>
       </c>
       <c r="F14" s="25" t="n">
-        <v>0.01417978036907063</v>
+        <v>0.0175587411994233</v>
       </c>
       <c r="G14" s="25" t="n">
-        <v>0.01921766776427836</v>
+        <v>0.01259130830230501</v>
       </c>
       <c r="H14" s="25" t="n">
-        <v>0.02132464339822197</v>
+        <v>0.01618095319488355</v>
       </c>
       <c r="I14" s="25" t="n">
-        <v>0.02178443968593867</v>
+        <v>0.01924952665098396</v>
       </c>
       <c r="J14" s="25" t="n">
-        <v>0.01787039680274048</v>
+        <v>0.0200647805772924</v>
       </c>
       <c r="K14" s="46" t="n"/>
       <c r="L14" s="28" t="inlineStr">
@@ -1834,8 +1840,8 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="51" t="n">
-        <v>46204</v>
+      <c r="C15" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D15" s="45" t="inlineStr">
         <is>
@@ -1848,19 +1854,19 @@
         </is>
       </c>
       <c r="F15" s="25" t="n">
-        <v>0.002869028833739851</v>
+        <v>0.001990031912223467</v>
       </c>
       <c r="G15" s="25" t="n">
-        <v>0.003770800147592235</v>
+        <v>0.002822674888980803</v>
       </c>
       <c r="H15" s="25" t="n">
-        <v>0.004156989616562967</v>
+        <v>0.003210504482080712</v>
       </c>
       <c r="I15" s="25" t="n">
-        <v>0.003618785031471727</v>
+        <v>0.004265724765656786</v>
       </c>
       <c r="J15" s="25" t="n">
-        <v>0.0001360630606932478</v>
+        <v>0.004119604954438749</v>
       </c>
       <c r="K15" s="46" t="n"/>
       <c r="L15" s="28" t="inlineStr">
@@ -1909,8 +1915,8 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="51" t="n">
-        <v>46204</v>
+      <c r="C16" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D16" s="45" t="inlineStr">
         <is>
@@ -1923,19 +1929,19 @@
         </is>
       </c>
       <c r="F16" s="25" t="n">
-        <v>0.02533641330253361</v>
+        <v>0.02497845104260272</v>
       </c>
       <c r="G16" s="25" t="n">
-        <v>0.02673245452537002</v>
+        <v>0.02472810111699007</v>
       </c>
       <c r="H16" s="25" t="n">
-        <v>0.02489439023040468</v>
+        <v>0.02657758254738746</v>
       </c>
       <c r="I16" s="25" t="n">
-        <v>0.02251894289410467</v>
+        <v>0.02699799020107251</v>
       </c>
       <c r="J16" s="25" t="n">
-        <v>0.02201458987977717</v>
+        <v>0.024229381371576</v>
       </c>
       <c r="K16" s="46" t="n"/>
       <c r="L16" s="28" t="n"/>
@@ -2126,8 +2132,8 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="51" t="n">
-        <v>46204</v>
+      <c r="C19" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D19" s="45" t="inlineStr">
         <is>
@@ -2140,19 +2146,19 @@
         </is>
       </c>
       <c r="F19" s="25" t="n">
-        <v>0.003744135940935589</v>
+        <v>-0.000266081649054728</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>0.003044427530958238</v>
+        <v>0.003104845738190587</v>
       </c>
       <c r="H19" s="25" t="n">
-        <v>0.002394596009377858</v>
+        <v>0.003586110382227004</v>
       </c>
       <c r="I19" s="25" t="n">
-        <v>-0.004070879897950741</v>
+        <v>0.003340299146002312</v>
       </c>
       <c r="J19" s="25" t="n">
-        <v>-0.001185470781469022</v>
+        <v>-0.003808410193644085</v>
       </c>
       <c r="K19" s="46" t="n"/>
       <c r="L19" s="28" t="n"/>
@@ -2197,8 +2203,8 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="51" t="n">
-        <v>46204</v>
+      <c r="C20" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D20" s="45" t="inlineStr">
         <is>
@@ -2211,19 +2217,19 @@
         </is>
       </c>
       <c r="F20" s="25" t="n">
-        <v>0.004523055945102436</v>
+        <v>0.01301309563112138</v>
       </c>
       <c r="G20" s="25" t="n">
-        <v>0.005166433768880193</v>
+        <v>0.01493573774828597</v>
       </c>
       <c r="H20" s="25" t="n">
-        <v>0.001067799720814703</v>
+        <v>0.01491547162301134</v>
       </c>
       <c r="I20" s="25" t="n">
-        <v>-0.009695084625184218</v>
+        <v>0.01221779548472771</v>
       </c>
       <c r="J20" s="25" t="n">
-        <v>7.7652239989875e-05</v>
+        <v>0.002297953282280082</v>
       </c>
       <c r="K20" s="46" t="n"/>
       <c r="L20" s="28" t="inlineStr">
@@ -2276,8 +2282,8 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="51" t="n">
-        <v>46204</v>
+      <c r="C21" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D21" s="45" t="inlineStr">
         <is>
@@ -2290,19 +2296,19 @@
         </is>
       </c>
       <c r="F21" s="45" t="n">
-        <v>3</v>
+        <v>4.1</v>
       </c>
       <c r="G21" s="45" t="n">
-        <v>2.6</v>
+        <v>4.6</v>
       </c>
       <c r="H21" s="45" t="n">
-        <v>2.8</v>
+        <v>4.4</v>
       </c>
       <c r="I21" s="45" t="n">
-        <v>2.9</v>
+        <v>4.4</v>
       </c>
       <c r="J21" s="45" t="n">
-        <v>3.5</v>
+        <v>4.4</v>
       </c>
       <c r="K21" s="46" t="n"/>
       <c r="L21" s="28" t="n"/>
@@ -2365,19 +2371,19 @@
         </is>
       </c>
       <c r="F22" s="24" t="n">
-        <v>17.19</v>
+        <v>16.982</v>
       </c>
       <c r="G22" s="24" t="n">
-        <v>16.757</v>
+        <v>16.58</v>
       </c>
       <c r="H22" s="24" t="n">
-        <v>17.221</v>
+        <v>17.217</v>
       </c>
       <c r="I22" s="24" t="n">
-        <v>16.744</v>
+        <v>16.87</v>
       </c>
       <c r="J22" s="24" t="n">
-        <v>16.636</v>
+        <v>16.544</v>
       </c>
       <c r="K22" s="46" t="n"/>
       <c r="L22" s="28" t="inlineStr">
@@ -2440,19 +2446,19 @@
         </is>
       </c>
       <c r="F23" s="25" t="n">
-        <v>0.01715976331360963</v>
+        <v>0.01415347865034329</v>
       </c>
       <c r="G23" s="25" t="n">
-        <v>-0.01417813860454169</v>
+        <v>-0.01561479546399108</v>
       </c>
       <c r="H23" s="25" t="n">
-        <v>0.05767104778282767</v>
+        <v>0.05438177475656795</v>
       </c>
       <c r="I23" s="25" t="n">
-        <v>0.04369506950071686</v>
+        <v>0.04406485951231586</v>
       </c>
       <c r="J23" s="25" t="n">
-        <v>-0.05385884092589429</v>
+        <v>-0.05549212148892429</v>
       </c>
       <c r="K23" s="46" t="n"/>
       <c r="M23" s="15" t="inlineStr">
@@ -2539,8 +2545,8 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N24" s="51" t="n">
-        <v>46204</v>
+      <c r="N24" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O24" s="45" t="inlineStr">
         <is>
@@ -2553,19 +2559,19 @@
         </is>
       </c>
       <c r="Q24" s="38" t="n">
-        <v>0.00155948088304636</v>
+        <v>0.003102796328484869</v>
       </c>
       <c r="R24" s="38" t="n">
-        <v>-0.0009272207697451629</v>
+        <v>0.0005034094549449808</v>
       </c>
       <c r="S24" s="38" t="n">
-        <v>0.004811143524811712</v>
+        <v>-0.001028641964020527</v>
       </c>
       <c r="T24" s="38" t="n">
-        <v>0.004164014631565349</v>
+        <v>0.004354414105546933</v>
       </c>
       <c r="U24" s="23" t="n">
-        <v>0.006669806004369283</v>
+        <v>0.004358018523500373</v>
       </c>
     </row>
     <row r="25">
@@ -2614,8 +2620,8 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N25" s="51" t="n">
-        <v>46204</v>
+      <c r="N25" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O25" s="45" t="inlineStr">
         <is>
@@ -2628,19 +2634,19 @@
         </is>
       </c>
       <c r="Q25" s="38" t="n">
-        <v>0.03701165721487081</v>
+        <v>0.03419031824505426</v>
       </c>
       <c r="R25" s="38" t="n">
-        <v>0.03716970562476833</v>
+        <v>0.033615431894473</v>
       </c>
       <c r="S25" s="38" t="n">
-        <v>0.04111410033233105</v>
+        <v>0.03453010336936787</v>
       </c>
       <c r="T25" s="38" t="n">
-        <v>0.03801823226317869</v>
+        <v>0.0382333396620468</v>
       </c>
       <c r="U25" s="23" t="n">
-        <v>0.03542928831754543</v>
+        <v>0.03573947987920389</v>
       </c>
     </row>
     <row r="26">
@@ -2668,19 +2674,19 @@
         </is>
       </c>
       <c r="F26" s="38" t="n">
-        <v>0.02059204359604272</v>
+        <v>0.02173921402703938</v>
       </c>
       <c r="G26" s="38" t="n">
-        <v>0.02552585944536068</v>
+        <v>0.02391240953315132</v>
       </c>
       <c r="H26" s="38" t="n">
-        <v>0.005923787970366412</v>
+        <v>0.005295862445843902</v>
       </c>
       <c r="I26" s="38" t="n">
-        <v>0.007794617579222285</v>
+        <v>0.009411852445720736</v>
       </c>
       <c r="J26" s="38" t="n">
-        <v>0.01778138610314484</v>
+        <v>0.01849694172720051</v>
       </c>
       <c r="K26" s="46" t="n"/>
       <c r="L26" s="28" t="inlineStr">
@@ -2693,8 +2699,8 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="51" t="n">
-        <v>46204</v>
+      <c r="N26" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O26" s="45" t="inlineStr">
         <is>
@@ -2707,19 +2713,19 @@
         </is>
       </c>
       <c r="Q26" s="38" t="n">
-        <v>0.002455155058386671</v>
+        <v>0.002474391583994873</v>
       </c>
       <c r="R26" s="38" t="n">
-        <v>0.001467571284778035</v>
+        <v>0.001261839361694106</v>
       </c>
       <c r="S26" s="38" t="n">
-        <v>0.003593433116647615</v>
+        <v>0.001332860796942947</v>
       </c>
       <c r="T26" s="38" t="n">
-        <v>0.002613206744856766</v>
+        <v>0.003099037829900508</v>
       </c>
       <c r="U26" s="23" t="n">
-        <v>0.002962135839517099</v>
+        <v>0.002828799503991286</v>
       </c>
     </row>
     <row r="27">
@@ -2747,19 +2753,19 @@
         </is>
       </c>
       <c r="F27" s="38" t="n">
-        <v>0.00317839655928509</v>
+        <v>0.006940517752098252</v>
       </c>
       <c r="G27" s="38" t="n">
-        <v>-0.0201499882390509</v>
+        <v>-0.01948561470458643</v>
       </c>
       <c r="H27" s="38" t="n">
-        <v>-0.004277328978805506</v>
+        <v>-0.004482704112548475</v>
       </c>
       <c r="I27" s="38" t="n">
-        <v>-0.01832684674964358</v>
+        <v>-0.01618651426201678</v>
       </c>
       <c r="J27" s="38" t="n">
-        <v>-0.01299350008050415</v>
+        <v>-0.01101732062248628</v>
       </c>
       <c r="K27" s="46" t="n"/>
       <c r="L27" s="28" t="n"/>
@@ -2768,8 +2774,8 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="51" t="n">
-        <v>46204</v>
+      <c r="N27" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O27" s="45" t="inlineStr">
         <is>
@@ -2782,19 +2788,19 @@
         </is>
       </c>
       <c r="Q27" s="38" t="n">
-        <v>0.03344143004033837</v>
+        <v>0.03007595976185597</v>
       </c>
       <c r="R27" s="38" t="n">
-        <v>0.03343614465473631</v>
+        <v>0.02983468262070393</v>
       </c>
       <c r="S27" s="38" t="n">
-        <v>0.03463709356864603</v>
+        <v>0.03041234252733225</v>
       </c>
       <c r="T27" s="38" t="n">
-        <v>0.03329827413108968</v>
+        <v>0.0316170977125689</v>
       </c>
       <c r="U27" s="23" t="n">
-        <v>0.03253849776876586</v>
+        <v>0.03083872406870407</v>
       </c>
     </row>
     <row r="28">
@@ -2923,7 +2929,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,19 +2942,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.35</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.34</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.36</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.34</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3008,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,19 +3021,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
-        <v>2.34</v>
+        <v>2.35</v>
       </c>
       <c r="R30" s="45" t="n">
         <v>2.34</v>
       </c>
       <c r="S30" s="45" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="T30" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.35</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.33</v>
       </c>
     </row>
     <row r="31">
@@ -3302,7 +3308,7 @@
         </is>
       </c>
       <c r="N34" s="51" t="n">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="O34" s="45" t="inlineStr">
         <is>
@@ -3315,19 +3321,19 @@
         </is>
       </c>
       <c r="Q34" s="38" t="n">
-        <v>-0.004490110224068822</v>
+        <v>-0.003222678885696339</v>
       </c>
       <c r="R34" s="38" t="n">
-        <v>-0.003221577692024325</v>
+        <v>-0.001219091051912563</v>
       </c>
       <c r="S34" s="38" t="n">
-        <v>-0.007455850803781246</v>
+        <v>-0.0006782988032907144</v>
       </c>
       <c r="T34" s="38" t="n">
-        <v>-0.002219562698691556</v>
+        <v>-0.004701862813512956</v>
       </c>
       <c r="U34" s="23" t="n">
-        <v>-0.001052481507739263</v>
+        <v>-2.432480890000966e-05</v>
       </c>
     </row>
     <row r="35" ht="31.5" customHeight="1">
@@ -3381,7 +3387,7 @@
         </is>
       </c>
       <c r="N35" s="51" t="n">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="O35" s="45" t="inlineStr">
         <is>
@@ -3394,19 +3400,19 @@
         </is>
       </c>
       <c r="Q35" s="38" t="n">
-        <v>3.663118525487619e-05</v>
+        <v>-0.0004453719334049921</v>
       </c>
       <c r="R35" s="38" t="n">
-        <v>0.003597934817094028</v>
+        <v>0.001092209910193764</v>
       </c>
       <c r="S35" s="38" t="n">
-        <v>-0.002659880805601422</v>
+        <v>0.00369982572748162</v>
       </c>
       <c r="T35" s="38" t="n">
-        <v>-0.002546983253221669</v>
+        <v>-0.002206341131705591</v>
       </c>
       <c r="U35" s="23" t="n">
-        <v>-0.004493337788724072</v>
+        <v>-0.002739653360595784</v>
       </c>
     </row>
     <row r="36" ht="31.5" customHeight="1">
@@ -3456,7 +3462,7 @@
         </is>
       </c>
       <c r="N36" s="51" t="n">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="O36" s="45" t="inlineStr">
         <is>
@@ -3469,19 +3475,19 @@
         </is>
       </c>
       <c r="Q36" s="38" t="n">
-        <v>-0.004490110224068822</v>
+        <v>-0.003222678885696339</v>
       </c>
       <c r="R36" s="38" t="n">
-        <v>-0.003221577692024325</v>
+        <v>-0.001219091051912563</v>
       </c>
       <c r="S36" s="38" t="n">
-        <v>-0.007455850803781246</v>
+        <v>-0.0006782988032907144</v>
       </c>
       <c r="T36" s="38" t="n">
-        <v>-0.002219562698691556</v>
+        <v>-0.004701862813512956</v>
       </c>
       <c r="U36" s="23" t="n">
-        <v>-0.001052481507739263</v>
+        <v>-2.432480890000966e-05</v>
       </c>
     </row>
     <row r="37">
@@ -3699,13 +3705,13 @@
       <c r="R39" s="45" t="n">
         <v>120.597</v>
       </c>
-      <c r="S39" s="53" t="n">
+      <c r="S39" s="45" t="n">
         <v>120.0835</v>
       </c>
       <c r="T39" s="53" t="n">
         <v>118.7792</v>
       </c>
-      <c r="U39" s="21" t="n">
+      <c r="U39" s="54" t="n">
         <v>119.0363</v>
       </c>
     </row>
@@ -3774,13 +3780,13 @@
       <c r="R40" s="38" t="n">
         <v>0.004032046569596641</v>
       </c>
-      <c r="S40" s="54" t="n">
+      <c r="S40" s="38" t="n">
         <v>-0.004232386546914929</v>
       </c>
-      <c r="T40" s="54" t="n">
+      <c r="T40" s="55" t="n">
         <v>-0.0291232297604588</v>
       </c>
-      <c r="U40" s="23" t="n">
+      <c r="U40" s="56" t="n">
         <v>-0.04111399852747133</v>
       </c>
     </row>
@@ -4034,19 +4040,19 @@
         </is>
       </c>
       <c r="F44" s="24" t="n">
-        <v>5543.809</v>
+        <v>5626.646</v>
       </c>
       <c r="G44" s="24" t="n">
-        <v>5416.715</v>
+        <v>5483.833</v>
       </c>
       <c r="H44" s="24" t="n">
-        <v>5343.513</v>
+        <v>5409.276</v>
       </c>
       <c r="I44" s="24" t="n">
-        <v>5324.402</v>
+        <v>5404.135</v>
       </c>
       <c r="J44" s="24" t="n">
-        <v>5236.97</v>
+        <v>5332.951</v>
       </c>
       <c r="K44" s="46" t="n"/>
       <c r="L44" s="28" t="n"/>
@@ -4105,19 +4111,19 @@
         </is>
       </c>
       <c r="F45" s="38" t="n">
-        <v>0.02346329832749183</v>
+        <v>0.0260425508946025</v>
       </c>
       <c r="G45" s="38" t="n">
-        <v>0.01369922745579544</v>
+        <v>0.0137831754194091</v>
       </c>
       <c r="H45" s="38" t="n">
-        <v>0.003589323270481781</v>
+        <v>0.0009513085812993261</v>
       </c>
       <c r="I45" s="38" t="n">
-        <v>0.01669515005814426</v>
+        <v>0.01334795688165902</v>
       </c>
       <c r="J45" s="38" t="n">
-        <v>0.007978609251013902</v>
+        <v>0.0111412368534316</v>
       </c>
       <c r="K45" s="46" t="n"/>
       <c r="L45" s="28" t="n"/>
@@ -4269,7 +4275,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4354,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.92</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.81</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.87</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.85</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.71</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.76</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4429,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,16 +4442,16 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>5.06</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.98</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>5.03</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.99</v>
-      </c>
-      <c r="T49" s="45" t="n">
-        <v>4.83</v>
       </c>
       <c r="U49" s="21" t="n">
         <v>4.83</v>
@@ -4502,7 +4508,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,16 +4521,16 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5.24</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>5.17</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>5.18</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>5.11</v>
-      </c>
-      <c r="T50" s="45" t="n">
-        <v>4.96</v>
       </c>
       <c r="U50" s="21" t="n">
         <v>4.96</v>
@@ -4627,8 +4633,8 @@
           <t>DBAA</t>
         </is>
       </c>
-      <c r="N52" s="55" t="n">
-        <v>46293</v>
+      <c r="N52" s="57" t="n">
+        <v>46294</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.72</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.7</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.63</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.57</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.5</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.38</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-01
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>3.7372</v>
+        <v>3.6773</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.54</v>
@@ -1726,7 +1726,7 @@
         </is>
       </c>
       <c r="N13" s="52" t="n">
-        <v>46279</v>
+        <v>46286</v>
       </c>
       <c r="O13" s="45" t="inlineStr">
         <is>
@@ -1745,13 +1745,13 @@
         <v>198000</v>
       </c>
       <c r="S13" s="24" t="n">
-        <v>207000</v>
+        <v>198000</v>
       </c>
       <c r="T13" s="24" t="n">
         <v>207000</v>
       </c>
       <c r="U13" s="26" t="n">
-        <v>204000</v>
+        <v>207000</v>
       </c>
     </row>
     <row r="14">
@@ -1801,7 +1801,7 @@
         </is>
       </c>
       <c r="N14" s="52" t="n">
-        <v>46272</v>
+        <v>46279</v>
       </c>
       <c r="O14" s="45" t="inlineStr">
         <is>
@@ -1814,19 +1814,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1719000</v>
+        <v>1701000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1712000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1717000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1765000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1775000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1771000</v>
       </c>
     </row>
     <row r="15">
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2945,16 +2945,16 @@
         <v>2.36</v>
       </c>
       <c r="R29" s="45" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="S29" s="45" t="n">
         <v>2.35</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.34</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.33</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.36</v>
       </c>
     </row>
     <row r="30">
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3021,19 +3021,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.35</v>
-      </c>
-      <c r="R30" s="45" t="n">
-        <v>2.34</v>
       </c>
       <c r="S30" s="45" t="n">
         <v>2.34</v>
       </c>
       <c r="T30" s="45" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="U30" s="21" t="n">
         <v>2.33</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.35</v>
       </c>
     </row>
     <row r="31">
@@ -3536,8 +3536,8 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="51" t="n">
-        <v>46174</v>
+      <c r="N37" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="O37" s="45" t="inlineStr">
         <is>
@@ -3550,19 +3550,19 @@
         </is>
       </c>
       <c r="Q37" s="38" t="n">
-        <v>0.003675878722833481</v>
+        <v>0.00118133140204435</v>
       </c>
       <c r="R37" s="38" t="n">
-        <v>0.006967689254868681</v>
+        <v>0.003945360923047536</v>
       </c>
       <c r="S37" s="38" t="n">
-        <v>0.00856545961002797</v>
+        <v>0.007306018310070606</v>
       </c>
       <c r="T37" s="38" t="n">
-        <v>0.007608622698956014</v>
+        <v>0.008298830536790813</v>
       </c>
       <c r="U37" s="23" t="n">
-        <v>0.003179830266230477</v>
+        <v>0.007882278295670897</v>
       </c>
     </row>
     <row r="38">
@@ -3611,8 +3611,8 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="51" t="n">
-        <v>46174</v>
+      <c r="N38" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="O38" s="45" t="inlineStr">
         <is>
@@ -3625,19 +3625,19 @@
         </is>
       </c>
       <c r="Q38" s="38" t="n">
-        <v>0.01525308725742975</v>
+        <v>0.01928847496245344</v>
       </c>
       <c r="R38" s="38" t="n">
-        <v>0.01210861241276107</v>
+        <v>0.01611755196583463</v>
       </c>
       <c r="S38" s="38" t="n">
-        <v>0.009742493823792416</v>
+        <v>0.0127260710933798</v>
       </c>
       <c r="T38" s="38" t="n">
-        <v>0.007762345302316447</v>
+        <v>0.01001067158206193</v>
       </c>
       <c r="U38" s="23" t="n">
-        <v>0.008178342616885069</v>
+        <v>0.008275963087739823</v>
       </c>
     </row>
     <row r="39" ht="31.5" customHeight="1">
@@ -3726,7 +3726,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="52" t="n">
+      <c r="C40" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D40" s="45" t="inlineStr">
@@ -3797,7 +3797,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="52" t="n">
+      <c r="C41" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D41" s="45" t="inlineStr">
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4367,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.89</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.92</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.81</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.87</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.85</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.71</v>
       </c>
     </row>
     <row r="49">
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4445,16 +4445,16 @@
         <v>5.06</v>
       </c>
       <c r="R49" s="45" t="n">
+        <v>5.06</v>
+      </c>
+      <c r="S49" s="45" t="n">
         <v>4.98</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>5.03</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.99</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.83</v>
       </c>
     </row>
     <row r="50">
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4521,19 +4521,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5.26</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>5.24</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>5.17</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>5.18</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>5.11</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.96</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4583,7 +4583,7 @@
         </is>
       </c>
       <c r="N51" s="52" t="n">
-        <v>46286</v>
+        <v>46293</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
         <is>
@@ -4596,19 +4596,19 @@
         </is>
       </c>
       <c r="Q51" s="45" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="R51" s="45" t="n">
         <v>7.03</v>
       </c>
-      <c r="R51" s="45" t="n">
+      <c r="S51" s="45" t="n">
         <v>6.95</v>
       </c>
-      <c r="S51" s="45" t="n">
+      <c r="T51" s="45" t="n">
         <v>6.76</v>
       </c>
-      <c r="T51" s="45" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.71</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.66</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="N52" s="57" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4647,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.76</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.72</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.7</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.63</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.57</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.5</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-02
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -955,8 +955,8 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="51" t="n">
-        <v>46235</v>
+      <c r="N3" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O3" s="45" t="inlineStr">
         <is>
@@ -969,19 +969,19 @@
         </is>
       </c>
       <c r="Q3" s="24" t="n">
-        <v>162</v>
+        <v>29</v>
       </c>
       <c r="R3" s="24" t="n">
-        <v>21</v>
+        <v>133</v>
       </c>
       <c r="S3" s="24" t="n">
+        <v>-10</v>
+      </c>
+      <c r="T3" s="24" t="n">
         <v>31</v>
       </c>
-      <c r="T3" s="24" t="n">
+      <c r="U3" s="26" t="n">
         <v>63</v>
-      </c>
-      <c r="U3" s="26" t="n">
-        <v>148</v>
       </c>
     </row>
     <row r="4">
@@ -1026,8 +1026,8 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="51" t="n">
-        <v>46235</v>
+      <c r="N4" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O4" s="45" t="inlineStr">
         <is>
@@ -1040,19 +1040,19 @@
         </is>
       </c>
       <c r="Q4" s="38" t="n">
-        <v>0.003805088596092685</v>
+        <v>0.003128390140525267</v>
       </c>
       <c r="R4" s="38" t="n">
-        <v>0.00234007392362907</v>
+        <v>0.003426472815386945</v>
       </c>
       <c r="S4" s="38" t="n">
+        <v>0.002144542140253056</v>
+      </c>
+      <c r="T4" s="38" t="n">
         <v>0.00261234997917692</v>
       </c>
-      <c r="T4" s="38" t="n">
+      <c r="U4" s="23" t="n">
         <v>0.002290249719239359</v>
-      </c>
-      <c r="U4" s="23" t="n">
-        <v>0.001974950310754961</v>
       </c>
     </row>
     <row r="5" ht="31.5" customHeight="1">
@@ -1180,8 +1180,8 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="51" t="n">
-        <v>46235</v>
+      <c r="N6" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O6" s="45" t="inlineStr">
         <is>
@@ -1194,16 +1194,16 @@
         </is>
       </c>
       <c r="Q6" s="45" t="n">
-        <v>4.1</v>
+        <v>4.2</v>
       </c>
       <c r="R6" s="45" t="n">
         <v>4.1</v>
       </c>
       <c r="S6" s="45" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="T6" s="45" t="n">
         <v>4.2</v>
-      </c>
-      <c r="T6" s="45" t="n">
-        <v>4.3</v>
       </c>
       <c r="U6" s="21" t="n">
         <v>4.3</v>
@@ -1259,8 +1259,8 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="51" t="n">
-        <v>46235</v>
+      <c r="N7" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O7" s="45" t="inlineStr">
         <is>
@@ -1273,19 +1273,19 @@
         </is>
       </c>
       <c r="Q7" s="45" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="R7" s="45" t="n">
         <v>7.7</v>
-      </c>
-      <c r="R7" s="45" t="n">
-        <v>7.9</v>
       </c>
       <c r="S7" s="45" t="n">
         <v>7.9</v>
       </c>
       <c r="T7" s="45" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="U7" s="21" t="n">
         <v>8.1</v>
-      </c>
-      <c r="U7" s="21" t="n">
-        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
@@ -1299,8 +1299,8 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="51" t="n">
-        <v>46204</v>
+      <c r="C8" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D8" s="45" t="inlineStr">
         <is>
@@ -1313,19 +1313,19 @@
         </is>
       </c>
       <c r="F8" s="45" t="n">
-        <v>0.76</v>
+        <v>0.62</v>
       </c>
       <c r="G8" s="45" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.24</v>
       </c>
       <c r="H8" s="45" t="n">
-        <v>0.54</v>
+        <v>0.1</v>
       </c>
       <c r="I8" s="45" t="n">
-        <v>0.46</v>
+        <v>0.12</v>
       </c>
       <c r="J8" s="45" t="n">
-        <v>0.54</v>
+        <v>0.1</v>
       </c>
       <c r="K8" s="46" t="n"/>
       <c r="L8" s="28" t="inlineStr">
@@ -1338,8 +1338,8 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="51" t="n">
-        <v>46235</v>
+      <c r="N8" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O8" s="45" t="inlineStr">
         <is>
@@ -1352,16 +1352,16 @@
         </is>
       </c>
       <c r="Q8" s="45" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="R8" s="45" t="n">
         <v>61.6</v>
       </c>
-      <c r="R8" s="45" t="n">
+      <c r="S8" s="45" t="n">
         <v>61.4</v>
       </c>
-      <c r="S8" s="45" t="n">
+      <c r="T8" s="45" t="n">
         <v>61.5</v>
-      </c>
-      <c r="T8" s="45" t="n">
-        <v>61.8</v>
       </c>
       <c r="U8" s="21" t="n">
         <v>61.8</v>
@@ -1417,8 +1417,8 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="51" t="n">
-        <v>46235</v>
+      <c r="N9" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O9" s="45" t="inlineStr">
         <is>
@@ -1431,19 +1431,19 @@
         </is>
       </c>
       <c r="Q9" s="45" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="R9" s="45" t="n">
         <v>59.1</v>
       </c>
-      <c r="R9" s="45" t="n">
+      <c r="S9" s="45" t="n">
         <v>58.9</v>
       </c>
-      <c r="S9" s="45" t="n">
+      <c r="T9" s="45" t="n">
         <v>59</v>
       </c>
-      <c r="T9" s="45" t="n">
+      <c r="U9" s="21" t="n">
         <v>59.2</v>
-      </c>
-      <c r="U9" s="21" t="n">
-        <v>59.1</v>
       </c>
     </row>
     <row r="10">
@@ -1879,8 +1879,8 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="51" t="n">
-        <v>46235</v>
+      <c r="N15" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O15" s="45" t="inlineStr">
         <is>
@@ -1896,7 +1896,7 @@
         <v>34.4</v>
       </c>
       <c r="R15" s="24" t="n">
-        <v>34.3</v>
+        <v>34.4</v>
       </c>
       <c r="S15" s="24" t="n">
         <v>34.3</v>
@@ -2357,8 +2357,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="51" t="n">
-        <v>46235</v>
+      <c r="C22" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="D22" s="45" t="inlineStr">
         <is>
@@ -2371,19 +2371,19 @@
         </is>
       </c>
       <c r="F22" s="24" t="n">
-        <v>16.982</v>
+        <v>16.378</v>
       </c>
       <c r="G22" s="24" t="n">
-        <v>16.58</v>
+        <v>16.98</v>
       </c>
       <c r="H22" s="24" t="n">
-        <v>17.217</v>
+        <v>16.601</v>
       </c>
       <c r="I22" s="24" t="n">
+        <v>17.218</v>
+      </c>
+      <c r="J22" s="24" t="n">
         <v>16.87</v>
-      </c>
-      <c r="J22" s="24" t="n">
-        <v>16.544</v>
       </c>
       <c r="K22" s="46" t="n"/>
       <c r="L22" s="28" t="inlineStr">
@@ -2432,8 +2432,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="51" t="n">
-        <v>46235</v>
+      <c r="C23" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="D23" s="45" t="inlineStr">
         <is>
@@ -2446,19 +2446,19 @@
         </is>
       </c>
       <c r="F23" s="25" t="n">
-        <v>0.01415347865034329</v>
+        <v>-0.03437297329166903</v>
       </c>
       <c r="G23" s="25" t="n">
-        <v>-0.01561479546399108</v>
+        <v>0.01403404001194383</v>
       </c>
       <c r="H23" s="25" t="n">
-        <v>0.05438177475656795</v>
+        <v>-0.01436798670070658</v>
       </c>
       <c r="I23" s="25" t="n">
+        <v>0.0544430154939065</v>
+      </c>
+      <c r="J23" s="25" t="n">
         <v>0.04406485951231586</v>
-      </c>
-      <c r="J23" s="25" t="n">
-        <v>-0.05549212148892429</v>
       </c>
       <c r="K23" s="46" t="n"/>
       <c r="M23" s="15" t="inlineStr">
@@ -2814,7 +2814,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="52" t="n">
+      <c r="C28" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D28" s="45" t="inlineStr">
@@ -2828,10 +2828,10 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>-0.0001712622024319099</v>
+        <v>-0.0007144966046649381</v>
       </c>
       <c r="G28" s="25" t="n">
-        <v>0.008586004485092946</v>
+        <v>0.008699174159193968</v>
       </c>
       <c r="H28" s="25" t="n">
         <v>0.005802145925317914</v>
@@ -2889,7 +2889,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="52" t="n">
+      <c r="C29" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D29" s="45" t="inlineStr">
@@ -2903,10 +2903,10 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>0.08478942006420237</v>
+        <v>0.08432167823206402</v>
       </c>
       <c r="G29" s="25" t="n">
-        <v>0.1175783415612873</v>
+        <v>0.1177037408590512</v>
       </c>
       <c r="H29" s="25" t="n">
         <v>0.07703978368044752</v>
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2948,13 +2948,13 @@
         <v>2.36</v>
       </c>
       <c r="S29" s="45" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="T29" s="45" t="n">
         <v>2.35</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.34</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.33</v>
       </c>
     </row>
     <row r="30">
@@ -2968,7 +2968,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="52" t="n">
+      <c r="C30" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D30" s="45" t="inlineStr">
@@ -2982,10 +2982,10 @@
         </is>
       </c>
       <c r="F30" s="25" t="n">
-        <v>0.0005108458969496077</v>
+        <v>-7.980998837964215e-05</v>
       </c>
       <c r="G30" s="25" t="n">
-        <v>0.0141466210331016</v>
+        <v>0.01426966328516333</v>
       </c>
       <c r="H30" s="25" t="n">
         <v>0.003538609511678281</v>
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3024,16 +3024,16 @@
         <v>2.36</v>
       </c>
       <c r="R30" s="45" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="S30" s="45" t="n">
         <v>2.35</v>
-      </c>
-      <c r="S30" s="45" t="n">
-        <v>2.34</v>
       </c>
       <c r="T30" s="45" t="n">
         <v>2.34</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.33</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="31">
@@ -3043,7 +3043,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="52" t="n">
+      <c r="C31" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D31" s="45" t="inlineStr">
@@ -3057,10 +3057,10 @@
         </is>
       </c>
       <c r="F31" s="25" t="n">
-        <v>0.0789205492280784</v>
+        <v>0.07841442756607125</v>
       </c>
       <c r="G31" s="25" t="n">
-        <v>0.0989414295087489</v>
+        <v>0.09907475956730888</v>
       </c>
       <c r="H31" s="25" t="n">
         <v>0.05755592766471823</v>
@@ -3232,8 +3232,8 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="51" t="n">
-        <v>46235</v>
+      <c r="N33" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O33" s="45" t="inlineStr">
         <is>
@@ -3246,19 +3246,19 @@
         </is>
       </c>
       <c r="Q33" s="38" t="n">
-        <v>0.002656042496679945</v>
+        <v>0.001324152542373058</v>
       </c>
       <c r="R33" s="38" t="n">
-        <v>0.001596169193934349</v>
+        <v>0.003188097768331399</v>
       </c>
       <c r="S33" s="38" t="n">
+        <v>0.001330140994945328</v>
+      </c>
+      <c r="T33" s="38" t="n">
         <v>0.002667377967457973</v>
       </c>
-      <c r="T33" s="38" t="n">
+      <c r="U33" s="23" t="n">
         <v>0.002138465650895593</v>
-      </c>
-      <c r="U33" s="23" t="n">
-        <v>0.001606425702811221</v>
       </c>
     </row>
     <row r="34" ht="31.5" customHeight="1">
@@ -3321,10 +3321,10 @@
         </is>
       </c>
       <c r="Q34" s="38" t="n">
-        <v>-0.003222678885696339</v>
+        <v>-0.002958631913215778</v>
       </c>
       <c r="R34" s="38" t="n">
-        <v>-0.001219091051912563</v>
+        <v>-0.001484371505816431</v>
       </c>
       <c r="S34" s="38" t="n">
         <v>-0.0006782988032907144</v>
@@ -3400,10 +3400,10 @@
         </is>
       </c>
       <c r="Q35" s="38" t="n">
-        <v>-0.0004453719334049921</v>
+        <v>8.50375855385721e-05</v>
       </c>
       <c r="R35" s="38" t="n">
-        <v>0.001092209910193764</v>
+        <v>0.0008263155649319565</v>
       </c>
       <c r="S35" s="38" t="n">
         <v>0.00369982572748162</v>
@@ -3475,10 +3475,10 @@
         </is>
       </c>
       <c r="Q36" s="38" t="n">
-        <v>-0.003222678885696339</v>
+        <v>-0.002958631913215778</v>
       </c>
       <c r="R36" s="38" t="n">
-        <v>-0.001219091051912563</v>
+        <v>-0.001484371505816431</v>
       </c>
       <c r="S36" s="38" t="n">
         <v>-0.0006782988032907144</v>
@@ -3686,8 +3686,8 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="51" t="n">
-        <v>46235</v>
+      <c r="N39" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O39" s="45" t="inlineStr">
         <is>
@@ -3700,19 +3700,19 @@
         </is>
       </c>
       <c r="Q39" s="45" t="n">
+        <v>119.2152</v>
+      </c>
+      <c r="R39" s="53" t="n">
         <v>118.8512</v>
       </c>
-      <c r="R39" s="45" t="n">
+      <c r="S39" s="45" t="n">
         <v>120.597</v>
       </c>
-      <c r="S39" s="45" t="n">
+      <c r="T39" s="53" t="n">
         <v>120.0835</v>
       </c>
-      <c r="T39" s="53" t="n">
+      <c r="U39" s="54" t="n">
         <v>118.7792</v>
-      </c>
-      <c r="U39" s="54" t="n">
-        <v>119.0363</v>
       </c>
     </row>
     <row r="40" ht="31.5" customHeight="1">
@@ -3761,8 +3761,8 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="51" t="n">
-        <v>46235</v>
+      <c r="N40" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O40" s="45" t="inlineStr">
         <is>
@@ -3775,19 +3775,19 @@
         </is>
       </c>
       <c r="Q40" s="38" t="n">
+        <v>-0.006780855642506724</v>
+      </c>
+      <c r="R40" s="55" t="n">
         <v>-0.01430303593258345</v>
       </c>
-      <c r="R40" s="38" t="n">
+      <c r="S40" s="38" t="n">
         <v>0.004032046569596641</v>
       </c>
-      <c r="S40" s="38" t="n">
+      <c r="T40" s="55" t="n">
         <v>-0.004232386546914929</v>
       </c>
-      <c r="T40" s="55" t="n">
+      <c r="U40" s="56" t="n">
         <v>-0.0291232297604588</v>
-      </c>
-      <c r="U40" s="56" t="n">
-        <v>-0.04111399852747133</v>
       </c>
     </row>
     <row r="41">
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4367,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.89</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.92</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.81</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.87</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.85</v>
       </c>
     </row>
     <row r="49">
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4442,19 +4442,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
-        <v>5.06</v>
+        <v>5.09</v>
       </c>
       <c r="R49" s="45" t="n">
         <v>5.06</v>
       </c>
       <c r="S49" s="45" t="n">
+        <v>5.06</v>
+      </c>
+      <c r="T49" s="45" t="n">
         <v>4.98</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>5.03</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.99</v>
       </c>
     </row>
     <row r="50">
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4521,19 +4521,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5.29</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>5.26</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>5.24</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>5.17</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>5.18</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>5.11</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="N52" s="57" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4647,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.73</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.76</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.72</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.7</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.63</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.57</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-03
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2942,7 +2942,7 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
-        <v>2.36</v>
+        <v>2.35</v>
       </c>
       <c r="R29" s="45" t="n">
         <v>2.36</v>
@@ -2951,10 +2951,10 @@
         <v>2.36</v>
       </c>
       <c r="T29" s="45" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="U29" s="21" t="n">
         <v>2.35</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.34</v>
       </c>
     </row>
     <row r="30">
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3027,10 +3027,10 @@
         <v>2.36</v>
       </c>
       <c r="S30" s="45" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="T30" s="45" t="n">
         <v>2.35</v>
-      </c>
-      <c r="T30" s="45" t="n">
-        <v>2.34</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.34</v>
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4367,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.88</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.89</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.92</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.81</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.87</v>
       </c>
     </row>
     <row r="49">
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4442,19 +4442,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>5.01</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>5.09</v>
-      </c>
-      <c r="R49" s="45" t="n">
-        <v>5.06</v>
       </c>
       <c r="S49" s="45" t="n">
         <v>5.06</v>
       </c>
       <c r="T49" s="45" t="n">
+        <v>5.06</v>
+      </c>
+      <c r="U49" s="21" t="n">
         <v>4.98</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>5.03</v>
       </c>
     </row>
     <row r="50">
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4521,19 +4521,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5.24</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>5.29</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>5.26</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>5.24</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>5.17</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>5.18</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-05
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2942,10 +2942,10 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.35</v>
-      </c>
-      <c r="R29" s="45" t="n">
-        <v>2.36</v>
       </c>
       <c r="S29" s="45" t="n">
         <v>2.36</v>
@@ -2954,7 +2954,7 @@
         <v>2.36</v>
       </c>
       <c r="U29" s="21" t="n">
-        <v>2.35</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="30">
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3030,10 +3030,10 @@
         <v>2.36</v>
       </c>
       <c r="T30" s="45" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="U30" s="21" t="n">
         <v>2.35</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.34</v>
       </c>
     </row>
     <row r="31">
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4367,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.83</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.78</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.88</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.89</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.92</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.81</v>
       </c>
     </row>
     <row r="49">
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4442,19 +4442,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>5.06</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>5.01</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>5.09</v>
-      </c>
-      <c r="S49" s="45" t="n">
-        <v>5.06</v>
       </c>
       <c r="T49" s="45" t="n">
         <v>5.06</v>
       </c>
       <c r="U49" s="21" t="n">
-        <v>4.98</v>
+        <v>5.06</v>
       </c>
     </row>
     <row r="50">
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4521,19 +4521,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>5.24</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>5.29</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>5.26</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>5.24</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>5.17</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="N52" s="57" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4647,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.73</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.76</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.72</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.7</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.63</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-06
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>3.6773</v>
+        <v>3.6844</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.54</v>
@@ -1492,7 +1492,7 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="52" t="n">
+      <c r="N10" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O10" s="45" t="inlineStr">
@@ -1571,7 +1571,7 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="52" t="n">
+      <c r="N11" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O11" s="45" t="inlineStr">
@@ -1646,7 +1646,7 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="52" t="n">
+      <c r="N12" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O12" s="45" t="inlineStr">
@@ -3536,7 +3536,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="52" t="n">
+      <c r="N37" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O37" s="45" t="inlineStr">
@@ -3611,7 +3611,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="52" t="n">
+      <c r="N38" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O38" s="45" t="inlineStr">
@@ -4148,8 +4148,8 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="51" t="n">
-        <v>46204</v>
+      <c r="C46" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D46" s="45" t="inlineStr">
         <is>
@@ -4162,19 +4162,19 @@
         </is>
       </c>
       <c r="F46" s="24" t="n">
+        <v>315182</v>
+      </c>
+      <c r="G46" s="24" t="n">
         <v>310723</v>
       </c>
-      <c r="G46" s="24" t="n">
+      <c r="H46" s="24" t="n">
         <v>317335</v>
       </c>
-      <c r="H46" s="24" t="n">
+      <c r="I46" s="24" t="n">
         <v>319979</v>
       </c>
-      <c r="I46" s="24" t="n">
+      <c r="J46" s="24" t="n">
         <v>329893</v>
-      </c>
-      <c r="J46" s="24" t="n">
-        <v>321163</v>
       </c>
       <c r="K46" s="46" t="n"/>
       <c r="L46" s="29" t="inlineStr">
@@ -4235,8 +4235,8 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="51" t="n">
-        <v>46204</v>
+      <c r="C47" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D47" s="45" t="inlineStr">
         <is>
@@ -4249,19 +4249,19 @@
         </is>
       </c>
       <c r="F47" s="38" t="n">
+        <v>0.01435040212665295</v>
+      </c>
+      <c r="G47" s="38" t="n">
         <v>-0.020836025020877</v>
       </c>
-      <c r="G47" s="38" t="n">
+      <c r="H47" s="38" t="n">
         <v>-0.008263042262148468</v>
       </c>
-      <c r="H47" s="38" t="n">
+      <c r="I47" s="38" t="n">
         <v>-0.03005216843036984</v>
       </c>
-      <c r="I47" s="38" t="n">
+      <c r="J47" s="38" t="n">
         <v>0.02718245875147507</v>
-      </c>
-      <c r="J47" s="38" t="n">
-        <v>0.02402527835524881</v>
       </c>
       <c r="K47" s="46" t="n"/>
       <c r="L47" s="28" t="inlineStr">
@@ -4314,8 +4314,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="51" t="n">
-        <v>46204</v>
+      <c r="C48" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D48" s="45" t="inlineStr">
         <is>
@@ -4328,19 +4328,19 @@
         </is>
       </c>
       <c r="F48" s="24" t="n">
-        <v>399299</v>
+        <v>420754</v>
       </c>
       <c r="G48" s="24" t="n">
+        <v>403550</v>
+      </c>
+      <c r="H48" s="24" t="n">
         <v>388517</v>
       </c>
-      <c r="H48" s="24" t="n">
+      <c r="I48" s="24" t="n">
         <v>395731</v>
       </c>
-      <c r="I48" s="24" t="n">
+      <c r="J48" s="24" t="n">
         <v>382776</v>
-      </c>
-      <c r="J48" s="24" t="n">
-        <v>374820</v>
       </c>
       <c r="K48" s="46" t="n"/>
       <c r="L48" s="28" t="inlineStr">
@@ -4389,8 +4389,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="51" t="n">
-        <v>46204</v>
+      <c r="C49" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D49" s="45" t="inlineStr">
         <is>
@@ -4403,19 +4403,19 @@
         </is>
       </c>
       <c r="F49" s="38" t="n">
-        <v>0.02775168139360695</v>
+        <v>0.04263164415809695</v>
       </c>
       <c r="G49" s="38" t="n">
+        <v>0.03869328755241086</v>
+      </c>
+      <c r="H49" s="38" t="n">
         <v>-0.01822955492493639</v>
       </c>
-      <c r="H49" s="38" t="n">
+      <c r="I49" s="38" t="n">
         <v>0.03384485965682282</v>
       </c>
-      <c r="I49" s="38" t="n">
+      <c r="J49" s="38" t="n">
         <v>0.02122618857051384</v>
-      </c>
-      <c r="J49" s="38" t="n">
-        <v>0.02374312738475992</v>
       </c>
       <c r="K49" s="46" t="n"/>
       <c r="L49" s="28" t="inlineStr">
@@ -4468,8 +4468,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="51" t="n">
-        <v>46204</v>
+      <c r="C50" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D50" s="45" t="inlineStr">
         <is>
@@ -4482,19 +4482,19 @@
         </is>
       </c>
       <c r="F50" s="24" t="n">
-        <v>31016</v>
+        <v>31000</v>
       </c>
       <c r="G50" s="24" t="n">
+        <v>30982</v>
+      </c>
+      <c r="H50" s="24" t="n">
         <v>30791</v>
       </c>
-      <c r="H50" s="24" t="n">
+      <c r="I50" s="24" t="n">
         <v>30517</v>
       </c>
-      <c r="I50" s="24" t="n">
+      <c r="J50" s="24" t="n">
         <v>30177</v>
-      </c>
-      <c r="J50" s="24" t="n">
-        <v>32455</v>
       </c>
       <c r="K50" s="46" t="n"/>
       <c r="L50" s="28" t="inlineStr">
@@ -4543,8 +4543,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="51" t="n">
-        <v>46204</v>
+      <c r="C51" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D51" s="45" t="inlineStr">
         <is>
@@ -4557,19 +4557,19 @@
         </is>
       </c>
       <c r="F51" s="38" t="n">
-        <v>0.007307330063979656</v>
+        <v>0.0005809825059712725</v>
       </c>
       <c r="G51" s="38" t="n">
+        <v>0.00620311129875617</v>
+      </c>
+      <c r="H51" s="38" t="n">
         <v>0.008978602090637944</v>
       </c>
-      <c r="H51" s="38" t="n">
+      <c r="I51" s="38" t="n">
         <v>0.01126685886602385</v>
       </c>
-      <c r="I51" s="38" t="n">
+      <c r="J51" s="38" t="n">
         <v>-0.07018949314435374</v>
-      </c>
-      <c r="J51" s="38" t="n">
-        <v>0.08060864353732433</v>
       </c>
       <c r="K51" s="46" t="n"/>
       <c r="L51" s="28" t="inlineStr">
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="N52" s="57" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4647,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.77</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.75</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.73</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.76</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.72</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.7</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-07
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1105,7 +1105,7 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="52" t="n">
+      <c r="N5" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="O5" s="45" t="inlineStr">
@@ -1532,7 +1532,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="52" t="n">
+      <c r="C11" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="45" t="inlineStr">
@@ -1607,7 +1607,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="52" t="n">
+      <c r="C12" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="45" t="inlineStr">
@@ -1686,7 +1686,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="52" t="n">
+      <c r="C13" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="45" t="inlineStr">
@@ -1761,7 +1761,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="52" t="n">
+      <c r="C14" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="45" t="inlineStr">
@@ -1840,7 +1840,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="52" t="n">
+      <c r="C15" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="45" t="inlineStr">
@@ -1915,7 +1915,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="52" t="n">
+      <c r="C16" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="45" t="inlineStr">
@@ -2132,7 +2132,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="52" t="n">
+      <c r="C19" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="45" t="inlineStr">
@@ -2203,7 +2203,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="52" t="n">
+      <c r="C20" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="45" t="inlineStr">
@@ -2282,7 +2282,7 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="52" t="n">
+      <c r="C21" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D21" s="45" t="inlineStr">
@@ -2506,8 +2506,8 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="51" t="n">
-        <v>46204</v>
+      <c r="C24" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D24" s="45" t="inlineStr">
         <is>
@@ -2520,19 +2520,19 @@
         </is>
       </c>
       <c r="F24" s="38" t="n">
-        <v>0.002069337953391592</v>
+        <v>-0.003526891785422759</v>
       </c>
       <c r="G24" s="38" t="n">
+        <v>0.002054025110949986</v>
+      </c>
+      <c r="H24" s="38" t="n">
         <v>0.004986963805690525</v>
       </c>
-      <c r="H24" s="38" t="n">
+      <c r="I24" s="38" t="n">
         <v>-0.001636032119741393</v>
       </c>
-      <c r="I24" s="38" t="n">
+      <c r="J24" s="38" t="n">
         <v>0.008761168564920929</v>
-      </c>
-      <c r="J24" s="38" t="n">
-        <v>0.008334847450631955</v>
       </c>
       <c r="K24" s="46" t="n"/>
       <c r="L24" s="28" t="inlineStr">
@@ -2545,7 +2545,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N24" s="52" t="n">
+      <c r="N24" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O24" s="45" t="inlineStr">
@@ -2585,8 +2585,8 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="51" t="n">
-        <v>46204</v>
+      <c r="C25" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D25" s="45" t="inlineStr">
         <is>
@@ -2599,19 +2599,19 @@
         </is>
       </c>
       <c r="F25" s="38" t="n">
-        <v>0.004001237090364151</v>
+        <v>0.003410672553578076</v>
       </c>
       <c r="G25" s="38" t="n">
-        <v>0.002058428469037255</v>
+        <v>0.003919489291496436</v>
       </c>
       <c r="H25" s="38" t="n">
-        <v>0.001101254055870582</v>
+        <v>0.00226259325942535</v>
       </c>
       <c r="I25" s="38" t="n">
-        <v>0.002229132702467274</v>
+        <v>0.001341721704025023</v>
       </c>
       <c r="J25" s="38" t="n">
-        <v>0.002637510626163131</v>
+        <v>0.002471524029989514</v>
       </c>
       <c r="K25" s="46" t="n"/>
       <c r="L25" s="28" t="n"/>
@@ -2620,7 +2620,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N25" s="52" t="n">
+      <c r="N25" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O25" s="45" t="inlineStr">
@@ -2699,7 +2699,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="52" t="n">
+      <c r="N26" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O26" s="45" t="inlineStr">
@@ -2774,7 +2774,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="52" t="n">
+      <c r="N27" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O27" s="45" t="inlineStr">
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2942,13 +2942,13 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.36</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.35</v>
-      </c>
-      <c r="S29" s="45" t="n">
-        <v>2.36</v>
       </c>
       <c r="T29" s="45" t="n">
         <v>2.36</v>
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
         <v>2.36</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.35</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="31">
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4367,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.83</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.78</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.88</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.89</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.92</v>
       </c>
     </row>
     <row r="49">
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4445,13 +4445,13 @@
         <v>5.06</v>
       </c>
       <c r="R49" s="45" t="n">
+        <v>5.06</v>
+      </c>
+      <c r="S49" s="45" t="n">
         <v>5.01</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>5.09</v>
-      </c>
-      <c r="T49" s="45" t="n">
-        <v>5.06</v>
       </c>
       <c r="U49" s="21" t="n">
         <v>5.06</v>
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4521,19 +4521,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5.31</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>5.28</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>5.24</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>5.29</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>5.26</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>5.24</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="N52" s="57" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4647,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.73</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.77</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.75</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.73</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.76</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.72</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-08
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>3.6844</v>
+        <v>3.5862</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.54</v>
@@ -1299,7 +1299,7 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="52" t="n">
+      <c r="C8" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="45" t="inlineStr">
@@ -1726,7 +1726,7 @@
         </is>
       </c>
       <c r="N13" s="52" t="n">
-        <v>46286</v>
+        <v>46293</v>
       </c>
       <c r="O13" s="45" t="inlineStr">
         <is>
@@ -1742,13 +1742,13 @@
         <v>197000</v>
       </c>
       <c r="R13" s="24" t="n">
-        <v>198000</v>
+        <v>199000</v>
       </c>
       <c r="S13" s="24" t="n">
         <v>198000</v>
       </c>
       <c r="T13" s="24" t="n">
-        <v>207000</v>
+        <v>198000</v>
       </c>
       <c r="U13" s="26" t="n">
         <v>207000</v>
@@ -1801,7 +1801,7 @@
         </is>
       </c>
       <c r="N14" s="52" t="n">
-        <v>46279</v>
+        <v>46286</v>
       </c>
       <c r="O14" s="45" t="inlineStr">
         <is>
@@ -1814,19 +1814,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1701000</v>
+        <v>1716000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1699000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1712000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1717000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1765000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1775000</v>
       </c>
     </row>
     <row r="15">
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2945,13 +2945,13 @@
         <v>2.35</v>
       </c>
       <c r="R29" s="45" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="S29" s="45" t="n">
         <v>2.36</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.35</v>
-      </c>
-      <c r="T29" s="45" t="n">
-        <v>2.36</v>
       </c>
       <c r="U29" s="21" t="n">
         <v>2.36</v>
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3686,7 +3686,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="52" t="n">
+      <c r="N39" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="O39" s="45" t="inlineStr">
@@ -3761,7 +3761,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="52" t="n">
+      <c r="N40" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="O40" s="45" t="inlineStr">
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4367,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.79</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.84</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.83</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.78</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.88</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.89</v>
       </c>
     </row>
     <row r="49">
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4442,19 +4442,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
-        <v>5.06</v>
+        <v>5.03</v>
       </c>
       <c r="R49" s="45" t="n">
         <v>5.06</v>
       </c>
       <c r="S49" s="45" t="n">
+        <v>5.06</v>
+      </c>
+      <c r="T49" s="45" t="n">
         <v>5.01</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>5.09</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>5.06</v>
       </c>
     </row>
     <row r="50">
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4521,19 +4521,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>5.31</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>5.28</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>5.24</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>5.29</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>5.26</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4583,7 +4583,7 @@
         </is>
       </c>
       <c r="N51" s="52" t="n">
-        <v>46293</v>
+        <v>46300</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
         <is>
@@ -4596,19 +4596,19 @@
         </is>
       </c>
       <c r="Q51" s="45" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="R51" s="45" t="n">
         <v>7.28</v>
       </c>
-      <c r="R51" s="45" t="n">
+      <c r="S51" s="45" t="n">
         <v>7.03</v>
       </c>
-      <c r="S51" s="45" t="n">
+      <c r="T51" s="45" t="n">
         <v>6.95</v>
       </c>
-      <c r="T51" s="45" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.76</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.71</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="N52" s="57" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4647,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.74</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.73</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.77</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.75</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.73</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.76</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-09
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -955,7 +955,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="52" t="n">
+      <c r="N3" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="O3" s="45" t="inlineStr">
@@ -1026,7 +1026,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="52" t="n">
+      <c r="N4" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="O4" s="45" t="inlineStr">
@@ -1180,7 +1180,7 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="52" t="n">
+      <c r="N6" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="O6" s="45" t="inlineStr">
@@ -1259,7 +1259,7 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="52" t="n">
+      <c r="N7" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="O7" s="45" t="inlineStr">
@@ -1338,7 +1338,7 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="52" t="n">
+      <c r="N8" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="O8" s="45" t="inlineStr">
@@ -1417,7 +1417,7 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="52" t="n">
+      <c r="N9" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="O9" s="45" t="inlineStr">
@@ -1879,7 +1879,7 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="52" t="n">
+      <c r="N15" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="O15" s="45" t="inlineStr">
@@ -2357,7 +2357,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="52" t="n">
+      <c r="C22" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="D22" s="45" t="inlineStr">
@@ -2432,7 +2432,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="52" t="n">
+      <c r="C23" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="D23" s="45" t="inlineStr">
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2942,19 +2942,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
-        <v>2.35</v>
+        <v>2.33</v>
       </c>
       <c r="R29" s="45" t="n">
         <v>2.35</v>
       </c>
       <c r="S29" s="45" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="T29" s="45" t="n">
         <v>2.36</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.35</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.36</v>
       </c>
     </row>
     <row r="30">
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3021,7 +3021,7 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
-        <v>2.36</v>
+        <v>2.35</v>
       </c>
       <c r="R30" s="45" t="n">
         <v>2.36</v>
@@ -3232,7 +3232,7 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="52" t="n">
+      <c r="N33" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="O33" s="45" t="inlineStr">
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4367,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.77</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.79</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.84</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.83</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.78</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.88</v>
       </c>
     </row>
     <row r="49">
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4445,16 +4445,16 @@
         <v>5.03</v>
       </c>
       <c r="R49" s="45" t="n">
-        <v>5.06</v>
+        <v>5.03</v>
       </c>
       <c r="S49" s="45" t="n">
         <v>5.06</v>
       </c>
       <c r="T49" s="45" t="n">
+        <v>5.06</v>
+      </c>
+      <c r="U49" s="21" t="n">
         <v>5.01</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>5.09</v>
       </c>
     </row>
     <row r="50">
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4521,19 +4521,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>5.27</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>5.31</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>5.28</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>5.24</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>5.29</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="N52" s="57" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4647,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.74</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.73</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.77</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.75</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.73</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-10
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2942,19 +2942,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.33</v>
-      </c>
-      <c r="R29" s="45" t="n">
-        <v>2.35</v>
       </c>
       <c r="S29" s="45" t="n">
         <v>2.35</v>
       </c>
       <c r="T29" s="45" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="U29" s="21" t="n">
         <v>2.36</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.35</v>
       </c>
     </row>
     <row r="30">
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3021,10 +3021,10 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.35</v>
-      </c>
-      <c r="R30" s="45" t="n">
-        <v>2.36</v>
       </c>
       <c r="S30" s="45" t="n">
         <v>2.36</v>
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4367,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.77</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.79</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.84</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.83</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.78</v>
       </c>
     </row>
     <row r="49">
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4442,19 +4442,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
-        <v>5.03</v>
+        <v>4.99</v>
       </c>
       <c r="R49" s="45" t="n">
         <v>5.03</v>
       </c>
       <c r="S49" s="45" t="n">
-        <v>5.06</v>
+        <v>5.03</v>
       </c>
       <c r="T49" s="45" t="n">
         <v>5.06</v>
       </c>
       <c r="U49" s="21" t="n">
-        <v>5.01</v>
+        <v>5.06</v>
       </c>
     </row>
     <row r="50">
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4521,19 +4521,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5.22</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>5.28</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>5.27</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>5.31</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>5.28</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>5.24</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-11
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1879,8 +1879,10 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="51" t="n">
-        <v>46266</v>
+      <c r="N15" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'AWHAETP' not found in values file."</t>
+        </is>
       </c>
       <c r="O15" s="45" t="inlineStr">
         <is>
@@ -1893,19 +1895,19 @@
         </is>
       </c>
       <c r="Q15" s="24" t="n">
-        <v>34.4</v>
+        <v>1</v>
       </c>
       <c r="R15" s="24" t="n">
-        <v>34.4</v>
+        <v>1</v>
       </c>
       <c r="S15" s="24" t="n">
-        <v>34.3</v>
+        <v>1</v>
       </c>
       <c r="T15" s="24" t="n">
-        <v>34.3</v>
+        <v>1</v>
       </c>
       <c r="U15" s="26" t="n">
-        <v>34.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-12
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1840,8 +1840,10 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="51" t="n">
-        <v>46235</v>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCESC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D15" s="45" t="inlineStr">
         <is>
@@ -1854,19 +1856,19 @@
         </is>
       </c>
       <c r="F15" s="25" t="n">
-        <v>0.001990031912223467</v>
+        <v>1</v>
       </c>
       <c r="G15" s="25" t="n">
-        <v>0.002822674888980803</v>
+        <v>1</v>
       </c>
       <c r="H15" s="25" t="n">
-        <v>0.003210504482080712</v>
+        <v>1</v>
       </c>
       <c r="I15" s="25" t="n">
-        <v>0.004265724765656786</v>
+        <v>1</v>
       </c>
       <c r="J15" s="25" t="n">
-        <v>0.004119604954438749</v>
+        <v>1</v>
       </c>
       <c r="K15" s="46" t="n"/>
       <c r="L15" s="28" t="inlineStr">
@@ -1879,10 +1881,8 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'AWHAETP' not found in values file."</t>
-        </is>
+      <c r="N15" s="51" t="n">
+        <v>46266</v>
       </c>
       <c r="O15" s="45" t="inlineStr">
         <is>
@@ -1895,19 +1895,19 @@
         </is>
       </c>
       <c r="Q15" s="24" t="n">
-        <v>1</v>
+        <v>34.4</v>
       </c>
       <c r="R15" s="24" t="n">
-        <v>1</v>
+        <v>34.4</v>
       </c>
       <c r="S15" s="24" t="n">
-        <v>1</v>
+        <v>34.3</v>
       </c>
       <c r="T15" s="24" t="n">
-        <v>1</v>
+        <v>34.3</v>
       </c>
       <c r="U15" s="26" t="n">
-        <v>1</v>
+        <v>34.3</v>
       </c>
     </row>
     <row r="16">
@@ -1917,8 +1917,10 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="51" t="n">
-        <v>46235</v>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCESC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D16" s="45" t="inlineStr">
         <is>
@@ -1931,19 +1933,19 @@
         </is>
       </c>
       <c r="F16" s="25" t="n">
-        <v>0.02497845104260272</v>
+        <v>1</v>
       </c>
       <c r="G16" s="25" t="n">
-        <v>0.02472810111699007</v>
+        <v>1</v>
       </c>
       <c r="H16" s="25" t="n">
-        <v>0.02657758254738746</v>
+        <v>1</v>
       </c>
       <c r="I16" s="25" t="n">
-        <v>0.02699799020107251</v>
+        <v>1</v>
       </c>
       <c r="J16" s="25" t="n">
-        <v>0.024229381371576</v>
+        <v>1</v>
       </c>
       <c r="K16" s="46" t="n"/>
       <c r="L16" s="28" t="n"/>

</xml_diff>

<commit_message>
Update dashboards - 2026-10-13
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1840,10 +1840,8 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCESC96' not found in values file."</t>
-        </is>
+      <c r="C15" s="51" t="n">
+        <v>46235</v>
       </c>
       <c r="D15" s="45" t="inlineStr">
         <is>
@@ -1856,19 +1854,19 @@
         </is>
       </c>
       <c r="F15" s="25" t="n">
-        <v>1</v>
+        <v>0.001990031912223467</v>
       </c>
       <c r="G15" s="25" t="n">
-        <v>1</v>
+        <v>0.002822674888980803</v>
       </c>
       <c r="H15" s="25" t="n">
-        <v>1</v>
+        <v>0.003210504482080712</v>
       </c>
       <c r="I15" s="25" t="n">
-        <v>1</v>
+        <v>0.004265724765656786</v>
       </c>
       <c r="J15" s="25" t="n">
-        <v>1</v>
+        <v>0.004119604954438749</v>
       </c>
       <c r="K15" s="46" t="n"/>
       <c r="L15" s="28" t="inlineStr">
@@ -1917,10 +1915,8 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCESC96' not found in values file."</t>
-        </is>
+      <c r="C16" s="51" t="n">
+        <v>46235</v>
       </c>
       <c r="D16" s="45" t="inlineStr">
         <is>
@@ -1933,19 +1929,19 @@
         </is>
       </c>
       <c r="F16" s="25" t="n">
-        <v>1</v>
+        <v>0.02497845104260272</v>
       </c>
       <c r="G16" s="25" t="n">
-        <v>1</v>
+        <v>0.02472810111699007</v>
       </c>
       <c r="H16" s="25" t="n">
-        <v>1</v>
+        <v>0.02657758254738746</v>
       </c>
       <c r="I16" s="25" t="n">
-        <v>1</v>
+        <v>0.02699799020107251</v>
       </c>
       <c r="J16" s="25" t="n">
-        <v>1</v>
+        <v>0.024229381371576</v>
       </c>
       <c r="K16" s="46" t="n"/>
       <c r="L16" s="28" t="n"/>
@@ -3881,7 +3877,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="D42" s="45" t="inlineStr">
         <is>
@@ -3894,19 +3890,19 @@
         </is>
       </c>
       <c r="F42" s="39" t="n">
-        <v>3980000</v>
+        <v>3990000</v>
       </c>
       <c r="G42" s="39" t="n">
+        <v>3930000</v>
+      </c>
+      <c r="H42" s="39" t="n">
         <v>4060000</v>
       </c>
-      <c r="H42" s="39" t="n">
+      <c r="I42" s="39" t="n">
         <v>4130000</v>
       </c>
-      <c r="I42" s="39" t="n">
+      <c r="J42" s="39" t="n">
         <v>4190000</v>
-      </c>
-      <c r="J42" s="39" t="n">
-        <v>4040000</v>
       </c>
       <c r="K42" s="7" t="n"/>
       <c r="L42" s="28" t="n"/>
@@ -3952,7 +3948,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="D43" s="45" t="inlineStr">
         <is>
@@ -3965,7 +3961,7 @@
         </is>
       </c>
       <c r="F43" s="38" t="n">
-        <v>-0.01240694789081886</v>
+        <v>-0.02205882352941177</v>
       </c>
       <c r="G43" s="38" t="n">
         <v/>
@@ -4152,7 +4148,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="52" t="n">
+      <c r="C46" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D46" s="45" t="inlineStr">
@@ -4239,7 +4235,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="52" t="n">
+      <c r="C47" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D47" s="45" t="inlineStr">
@@ -4318,7 +4314,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="52" t="n">
+      <c r="C48" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D48" s="45" t="inlineStr">
@@ -4393,7 +4389,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="52" t="n">
+      <c r="C49" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D49" s="45" t="inlineStr">
@@ -4472,7 +4468,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="52" t="n">
+      <c r="C50" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D50" s="45" t="inlineStr">
@@ -4547,7 +4543,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="52" t="n">
+      <c r="C51" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D51" s="45" t="inlineStr">
@@ -4638,7 +4634,7 @@
         </is>
       </c>
       <c r="N52" s="57" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4651,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.69</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.7</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.74</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.73</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.77</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.75</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-14
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2092,8 +2092,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="51" t="n">
-        <v>46235</v>
+      <c r="N18" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O18" s="45" t="inlineStr">
         <is>
@@ -2106,19 +2106,19 @@
         </is>
       </c>
       <c r="Q18" s="38" t="n">
+        <v>0.006485480245771891</v>
+      </c>
+      <c r="R18" s="38" t="n">
         <v>0.003960181843858157</v>
       </c>
-      <c r="R18" s="38" t="n">
+      <c r="S18" s="38" t="n">
         <v>0.0007366914435544825</v>
       </c>
-      <c r="S18" s="38" t="n">
+      <c r="T18" s="38" t="n">
         <v>-0.004224816530380648</v>
       </c>
-      <c r="T18" s="38" t="n">
+      <c r="U18" s="23" t="n">
         <v>0.004729142286413968</v>
-      </c>
-      <c r="U18" s="23" t="n">
-        <v>0.006400377846336402</v>
       </c>
     </row>
     <row r="19" ht="31.5" customHeight="1">
@@ -2167,8 +2167,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="51" t="n">
-        <v>46235</v>
+      <c r="N19" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O19" s="45" t="inlineStr">
         <is>
@@ -2181,19 +2181,19 @@
         </is>
       </c>
       <c r="Q19" s="38" t="n">
+        <v>0.03717250844268993</v>
+      </c>
+      <c r="R19" s="38" t="n">
         <v>0.03353016322755652</v>
       </c>
-      <c r="R19" s="38" t="n">
+      <c r="S19" s="38" t="n">
         <v>0.03303856050706308</v>
       </c>
-      <c r="S19" s="38" t="n">
+      <c r="T19" s="38" t="n">
         <v>0.03463530729385406</v>
       </c>
-      <c r="T19" s="38" t="n">
+      <c r="U19" s="23" t="n">
         <v>0.04166614684049648</v>
-      </c>
-      <c r="U19" s="23" t="n">
-        <v>0.03779245836741563</v>
       </c>
     </row>
     <row r="20">
@@ -2242,8 +2242,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="51" t="n">
-        <v>46235</v>
+      <c r="N20" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O20" s="45" t="inlineStr">
         <is>
@@ -2256,19 +2256,19 @@
         </is>
       </c>
       <c r="Q20" s="38" t="n">
+        <v>0.003348481932704761</v>
+      </c>
+      <c r="R20" s="38" t="n">
         <v>0.002897956881014574</v>
       </c>
-      <c r="R20" s="38" t="n">
+      <c r="S20" s="38" t="n">
         <v>0.002154345141564873</v>
       </c>
-      <c r="S20" s="38" t="n">
+      <c r="T20" s="38" t="n">
         <v>-0.0001666066684318235</v>
       </c>
-      <c r="T20" s="38" t="n">
+      <c r="U20" s="23" t="n">
         <v>0.002080954496262777</v>
-      </c>
-      <c r="U20" s="23" t="n">
-        <v>0.00376460730477457</v>
       </c>
     </row>
     <row r="21">
@@ -2317,8 +2317,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="51" t="n">
-        <v>46235</v>
+      <c r="N21" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O21" s="45" t="inlineStr">
         <is>
@@ -2331,19 +2331,19 @@
         </is>
       </c>
       <c r="Q21" s="38" t="n">
+        <v>0.02565840844021818</v>
+      </c>
+      <c r="R21" s="38" t="n">
         <v>0.02446163178647254</v>
       </c>
-      <c r="R21" s="38" t="n">
+      <c r="S21" s="38" t="n">
         <v>0.0246651778923092</v>
       </c>
-      <c r="S21" s="38" t="n">
+      <c r="T21" s="38" t="n">
         <v>0.02565785056369746</v>
       </c>
-      <c r="T21" s="38" t="n">
+      <c r="U21" s="23" t="n">
         <v>0.02822942063611032</v>
-      </c>
-      <c r="U21" s="23" t="n">
-        <v>0.02743309430968526</v>
       </c>
     </row>
     <row r="22">
@@ -2506,7 +2506,7 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="52" t="n">
+      <c r="C24" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D24" s="45" t="inlineStr">
@@ -2585,7 +2585,7 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="52" t="n">
+      <c r="C25" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="D25" s="45" t="inlineStr">
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2942,19 +2942,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.32</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.33</v>
-      </c>
-      <c r="S29" s="45" t="n">
-        <v>2.35</v>
       </c>
       <c r="T29" s="45" t="n">
         <v>2.35</v>
       </c>
       <c r="U29" s="21" t="n">
-        <v>2.36</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="30">
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3024,10 +3024,10 @@
         <v>2.33</v>
       </c>
       <c r="R30" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="S30" s="45" t="n">
         <v>2.35</v>
-      </c>
-      <c r="S30" s="45" t="n">
-        <v>2.36</v>
       </c>
       <c r="T30" s="45" t="n">
         <v>2.36</v>
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46303</v>
+        <v>46307</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4367,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.75</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.77</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.79</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.84</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.83</v>
       </c>
     </row>
     <row r="49">
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4442,16 +4442,16 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.99</v>
-      </c>
-      <c r="R49" s="45" t="n">
-        <v>5.03</v>
       </c>
       <c r="S49" s="45" t="n">
         <v>5.03</v>
       </c>
       <c r="T49" s="45" t="n">
-        <v>5.06</v>
+        <v>5.03</v>
       </c>
       <c r="U49" s="21" t="n">
         <v>5.06</v>
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4521,19 +4521,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5.24</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>5.22</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>5.28</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>5.27</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>5.31</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>5.28</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="N52" s="57" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4647,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.69</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.7</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.74</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.73</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.77</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-15
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>3.5862</v>
+        <v>3.6429</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.54</v>
@@ -1726,7 +1726,7 @@
         </is>
       </c>
       <c r="N13" s="52" t="n">
-        <v>46293</v>
+        <v>46300</v>
       </c>
       <c r="O13" s="45" t="inlineStr">
         <is>
@@ -1739,19 +1739,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>197000</v>
+        <v>199000</v>
       </c>
       <c r="R13" s="24" t="n">
+        <v>198000</v>
+      </c>
+      <c r="S13" s="24" t="n">
         <v>199000</v>
-      </c>
-      <c r="S13" s="24" t="n">
-        <v>198000</v>
       </c>
       <c r="T13" s="24" t="n">
         <v>198000</v>
       </c>
       <c r="U13" s="26" t="n">
-        <v>207000</v>
+        <v>198000</v>
       </c>
     </row>
     <row r="14">
@@ -1801,7 +1801,7 @@
         </is>
       </c>
       <c r="N14" s="52" t="n">
-        <v>46286</v>
+        <v>46293</v>
       </c>
       <c r="O14" s="45" t="inlineStr">
         <is>
@@ -1814,19 +1814,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1716000</v>
+        <v>1710000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1714000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1699000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1712000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1717000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1765000</v>
       </c>
     </row>
     <row r="15">
@@ -1966,8 +1966,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="51" t="n">
-        <v>46235</v>
+      <c r="C17" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="D17" s="45" t="inlineStr">
         <is>
@@ -1980,19 +1980,19 @@
         </is>
       </c>
       <c r="F17" s="25" t="n">
-        <v>0.01127425850332675</v>
+        <v>0.007708413925190838</v>
       </c>
       <c r="G17" s="25" t="n">
-        <v>-0.004584539731313231</v>
+        <v>0.01288780200434303</v>
       </c>
       <c r="H17" s="25" t="n">
+        <v>-0.004070143457889142</v>
+      </c>
+      <c r="I17" s="25" t="n">
         <v>0.002027576683551802</v>
       </c>
-      <c r="I17" s="25" t="n">
+      <c r="J17" s="25" t="n">
         <v>0.01035195829379165</v>
-      </c>
-      <c r="J17" s="25" t="n">
-        <v>0.005864943726552774</v>
       </c>
       <c r="K17" s="46" t="n"/>
       <c r="L17" s="29" t="inlineStr">
@@ -2053,8 +2053,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="51" t="n">
-        <v>46235</v>
+      <c r="C18" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="D18" s="45" t="inlineStr">
         <is>
@@ -2067,19 +2067,19 @@
         </is>
       </c>
       <c r="F18" s="25" t="n">
-        <v>0.05361901579222471</v>
+        <v>0.06287627612889972</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>0.04476427794008134</v>
+        <v>0.05556055265010201</v>
       </c>
       <c r="H18" s="25" t="n">
+        <v>0.04530417597525348</v>
+      </c>
+      <c r="I18" s="25" t="n">
         <v>0.0592802540313897</v>
       </c>
-      <c r="I18" s="25" t="n">
+      <c r="J18" s="25" t="n">
         <v>0.06699898466493943</v>
-      </c>
-      <c r="J18" s="25" t="n">
-        <v>0.04091800582057446</v>
       </c>
       <c r="K18" s="46" t="n"/>
       <c r="L18" s="28" t="inlineStr">
@@ -2396,8 +2396,8 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="51" t="n">
-        <v>46235</v>
+      <c r="N22" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O22" s="45" t="inlineStr">
         <is>
@@ -2410,19 +2410,19 @@
         </is>
       </c>
       <c r="Q22" s="38" t="n">
-        <v>0.003999132564547425</v>
+        <v>0.01343380142329798</v>
       </c>
       <c r="R22" s="38" t="n">
-        <v>0.0007468069216873818</v>
+        <v>0.004702913512273366</v>
       </c>
       <c r="S22" s="38" t="n">
-        <v>-0.001255864953080388</v>
+        <v>0.001538137513323212</v>
       </c>
       <c r="T22" s="38" t="n">
-        <v>0.005145423904755253</v>
+        <v>-0.001217537641674205</v>
       </c>
       <c r="U22" s="23" t="n">
-        <v>0.01080359860874536</v>
+        <v>0.00520950141290899</v>
       </c>
     </row>
     <row r="23">
@@ -2466,8 +2466,8 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="51" t="n">
-        <v>46235</v>
+      <c r="N23" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O23" s="45" t="inlineStr">
         <is>
@@ -2480,19 +2480,19 @@
         </is>
       </c>
       <c r="Q23" s="38" t="n">
-        <v>0.05413622452737953</v>
+        <v>0.06346301041631999</v>
       </c>
       <c r="R23" s="38" t="n">
-        <v>0.0480424072675253</v>
+        <v>0.05581709938591151</v>
       </c>
       <c r="S23" s="38" t="n">
-        <v>0.05575734704467192</v>
+        <v>0.04897825491152896</v>
       </c>
       <c r="T23" s="38" t="n">
-        <v>0.05879732438762639</v>
+        <v>0.05586516884219601</v>
       </c>
       <c r="U23" s="23" t="n">
-        <v>0.05693000575666253</v>
+        <v>0.05886482217707373</v>
       </c>
     </row>
     <row r="24">
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2942,16 +2942,16 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.32</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.33</v>
-      </c>
-      <c r="T29" s="45" t="n">
-        <v>2.35</v>
       </c>
       <c r="U29" s="21" t="n">
         <v>2.35</v>
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3021,16 +3021,16 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
-        <v>2.33</v>
+        <v>2.35</v>
       </c>
       <c r="R30" s="45" t="n">
         <v>2.33</v>
       </c>
       <c r="S30" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="T30" s="45" t="n">
         <v>2.35</v>
-      </c>
-      <c r="T30" s="45" t="n">
-        <v>2.36</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.36</v>
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4367,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.79</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.8</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.75</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.77</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.79</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.84</v>
       </c>
     </row>
     <row r="49">
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4442,19 +4442,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>5.02</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.99</v>
-      </c>
-      <c r="S49" s="45" t="n">
-        <v>5.03</v>
       </c>
       <c r="T49" s="45" t="n">
         <v>5.03</v>
       </c>
       <c r="U49" s="21" t="n">
-        <v>5.06</v>
+        <v>5.03</v>
       </c>
     </row>
     <row r="50">
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4521,19 +4521,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5.21</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>5.24</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>5.22</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>5.28</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>5.27</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>5.31</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4583,7 +4583,7 @@
         </is>
       </c>
       <c r="N51" s="52" t="n">
-        <v>46300</v>
+        <v>46307</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
         <is>
@@ -4599,16 +4599,16 @@
         <v>7.4</v>
       </c>
       <c r="R51" s="45" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="S51" s="45" t="n">
         <v>7.28</v>
       </c>
-      <c r="S51" s="45" t="n">
+      <c r="T51" s="45" t="n">
         <v>7.03</v>
       </c>
-      <c r="T51" s="45" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.95</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.76</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="N52" s="57" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4647,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.63</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.67</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.69</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.7</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.74</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.73</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-16
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2942,19 +2942,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.34</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.32</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.33</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.35</v>
       </c>
     </row>
     <row r="30">
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3021,19 +3021,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.35</v>
-      </c>
-      <c r="R30" s="45" t="n">
-        <v>2.33</v>
       </c>
       <c r="S30" s="45" t="n">
         <v>2.33</v>
       </c>
       <c r="T30" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="U30" s="21" t="n">
         <v>2.35</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.36</v>
       </c>
     </row>
     <row r="31">
@@ -3122,8 +3122,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="51" t="n">
-        <v>46235</v>
+      <c r="C32" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="D32" s="45" t="inlineStr">
         <is>
@@ -3136,19 +3136,19 @@
         </is>
       </c>
       <c r="F32" s="25" t="n">
-        <v>0.0002212616963008784</v>
+        <v>0.00662558198988239</v>
       </c>
       <c r="G32" s="25" t="n">
-        <v>0.001977791174811783</v>
+        <v>0.0006375931922877331</v>
       </c>
       <c r="H32" s="25" t="n">
-        <v>0.001971948448746819</v>
+        <v>0.002327094725187218</v>
       </c>
       <c r="I32" s="25" t="n">
-        <v>0.0005975922782888166</v>
+        <v>0.002314959035544017</v>
       </c>
       <c r="J32" s="25" t="n">
-        <v>0.008303058183333656</v>
+        <v>0.001427223309754311</v>
       </c>
       <c r="K32" s="46" t="n"/>
       <c r="L32" s="28" t="n"/>
@@ -3193,8 +3193,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="51" t="n">
-        <v>46235</v>
+      <c r="C33" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="D33" s="45" t="inlineStr">
         <is>
@@ -3207,19 +3207,19 @@
         </is>
       </c>
       <c r="F33" s="25" t="n">
-        <v>0.0142042239731089</v>
+        <v>0.02245150883267093</v>
       </c>
       <c r="G33" s="25" t="n">
-        <v>0.01129997840893473</v>
+        <v>0.01615453723356625</v>
       </c>
       <c r="H33" s="25" t="n">
-        <v>0.01343634365900168</v>
+        <v>0.01282312991932782</v>
       </c>
       <c r="I33" s="25" t="n">
-        <v>0.01658091130138508</v>
+        <v>0.01460900584852951</v>
       </c>
       <c r="J33" s="25" t="n">
-        <v>0.01434223394335294</v>
+        <v>0.0174089169072604</v>
       </c>
       <c r="K33" s="46" t="n"/>
       <c r="L33" s="28" t="inlineStr">
@@ -3272,8 +3272,8 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="51" t="n">
-        <v>46235</v>
+      <c r="C34" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="D34" s="45" t="inlineStr">
         <is>
@@ -3286,19 +3286,19 @@
         </is>
       </c>
       <c r="F34" s="24" t="n">
-        <v>76.2717</v>
+        <v>76.85039999999999</v>
       </c>
       <c r="G34" s="24" t="n">
-        <v>76.3259</v>
+        <v>76.41840000000001</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>76.24379999999999</v>
+        <v>76.4409</v>
       </c>
       <c r="I34" s="24" t="n">
-        <v>76.1605</v>
+        <v>76.3321</v>
       </c>
       <c r="J34" s="24" t="n">
-        <v>76.1803</v>
+        <v>76.2225</v>
       </c>
       <c r="K34" s="46" t="n"/>
       <c r="L34" s="28" t="n"/>
@@ -3836,8 +3836,8 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="51" t="n">
-        <v>46235</v>
+      <c r="N41" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O41" s="45" t="inlineStr">
         <is>
@@ -3850,19 +3850,19 @@
         </is>
       </c>
       <c r="Q41" s="38" t="n">
-        <v>0.006053268765133124</v>
+        <v>0.02153110047846907</v>
       </c>
       <c r="R41" s="38" t="n">
-        <v>-0.01431980906921249</v>
+        <v>0.01210653753026625</v>
       </c>
       <c r="S41" s="38" t="n">
-        <v>-0.007109004739336622</v>
+        <v>-0.01373134328358216</v>
       </c>
       <c r="T41" s="38" t="n">
+        <v>-0.007701421800947905</v>
+      </c>
+      <c r="U41" s="23" t="n">
         <v>0.01199040767386084</v>
-      </c>
-      <c r="U41" s="23" t="n">
-        <v>0.03538175046554937</v>
       </c>
     </row>
     <row r="42">
@@ -3911,8 +3911,8 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="51" t="n">
-        <v>46235</v>
+      <c r="N42" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O42" s="45" t="inlineStr">
         <is>
@@ -3925,19 +3925,19 @@
         </is>
       </c>
       <c r="Q42" s="38" t="n">
-        <v>0.0862745098039215</v>
+        <v>0.1163398692810458</v>
       </c>
       <c r="R42" s="38" t="n">
+        <v>0.09281045751633979</v>
+      </c>
+      <c r="S42" s="38" t="n">
         <v>0.08115183246073283</v>
       </c>
-      <c r="S42" s="38" t="n">
-        <v>0.1004596191726854</v>
-      </c>
       <c r="T42" s="38" t="n">
+        <v>0.09980302035456327</v>
+      </c>
+      <c r="U42" s="23" t="n">
         <v>0.1134564643799473</v>
-      </c>
-      <c r="U42" s="23" t="n">
-        <v>0.09305373525557023</v>
       </c>
     </row>
     <row r="43">
@@ -3986,8 +3986,8 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="51" t="n">
-        <v>46235</v>
+      <c r="N43" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O43" s="45" t="inlineStr">
         <is>
@@ -4000,19 +4000,19 @@
         </is>
       </c>
       <c r="Q43" s="38" t="n">
-        <v>0.006675567423231055</v>
+        <v>0.01129568106312284</v>
       </c>
       <c r="R43" s="38" t="n">
-        <v>-0.003326679973386537</v>
+        <v>0.005344021376085584</v>
       </c>
       <c r="S43" s="38" t="n">
+        <v>-0.003992015968063978</v>
+      </c>
+      <c r="T43" s="38" t="n">
         <v>-0.002654280026542666</v>
       </c>
-      <c r="T43" s="38" t="n">
+      <c r="U43" s="23" t="n">
         <v>0.0175557056043214</v>
-      </c>
-      <c r="U43" s="23" t="n">
-        <v>0.02279005524861866</v>
       </c>
     </row>
     <row r="44">
@@ -4061,8 +4061,8 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="51" t="n">
-        <v>46235</v>
+      <c r="N44" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O44" s="45" t="inlineStr">
         <is>
@@ -4075,19 +4075,19 @@
         </is>
       </c>
       <c r="Q44" s="38" t="n">
-        <v>0.06950354609929087</v>
+        <v>0.08096590909090892</v>
       </c>
       <c r="R44" s="38" t="n">
-        <v>0.06090651558073671</v>
+        <v>0.0673758865248227</v>
       </c>
       <c r="S44" s="38" t="n">
+        <v>0.06019830028328613</v>
+      </c>
+      <c r="T44" s="38" t="n">
         <v>0.0674715909090909</v>
       </c>
-      <c r="T44" s="38" t="n">
+      <c r="U44" s="23" t="n">
         <v>0.06879432624113467</v>
-      </c>
-      <c r="U44" s="23" t="n">
-        <v>0.04516584333098099</v>
       </c>
     </row>
     <row r="45">
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4367,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.79</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.8</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.75</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.77</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.79</v>
       </c>
     </row>
     <row r="49">
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4445,13 +4445,13 @@
         <v>5</v>
       </c>
       <c r="R49" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="S49" s="45" t="n">
         <v>5.02</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.99</v>
-      </c>
-      <c r="T49" s="45" t="n">
-        <v>5.03</v>
       </c>
       <c r="U49" s="21" t="n">
         <v>5.03</v>
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4521,19 +4521,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5.19</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>5.21</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>5.24</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>5.22</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>5.28</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>5.27</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="N52" s="57" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4647,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.54</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.63</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.67</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.69</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.7</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.74</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-17
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2942,19 +2942,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.31</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.34</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.32</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.33</v>
       </c>
     </row>
     <row r="30">
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3021,19 +3021,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.32</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.35</v>
-      </c>
-      <c r="S30" s="45" t="n">
-        <v>2.33</v>
       </c>
       <c r="T30" s="45" t="n">
         <v>2.33</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.35</v>
+        <v>2.33</v>
       </c>
     </row>
     <row r="31">
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4367,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.77</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.82</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.79</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.8</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.75</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.77</v>
       </c>
     </row>
     <row r="49">
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4442,19 +4442,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
-        <v>5</v>
+        <v>4.91</v>
       </c>
       <c r="R49" s="45" t="n">
         <v>5</v>
       </c>
       <c r="S49" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="T49" s="45" t="n">
         <v>5.02</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.99</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>5.03</v>
       </c>
     </row>
     <row r="50">
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4521,19 +4521,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>5.19</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>5.21</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>5.24</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>5.22</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>5.28</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-19
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="N52" s="57" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4647,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.54</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.63</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.67</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.69</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.7</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-20
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>3.6429</v>
+        <v>3.4989</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.54</v>
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2942,19 +2942,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.31</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.34</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.33</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.32</v>
       </c>
     </row>
     <row r="30">
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3024,13 +3024,13 @@
         <v>2.35</v>
       </c>
       <c r="R30" s="45" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="S30" s="45" t="n">
         <v>2.32</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.35</v>
-      </c>
-      <c r="T30" s="45" t="n">
-        <v>2.33</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.33</v>
@@ -3426,8 +3426,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="51" t="n">
-        <v>46235</v>
+      <c r="C36" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="D36" s="45" t="inlineStr">
         <is>
@@ -3440,19 +3440,19 @@
         </is>
       </c>
       <c r="F36" s="24" t="n">
-        <v>1275</v>
+        <v>1221</v>
       </c>
       <c r="G36" s="24" t="n">
-        <v>1309</v>
+        <v>1288</v>
       </c>
       <c r="H36" s="24" t="n">
+        <v>1369</v>
+      </c>
+      <c r="I36" s="24" t="n">
         <v>1439</v>
       </c>
-      <c r="I36" s="24" t="n">
+      <c r="J36" s="24" t="n">
         <v>1182</v>
-      </c>
-      <c r="J36" s="24" t="n">
-        <v>1414</v>
       </c>
       <c r="K36" s="46" t="n"/>
       <c r="L36" s="28" t="n"/>
@@ -3497,8 +3497,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="51" t="n">
-        <v>46235</v>
+      <c r="C37" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="D37" s="45" t="inlineStr">
         <is>
@@ -3511,19 +3511,19 @@
         </is>
       </c>
       <c r="F37" s="25" t="n">
-        <v>-0.01239349341595662</v>
+        <v>-0.07429871114480667</v>
       </c>
       <c r="G37" s="25" t="n">
-        <v>-0.08589385474860335</v>
+        <v>-0.002323780015491867</v>
       </c>
       <c r="H37" s="25" t="n">
+        <v>-0.04399441340782123</v>
+      </c>
+      <c r="I37" s="25" t="n">
         <v>0.04350978970268311</v>
       </c>
-      <c r="I37" s="25" t="n">
+      <c r="J37" s="25" t="n">
         <v>-0.08301008533747091</v>
-      </c>
-      <c r="J37" s="25" t="n">
-        <v>0.01</v>
       </c>
       <c r="K37" s="46" t="n"/>
       <c r="L37" s="28" t="inlineStr">
@@ -3576,8 +3576,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="51" t="n">
-        <v>46235</v>
+      <c r="C38" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="D38" s="45" t="inlineStr">
         <is>
@@ -3590,19 +3590,19 @@
         </is>
       </c>
       <c r="F38" s="24" t="n">
+        <v>1400</v>
+      </c>
+      <c r="G38" s="24" t="n">
         <v>1403</v>
       </c>
-      <c r="G38" s="24" t="n">
+      <c r="H38" s="24" t="n">
         <v>1433</v>
       </c>
-      <c r="H38" s="24" t="n">
+      <c r="I38" s="24" t="n">
         <v>1374</v>
       </c>
-      <c r="I38" s="24" t="n">
+      <c r="J38" s="24" t="n">
         <v>1410</v>
-      </c>
-      <c r="J38" s="24" t="n">
-        <v>1423</v>
       </c>
       <c r="K38" s="46" t="n"/>
       <c r="L38" s="28" t="n"/>
@@ -3647,8 +3647,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="51" t="n">
-        <v>46235</v>
+      <c r="C39" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="D39" s="45" t="inlineStr">
         <is>
@@ -3661,19 +3661,19 @@
         </is>
       </c>
       <c r="F39" s="38" t="n">
+        <v>-0.03047091412742382</v>
+      </c>
+      <c r="G39" s="38" t="n">
         <v>0.04157386785449146</v>
       </c>
-      <c r="G39" s="38" t="n">
+      <c r="H39" s="38" t="n">
         <v>0.02357142857142857</v>
       </c>
-      <c r="H39" s="38" t="n">
+      <c r="I39" s="38" t="n">
         <v>-0.0178699070764832</v>
       </c>
-      <c r="I39" s="38" t="n">
+      <c r="J39" s="38" t="n">
         <v>-0.00423728813559322</v>
-      </c>
-      <c r="J39" s="38" t="n">
-        <v>-0.01522491349480969</v>
       </c>
       <c r="K39" s="46" t="n"/>
       <c r="L39" s="28" t="inlineStr">
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4367,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.77</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.82</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.79</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.8</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.75</v>
       </c>
     </row>
     <row r="49">
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4442,19 +4442,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.89</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.91</v>
-      </c>
-      <c r="R49" s="45" t="n">
-        <v>5</v>
       </c>
       <c r="S49" s="45" t="n">
         <v>5</v>
       </c>
       <c r="T49" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="U49" s="21" t="n">
         <v>5.02</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.99</v>
       </c>
     </row>
     <row r="50">
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4521,19 +4521,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>5.1</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>5.19</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>5.21</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>5.24</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>5.22</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="N52" s="57" t="n">
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4647,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.61</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.55</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.54</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.63</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.67</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.69</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-22
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1726,7 +1726,7 @@
         </is>
       </c>
       <c r="N13" s="52" t="n">
-        <v>46300</v>
+        <v>46307</v>
       </c>
       <c r="O13" s="45" t="inlineStr">
         <is>
@@ -1739,16 +1739,16 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
+        <v>194000</v>
+      </c>
+      <c r="R13" s="24" t="n">
+        <v>200000</v>
+      </c>
+      <c r="S13" s="24" t="n">
+        <v>198000</v>
+      </c>
+      <c r="T13" s="24" t="n">
         <v>199000</v>
-      </c>
-      <c r="R13" s="24" t="n">
-        <v>198000</v>
-      </c>
-      <c r="S13" s="24" t="n">
-        <v>199000</v>
-      </c>
-      <c r="T13" s="24" t="n">
-        <v>198000</v>
       </c>
       <c r="U13" s="26" t="n">
         <v>198000</v>
@@ -1801,7 +1801,7 @@
         </is>
       </c>
       <c r="N14" s="52" t="n">
-        <v>46293</v>
+        <v>46300</v>
       </c>
       <c r="O14" s="45" t="inlineStr">
         <is>
@@ -1814,19 +1814,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1710000</v>
+        <v>1728000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1703000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1714000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1699000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1712000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1717000</v>
       </c>
     </row>
     <row r="15">
@@ -1966,7 +1966,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="52" t="n">
+      <c r="C17" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="D17" s="45" t="inlineStr">
@@ -2053,7 +2053,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="52" t="n">
+      <c r="C18" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="D18" s="45" t="inlineStr">
@@ -2092,7 +2092,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="52" t="n">
+      <c r="N18" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="O18" s="45" t="inlineStr">
@@ -2167,7 +2167,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="52" t="n">
+      <c r="N19" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="O19" s="45" t="inlineStr">
@@ -2242,7 +2242,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="52" t="n">
+      <c r="N20" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="O20" s="45" t="inlineStr">
@@ -2317,7 +2317,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="52" t="n">
+      <c r="N21" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="O21" s="45" t="inlineStr">
@@ -2396,7 +2396,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="52" t="n">
+      <c r="N22" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="O22" s="45" t="inlineStr">
@@ -2466,7 +2466,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="52" t="n">
+      <c r="N23" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="O23" s="45" t="inlineStr">
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2942,19 +2942,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="R29" s="45" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="S29" s="45" t="n">
         <v>2.32</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.31</v>
-      </c>
-      <c r="T29" s="45" t="n">
-        <v>2.34</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.33</v>
       </c>
     </row>
     <row r="30">
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3021,19 +3021,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
-        <v>2.35</v>
+        <v>2.37</v>
       </c>
       <c r="R30" s="45" t="n">
         <v>2.35</v>
       </c>
       <c r="S30" s="45" t="n">
-        <v>2.32</v>
+        <v>2.35</v>
       </c>
       <c r="T30" s="45" t="n">
         <v>2.35</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.33</v>
+        <v>2.32</v>
       </c>
     </row>
     <row r="31">
@@ -3324,16 +3324,16 @@
         <v>-0.002958631913215778</v>
       </c>
       <c r="R34" s="38" t="n">
-        <v>-0.001484371505816431</v>
+        <v>-0.001484371505816307</v>
       </c>
       <c r="S34" s="38" t="n">
-        <v>-0.0006782988032907144</v>
+        <v>-0.0006782988032908383</v>
       </c>
       <c r="T34" s="38" t="n">
         <v>-0.004701862813512956</v>
       </c>
       <c r="U34" s="23" t="n">
-        <v>-2.432480890000966e-05</v>
+        <v>-2.432480889988557e-05</v>
       </c>
     </row>
     <row r="35" ht="31.5" customHeight="1">
@@ -3403,10 +3403,10 @@
         <v>8.50375855385721e-05</v>
       </c>
       <c r="R35" s="38" t="n">
-        <v>0.0008263155649319565</v>
+        <v>0.0008263155649324005</v>
       </c>
       <c r="S35" s="38" t="n">
-        <v>0.00369982572748162</v>
+        <v>0.003699825727481398</v>
       </c>
       <c r="T35" s="38" t="n">
         <v>-0.002206341131705591</v>
@@ -3478,16 +3478,16 @@
         <v>-0.002958631913215778</v>
       </c>
       <c r="R36" s="38" t="n">
-        <v>-0.001484371505816431</v>
+        <v>-0.001484371505816307</v>
       </c>
       <c r="S36" s="38" t="n">
-        <v>-0.0006782988032907144</v>
+        <v>-0.0006782988032908383</v>
       </c>
       <c r="T36" s="38" t="n">
         <v>-0.004701862813512956</v>
       </c>
       <c r="U36" s="23" t="n">
-        <v>-2.432480890000966e-05</v>
+        <v>-2.432480889988557e-05</v>
       </c>
     </row>
     <row r="37">
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46311</v>
+        <v>46315</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46311</v>
+        <v>46315</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4367,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
-        <v>4.74</v>
+        <v>4.79</v>
       </c>
       <c r="R48" s="45" t="n">
         <v>4.77</v>
       </c>
       <c r="S48" s="45" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="T48" s="45" t="n">
+        <v>4.77</v>
+      </c>
+      <c r="U48" s="21" t="n">
         <v>4.82</v>
-      </c>
-      <c r="T48" s="45" t="n">
-        <v>4.79</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.8</v>
       </c>
     </row>
     <row r="49">
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46311</v>
+        <v>46315</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4442,19 +4442,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.94</v>
+      </c>
+      <c r="R49" s="45" t="n">
+        <v>4.94</v>
+      </c>
+      <c r="S49" s="45" t="n">
         <v>4.89</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.91</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>5</v>
-      </c>
-      <c r="T49" s="45" t="n">
-        <v>5</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>5.02</v>
       </c>
     </row>
     <row r="50">
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46311</v>
+        <v>46315</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4521,19 +4521,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="R50" s="45" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="S50" s="45" t="n">
         <v>5.09</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>5.1</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>5.19</v>
-      </c>
-      <c r="T50" s="45" t="n">
-        <v>5.21</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>5.24</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4583,7 +4583,7 @@
         </is>
       </c>
       <c r="N51" s="52" t="n">
-        <v>46307</v>
+        <v>46314</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
         <is>
@@ -4596,19 +4596,19 @@
         </is>
       </c>
       <c r="Q51" s="45" t="n">
-        <v>7.4</v>
+        <v>7.32</v>
       </c>
       <c r="R51" s="45" t="n">
         <v>7.4</v>
       </c>
       <c r="S51" s="45" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="T51" s="45" t="n">
         <v>7.28</v>
       </c>
-      <c r="T51" s="45" t="n">
+      <c r="U51" s="21" t="n">
         <v>7.03</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.95</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="N52" s="57" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4647,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="R52" s="9" t="n">
+        <v>6.56</v>
+      </c>
+      <c r="S52" s="9" t="n">
         <v>6.61</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.55</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.54</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>6.63</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.67</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-23
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2854,7 +2854,7 @@
         </is>
       </c>
       <c r="N28" s="51" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="O28" s="45" t="inlineStr">
         <is>
@@ -2867,19 +2867,19 @@
         </is>
       </c>
       <c r="Q28" s="45" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="R28" s="45" t="n">
         <v>4</v>
       </c>
-      <c r="R28" s="45" t="n">
+      <c r="S28" s="45" t="n">
         <v>4.2</v>
       </c>
-      <c r="S28" s="45" t="n">
+      <c r="T28" s="45" t="n">
         <v>4.6</v>
       </c>
-      <c r="T28" s="45" t="n">
+      <c r="U28" s="21" t="n">
         <v>4.8</v>
-      </c>
-      <c r="U28" s="21" t="n">
-        <v>4.7</v>
       </c>
     </row>
     <row r="29">
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2942,19 +2942,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.34</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.31</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.32</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.33</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.31</v>
       </c>
     </row>
     <row r="30">
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3021,10 +3021,10 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.37</v>
-      </c>
-      <c r="R30" s="45" t="n">
-        <v>2.35</v>
       </c>
       <c r="S30" s="45" t="n">
         <v>2.35</v>
@@ -3033,7 +3033,7 @@
         <v>2.35</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.32</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="31">
@@ -3122,7 +3122,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="52" t="n">
+      <c r="C32" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="D32" s="45" t="inlineStr">
@@ -3193,7 +3193,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="52" t="n">
+      <c r="C33" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="D33" s="45" t="inlineStr">
@@ -3272,7 +3272,7 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="52" t="n">
+      <c r="C34" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="D34" s="45" t="inlineStr">
@@ -3836,7 +3836,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="52" t="n">
+      <c r="N41" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="O41" s="45" t="inlineStr">
@@ -3911,7 +3911,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="52" t="n">
+      <c r="N42" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="O42" s="45" t="inlineStr">
@@ -3986,7 +3986,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="52" t="n">
+      <c r="N43" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="O43" s="45" t="inlineStr">
@@ -4061,7 +4061,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="52" t="n">
+      <c r="N44" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="O44" s="45" t="inlineStr">
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4367,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.81</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.79</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.77</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.74</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.77</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.82</v>
       </c>
     </row>
     <row r="49">
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4442,19 +4442,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
-        <v>4.94</v>
+        <v>4.95</v>
       </c>
       <c r="R49" s="45" t="n">
         <v>4.94</v>
       </c>
       <c r="S49" s="45" t="n">
+        <v>4.94</v>
+      </c>
+      <c r="T49" s="45" t="n">
         <v>4.89</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.91</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="50">
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4521,19 +4521,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>5.12</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>5.15</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>5.09</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>5.1</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>5.19</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="N52" s="57" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4647,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.42</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.57</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.56</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.61</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.55</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.54</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-24
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2942,19 +2942,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.19</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.34</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.31</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.32</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.33</v>
       </c>
     </row>
     <row r="30">
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3021,13 +3021,13 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.32</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.37</v>
-      </c>
-      <c r="S30" s="45" t="n">
-        <v>2.35</v>
       </c>
       <c r="T30" s="45" t="n">
         <v>2.35</v>
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4367,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.81</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.79</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.77</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.74</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.77</v>
       </c>
     </row>
     <row r="49">
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4442,19 +4442,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.95</v>
-      </c>
-      <c r="R49" s="45" t="n">
-        <v>4.94</v>
       </c>
       <c r="S49" s="45" t="n">
         <v>4.94</v>
       </c>
       <c r="T49" s="45" t="n">
+        <v>4.94</v>
+      </c>
+      <c r="U49" s="21" t="n">
         <v>4.89</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.91</v>
       </c>
     </row>
     <row r="50">
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4521,19 +4521,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.96</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>5.13</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>5.12</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>5.15</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>5.09</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>5.1</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-26
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="N52" s="57" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4647,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.47</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.42</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.57</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.56</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.61</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.55</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-27
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>3.4989</v>
+        <v>3.4119</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.54</v>
@@ -2814,8 +2814,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="51" t="n">
-        <v>46235</v>
+      <c r="C28" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="D28" s="45" t="inlineStr">
         <is>
@@ -2828,19 +2828,19 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>-0.0007144966046649381</v>
+        <v>0.01844201263870571</v>
       </c>
       <c r="G28" s="25" t="n">
+        <v>0.00123117803365802</v>
+      </c>
+      <c r="H28" s="25" t="n">
         <v>0.008699174159193968</v>
       </c>
-      <c r="H28" s="25" t="n">
+      <c r="I28" s="25" t="n">
         <v>0.005802145925317914</v>
       </c>
-      <c r="I28" s="25" t="n">
+      <c r="J28" s="25" t="n">
         <v>-0.04004117699494203</v>
-      </c>
-      <c r="J28" s="25" t="n">
-        <v>0.08512722904348102</v>
       </c>
       <c r="K28" s="46" t="n"/>
       <c r="L28" s="28" t="inlineStr">
@@ -2889,8 +2889,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="51" t="n">
-        <v>46235</v>
+      <c r="C29" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="D29" s="45" t="inlineStr">
         <is>
@@ -2903,19 +2903,19 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>0.08432167823206402</v>
+        <v>0.09939295934705727</v>
       </c>
       <c r="G29" s="25" t="n">
+        <v>0.08643292389904465</v>
+      </c>
+      <c r="H29" s="25" t="n">
         <v>0.1177037408590512</v>
       </c>
-      <c r="H29" s="25" t="n">
+      <c r="I29" s="25" t="n">
         <v>0.07703978368044752</v>
       </c>
-      <c r="I29" s="25" t="n">
+      <c r="J29" s="25" t="n">
         <v>-0.02972368914374733</v>
-      </c>
-      <c r="J29" s="25" t="n">
-        <v>0.1779567725392831</v>
       </c>
       <c r="K29" s="46" t="n"/>
       <c r="L29" s="28" t="inlineStr">
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2942,19 +2942,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.2</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.19</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.34</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.31</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.32</v>
       </c>
     </row>
     <row r="30">
@@ -2968,8 +2968,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="51" t="n">
-        <v>46235</v>
+      <c r="C30" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="D30" s="45" t="inlineStr">
         <is>
@@ -2982,19 +2982,19 @@
         </is>
       </c>
       <c r="F30" s="25" t="n">
-        <v>-7.980998837964215e-05</v>
+        <v>0.02188394127363513</v>
       </c>
       <c r="G30" s="25" t="n">
+        <v>0.003061511154244023</v>
+      </c>
+      <c r="H30" s="25" t="n">
         <v>0.01426966328516333</v>
       </c>
-      <c r="H30" s="25" t="n">
+      <c r="I30" s="25" t="n">
         <v>0.003538609511678281</v>
       </c>
-      <c r="I30" s="25" t="n">
+      <c r="J30" s="25" t="n">
         <v>-0.04261964610139124</v>
-      </c>
-      <c r="J30" s="25" t="n">
-        <v>0.08475262626842106</v>
       </c>
       <c r="K30" s="46" t="n"/>
       <c r="L30" s="28" t="inlineStr">
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3024,13 +3024,13 @@
         <v>2.34</v>
       </c>
       <c r="R30" s="45" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="S30" s="45" t="n">
         <v>2.32</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.37</v>
-      </c>
-      <c r="T30" s="45" t="n">
-        <v>2.35</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.35</v>
@@ -3043,8 +3043,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="51" t="n">
-        <v>46235</v>
+      <c r="C31" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="D31" s="45" t="inlineStr">
         <is>
@@ -3057,19 +3057,19 @@
         </is>
       </c>
       <c r="F31" s="25" t="n">
-        <v>0.07841442756607125</v>
+        <v>0.1041800643086817</v>
       </c>
       <c r="G31" s="25" t="n">
+        <v>0.08180234399746594</v>
+      </c>
+      <c r="H31" s="25" t="n">
         <v>0.09907475956730888</v>
       </c>
-      <c r="H31" s="25" t="n">
+      <c r="I31" s="25" t="n">
         <v>0.05755592766471823</v>
       </c>
-      <c r="I31" s="25" t="n">
+      <c r="J31" s="25" t="n">
         <v>-0.04567753459150702</v>
-      </c>
-      <c r="J31" s="25" t="n">
-        <v>0.1533794281326583</v>
       </c>
       <c r="K31" s="46" t="n"/>
       <c r="L31" s="28" t="inlineStr">
@@ -3426,7 +3426,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="52" t="n">
+      <c r="C36" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="D36" s="45" t="inlineStr">
@@ -3497,7 +3497,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="52" t="n">
+      <c r="C37" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="D37" s="45" t="inlineStr">
@@ -3576,7 +3576,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="52" t="n">
+      <c r="C38" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="D38" s="45" t="inlineStr">
@@ -3590,7 +3590,7 @@
         </is>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1400</v>
+        <v>1398</v>
       </c>
       <c r="G38" s="24" t="n">
         <v>1403</v>
@@ -3647,7 +3647,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="52" t="n">
+      <c r="C39" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="D39" s="45" t="inlineStr">
@@ -3661,7 +3661,7 @@
         </is>
       </c>
       <c r="F39" s="38" t="n">
-        <v>-0.03047091412742382</v>
+        <v>-0.03185595567867036</v>
       </c>
       <c r="G39" s="38" t="n">
         <v>0.04157386785449146</v>
@@ -3726,8 +3726,8 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="51" t="n">
-        <v>46235</v>
+      <c r="C40" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="D40" s="45" t="inlineStr">
         <is>
@@ -3740,19 +3740,19 @@
         </is>
       </c>
       <c r="F40" s="24" t="n">
-        <v>684</v>
+        <v>676</v>
       </c>
       <c r="G40" s="24" t="n">
-        <v>643</v>
+        <v>680</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>672</v>
+        <v>647</v>
       </c>
       <c r="I40" s="24" t="n">
+        <v>680</v>
+      </c>
+      <c r="J40" s="24" t="n">
         <v>636</v>
-      </c>
-      <c r="J40" s="24" t="n">
-        <v>641</v>
       </c>
       <c r="K40" s="46" t="n"/>
       <c r="L40" s="28" t="n"/>
@@ -3797,8 +3797,8 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="51" t="n">
-        <v>46235</v>
+      <c r="C41" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="D41" s="45" t="inlineStr">
         <is>
@@ -3811,19 +3811,19 @@
         </is>
       </c>
       <c r="F41" s="38" t="n">
-        <v>-0.02005730659025788</v>
+        <v>-0.05322128851540616</v>
       </c>
       <c r="G41" s="38" t="n">
-        <v>-0.007716049382716049</v>
+        <v>-0.02578796561604585</v>
       </c>
       <c r="H41" s="38" t="n">
-        <v>0.01052631578947368</v>
+        <v>-0.00154320987654321</v>
       </c>
       <c r="I41" s="38" t="n">
+        <v>0.02255639097744361</v>
+      </c>
+      <c r="J41" s="38" t="n">
         <v>0.022508038585209</v>
-      </c>
-      <c r="J41" s="38" t="n">
-        <v>-0.08559201141226819</v>
       </c>
       <c r="K41" s="46" t="n"/>
       <c r="L41" s="28" t="inlineStr">
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4367,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.69</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.65</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.81</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.79</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.77</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.74</v>
       </c>
     </row>
     <row r="49">
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4442,19 +4442,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.78</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.95</v>
-      </c>
-      <c r="S49" s="45" t="n">
-        <v>4.94</v>
       </c>
       <c r="T49" s="45" t="n">
         <v>4.94</v>
       </c>
       <c r="U49" s="21" t="n">
-        <v>4.89</v>
+        <v>4.94</v>
       </c>
     </row>
     <row r="50">
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4521,19 +4521,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.96</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>5.13</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>5.12</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>5.15</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>5.09</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="N52" s="57" t="n">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4647,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.45</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.47</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.42</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.57</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.56</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.61</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-28
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>3.4119</v>
+        <v>3.2721</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.54</v>
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2942,19 +2942,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.2</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.19</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.34</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.31</v>
       </c>
     </row>
     <row r="30">
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3021,19 +3021,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
-        <v>2.34</v>
+        <v>2.35</v>
       </c>
       <c r="R30" s="45" t="n">
         <v>2.34</v>
       </c>
       <c r="S30" s="45" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="T30" s="45" t="n">
         <v>2.32</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.37</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.35</v>
       </c>
     </row>
     <row r="31">
@@ -3536,8 +3536,8 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="51" t="n">
-        <v>46204</v>
+      <c r="N37" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O37" s="45" t="inlineStr">
         <is>
@@ -3550,19 +3550,19 @@
         </is>
       </c>
       <c r="Q37" s="38" t="n">
-        <v>0.00118133140204435</v>
+        <v>-0.001544793068890105</v>
       </c>
       <c r="R37" s="38" t="n">
-        <v>0.003945360923047536</v>
+        <v>0.001021019951442215</v>
       </c>
       <c r="S37" s="38" t="n">
-        <v>0.007306018310070606</v>
+        <v>0.003915328780348393</v>
       </c>
       <c r="T37" s="38" t="n">
-        <v>0.008298830536790813</v>
+        <v>0.007284416391287296</v>
       </c>
       <c r="U37" s="23" t="n">
-        <v>0.007882278295670897</v>
+        <v>0.008298152435425976</v>
       </c>
     </row>
     <row r="38">
@@ -3611,8 +3611,8 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="51" t="n">
-        <v>46204</v>
+      <c r="N38" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O38" s="45" t="inlineStr">
         <is>
@@ -3625,19 +3625,19 @@
         </is>
       </c>
       <c r="Q38" s="38" t="n">
-        <v>0.01928847496245344</v>
+        <v>0.02090988467275437</v>
       </c>
       <c r="R38" s="38" t="n">
-        <v>0.01611755196583463</v>
+        <v>0.01915243379144463</v>
       </c>
       <c r="S38" s="38" t="n">
-        <v>0.0127260710933798</v>
+        <v>0.01614464735421413</v>
       </c>
       <c r="T38" s="38" t="n">
-        <v>0.01001067158206193</v>
+        <v>0.01278031439271615</v>
       </c>
       <c r="U38" s="23" t="n">
-        <v>0.008275963087739823</v>
+        <v>0.01008946517952163</v>
       </c>
     </row>
     <row r="39" ht="31.5" customHeight="1">
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4367,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.68</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.69</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.65</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.81</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.79</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.77</v>
       </c>
     </row>
     <row r="49">
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4442,16 +4442,16 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.82</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.78</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.95</v>
-      </c>
-      <c r="T49" s="45" t="n">
-        <v>4.94</v>
       </c>
       <c r="U49" s="21" t="n">
         <v>4.94</v>
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4524,16 +4524,16 @@
         <v>5</v>
       </c>
       <c r="R50" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="S50" s="45" t="n">
         <v>4.96</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>5.13</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>5.12</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>5.15</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-29
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -369,10 +369,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -917,7 +917,7 @@
         </is>
       </c>
       <c r="C3" s="51" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="D3" s="45" t="inlineStr">
         <is>
@@ -930,19 +930,19 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
+        <v>24611.077</v>
+      </c>
+      <c r="G3" s="24" t="n">
         <v>24408.011</v>
       </c>
-      <c r="G3" s="24" t="n">
+      <c r="H3" s="24" t="n">
         <v>24274.383</v>
       </c>
-      <c r="H3" s="24" t="n">
+      <c r="I3" s="24" t="n">
         <v>24125.479</v>
       </c>
-      <c r="I3" s="24" t="n">
+      <c r="J3" s="24" t="n">
         <v>24112.966</v>
-      </c>
-      <c r="J3" s="24" t="n">
-        <v>23884.563</v>
       </c>
       <c r="K3" s="46" t="n"/>
       <c r="L3" s="28" t="inlineStr">
@@ -955,7 +955,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="51" t="n">
+      <c r="N3" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O3" s="45" t="inlineStr">
@@ -992,7 +992,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="D4" s="45" t="inlineStr">
         <is>
@@ -1005,19 +1005,19 @@
         </is>
       </c>
       <c r="F4" s="25" t="n">
+        <v>0.008319645545882492</v>
+      </c>
+      <c r="G4" s="25" t="n">
         <v>0.005504897899979433</v>
       </c>
-      <c r="G4" s="25" t="n">
+      <c r="H4" s="25" t="n">
         <v>0.006172063982646803</v>
       </c>
-      <c r="H4" s="25" t="n">
+      <c r="I4" s="25" t="n">
         <v>0.0005189324283043639</v>
       </c>
-      <c r="I4" s="25" t="n">
+      <c r="J4" s="25" t="n">
         <v>0.009562787479092671</v>
-      </c>
-      <c r="J4" s="25" t="n">
-        <v>0.009909001665228123</v>
       </c>
       <c r="K4" s="46" t="n"/>
       <c r="L4" s="28" t="n"/>
@@ -1026,7 +1026,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="51" t="n">
+      <c r="N4" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O4" s="45" t="inlineStr">
@@ -1066,7 +1066,7 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C5" s="51" t="n">
+      <c r="C5" s="52" t="n">
         <v>46113</v>
       </c>
       <c r="D5" s="45" t="inlineStr">
@@ -1105,7 +1105,7 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="51" t="n">
+      <c r="N5" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O5" s="45" t="inlineStr">
@@ -1141,7 +1141,7 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C6" s="51" t="n">
+      <c r="C6" s="52" t="n">
         <v>46113</v>
       </c>
       <c r="D6" s="45" t="inlineStr">
@@ -1180,7 +1180,7 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="51" t="n">
+      <c r="N6" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O6" s="45" t="inlineStr">
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>46204</v>
+        <v>46296</v>
       </c>
       <c r="D7" s="45" t="inlineStr">
         <is>
@@ -1234,19 +1234,19 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
+        <v>3.2217</v>
+      </c>
+      <c r="G7" s="41" t="n">
         <v>3.2721</v>
       </c>
-      <c r="G7" s="41" t="n">
+      <c r="H7" s="41" t="n">
         <v>1.54</v>
       </c>
-      <c r="H7" s="41" t="n">
+      <c r="I7" s="41" t="n">
         <v>1.2392</v>
       </c>
-      <c r="I7" s="41" t="n">
+      <c r="J7" s="41" t="n">
         <v>4.2373</v>
-      </c>
-      <c r="J7" s="41" t="n">
-        <v>3.4728</v>
       </c>
       <c r="K7" s="46" t="n"/>
       <c r="L7" s="28" t="inlineStr">
@@ -1259,7 +1259,7 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="51" t="n">
+      <c r="N7" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O7" s="45" t="inlineStr">
@@ -1299,7 +1299,7 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="51" t="n">
+      <c r="C8" s="52" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="45" t="inlineStr">
@@ -1338,7 +1338,7 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="51" t="n">
+      <c r="N8" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O8" s="45" t="inlineStr">
@@ -1379,7 +1379,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="D9" s="45" t="inlineStr">
         <is>
@@ -1392,19 +1392,19 @@
         </is>
       </c>
       <c r="F9" s="24" t="n">
+        <v>16944.918</v>
+      </c>
+      <c r="G9" s="24" t="n">
         <v>16788.685</v>
       </c>
-      <c r="G9" s="24" t="n">
+      <c r="H9" s="24" t="n">
         <v>16634.157</v>
       </c>
-      <c r="H9" s="24" t="n">
+      <c r="I9" s="24" t="n">
         <v>16604.582</v>
       </c>
-      <c r="I9" s="24" t="n">
+      <c r="J9" s="24" t="n">
         <v>16526.176</v>
-      </c>
-      <c r="J9" s="24" t="n">
-        <v>16378.319</v>
       </c>
       <c r="K9" s="46" t="n"/>
       <c r="L9" s="28" t="inlineStr">
@@ -1417,7 +1417,7 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="51" t="n">
+      <c r="N9" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O9" s="45" t="inlineStr">
@@ -1454,7 +1454,7 @@
         </is>
       </c>
       <c r="C10" s="51" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="D10" s="45" t="inlineStr">
         <is>
@@ -1467,19 +1467,19 @@
         </is>
       </c>
       <c r="F10" s="25" t="n">
+        <v>0.009305850934721915</v>
+      </c>
+      <c r="G10" s="25" t="n">
         <v>0.009289800499057588</v>
       </c>
-      <c r="G10" s="25" t="n">
+      <c r="H10" s="25" t="n">
         <v>0.001781134869881074</v>
       </c>
-      <c r="H10" s="25" t="n">
+      <c r="I10" s="25" t="n">
         <v>0.004744352232482596</v>
       </c>
-      <c r="I10" s="25" t="n">
+      <c r="J10" s="25" t="n">
         <v>0.00902760533605429</v>
-      </c>
-      <c r="J10" s="25" t="n">
-        <v>0.005218157797150624</v>
       </c>
       <c r="K10" s="46" t="n"/>
       <c r="L10" s="28" t="inlineStr">
@@ -1492,7 +1492,7 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="51" t="n">
+      <c r="N10" s="52" t="n">
         <v>46235</v>
       </c>
       <c r="O10" s="45" t="inlineStr">
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="C11" s="51" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="D11" s="45" t="inlineStr">
         <is>
@@ -1546,19 +1546,19 @@
         </is>
       </c>
       <c r="F11" s="25" t="n">
-        <v>0.01928463198493957</v>
+        <v>-0.007956600361663568</v>
       </c>
       <c r="G11" s="25" t="n">
-        <v>-0.01085475520029067</v>
+        <v>0.01682449204743941</v>
       </c>
       <c r="H11" s="25" t="n">
+        <v>-0.01199018984467259</v>
+      </c>
+      <c r="I11" s="25" t="n">
         <v>0.01023170451938515</v>
       </c>
-      <c r="I11" s="25" t="n">
+      <c r="J11" s="25" t="n">
         <v>0.007535133136094663</v>
-      </c>
-      <c r="J11" s="25" t="n">
-        <v>-0.003363280350149767</v>
       </c>
       <c r="K11" s="46" t="n"/>
       <c r="L11" s="28" t="inlineStr">
@@ -1571,7 +1571,7 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="51" t="n">
+      <c r="N11" s="52" t="n">
         <v>46235</v>
       </c>
       <c r="O11" s="45" t="inlineStr">
@@ -1608,7 +1608,7 @@
         </is>
       </c>
       <c r="C12" s="51" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="D12" s="45" t="inlineStr">
         <is>
@@ -1621,19 +1621,19 @@
         </is>
       </c>
       <c r="F12" s="25" t="n">
-        <v>0.04613572101790768</v>
+        <v>0.03246447727486591</v>
       </c>
       <c r="G12" s="25" t="n">
-        <v>0.02706908747936812</v>
+        <v>0.04241281809613572</v>
       </c>
       <c r="H12" s="25" t="n">
+        <v>0.02589012025465696</v>
+      </c>
+      <c r="I12" s="25" t="n">
         <v>0.04882579907588244</v>
       </c>
-      <c r="I12" s="25" t="n">
+      <c r="J12" s="25" t="n">
         <v>0.03805486759382744</v>
-      </c>
-      <c r="J12" s="25" t="n">
-        <v>0.009190576160485103</v>
       </c>
       <c r="K12" s="46" t="n"/>
       <c r="L12" s="28" t="inlineStr">
@@ -1646,7 +1646,7 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="51" t="n">
+      <c r="N12" s="52" t="n">
         <v>46235</v>
       </c>
       <c r="O12" s="45" t="inlineStr">
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="C13" s="51" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="D13" s="45" t="inlineStr">
         <is>
@@ -1700,19 +1700,19 @@
         </is>
       </c>
       <c r="F13" s="25" t="n">
-        <v>0.01016111828439903</v>
+        <v>-0.0002777700619427392</v>
       </c>
       <c r="G13" s="25" t="n">
-        <v>-0.001261528973115378</v>
+        <v>0.008346637537461676</v>
       </c>
       <c r="H13" s="25" t="n">
+        <v>0.000897087269771113</v>
+      </c>
+      <c r="I13" s="25" t="n">
         <v>0.003996735061499113</v>
       </c>
-      <c r="I13" s="25" t="n">
+      <c r="J13" s="25" t="n">
         <v>-0.001629808637985675</v>
-      </c>
-      <c r="J13" s="25" t="n">
-        <v>0.003524899892842992</v>
       </c>
       <c r="K13" s="46" t="n"/>
       <c r="L13" s="28" t="inlineStr">
@@ -1725,8 +1725,8 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="52" t="n">
-        <v>46307</v>
+      <c r="N13" s="51" t="n">
+        <v>46314</v>
       </c>
       <c r="O13" s="45" t="inlineStr">
         <is>
@@ -1742,16 +1742,16 @@
         <v>194000</v>
       </c>
       <c r="R13" s="24" t="n">
+        <v>195000</v>
+      </c>
+      <c r="S13" s="24" t="n">
         <v>200000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>198000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>199000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>198000</v>
       </c>
     </row>
     <row r="14">
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="C14" s="51" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="D14" s="45" t="inlineStr">
         <is>
@@ -1775,19 +1775,19 @@
         </is>
       </c>
       <c r="F14" s="25" t="n">
-        <v>0.0175587411994233</v>
+        <v>0.02116612285430555</v>
       </c>
       <c r="G14" s="25" t="n">
-        <v>0.01259130830230501</v>
+        <v>0.0179263154918427</v>
       </c>
       <c r="H14" s="25" t="n">
+        <v>0.01477986527584345</v>
+      </c>
+      <c r="I14" s="25" t="n">
         <v>0.01618095319488355</v>
       </c>
-      <c r="I14" s="25" t="n">
+      <c r="J14" s="25" t="n">
         <v>0.01924952665098396</v>
-      </c>
-      <c r="J14" s="25" t="n">
-        <v>0.0200647805772924</v>
       </c>
       <c r="K14" s="46" t="n"/>
       <c r="L14" s="28" t="inlineStr">
@@ -1800,8 +1800,8 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="52" t="n">
-        <v>46300</v>
+      <c r="N14" s="51" t="n">
+        <v>46307</v>
       </c>
       <c r="O14" s="45" t="inlineStr">
         <is>
@@ -1814,19 +1814,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1728000</v>
+        <v>1701000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1722000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1703000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1714000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1699000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1712000</v>
       </c>
     </row>
     <row r="15">
@@ -1841,7 +1841,7 @@
         </is>
       </c>
       <c r="C15" s="51" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="D15" s="45" t="inlineStr">
         <is>
@@ -1854,19 +1854,19 @@
         </is>
       </c>
       <c r="F15" s="25" t="n">
-        <v>0.001990031912223467</v>
+        <v>0.001562248924279919</v>
       </c>
       <c r="G15" s="25" t="n">
-        <v>0.002822674888980803</v>
+        <v>0.002891803572227847</v>
       </c>
       <c r="H15" s="25" t="n">
+        <v>0.004072202944930714</v>
+      </c>
+      <c r="I15" s="25" t="n">
         <v>0.003210504482080712</v>
       </c>
-      <c r="I15" s="25" t="n">
+      <c r="J15" s="25" t="n">
         <v>0.004265724765656786</v>
-      </c>
-      <c r="J15" s="25" t="n">
-        <v>0.004119604954438749</v>
       </c>
       <c r="K15" s="46" t="n"/>
       <c r="L15" s="28" t="inlineStr">
@@ -1879,7 +1879,7 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="51" t="n">
+      <c r="N15" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O15" s="45" t="inlineStr">
@@ -1916,7 +1916,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="D16" s="45" t="inlineStr">
         <is>
@@ -1929,19 +1929,19 @@
         </is>
       </c>
       <c r="F16" s="25" t="n">
-        <v>0.02497845104260272</v>
+        <v>0.02549266937223498</v>
       </c>
       <c r="G16" s="25" t="n">
-        <v>0.02472810111699007</v>
+        <v>0.02717919562785406</v>
       </c>
       <c r="H16" s="25" t="n">
+        <v>0.02600492357436805</v>
+      </c>
+      <c r="I16" s="25" t="n">
         <v>0.02657758254738746</v>
       </c>
-      <c r="I16" s="25" t="n">
+      <c r="J16" s="25" t="n">
         <v>0.02699799020107251</v>
-      </c>
-      <c r="J16" s="25" t="n">
-        <v>0.024229381371576</v>
       </c>
       <c r="K16" s="46" t="n"/>
       <c r="L16" s="28" t="n"/>
@@ -1966,7 +1966,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="51" t="n">
+      <c r="C17" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="D17" s="45" t="inlineStr">
@@ -2053,7 +2053,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="51" t="n">
+      <c r="C18" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="D18" s="45" t="inlineStr">
@@ -2092,7 +2092,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="51" t="n">
+      <c r="N18" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O18" s="45" t="inlineStr">
@@ -2133,7 +2133,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="D19" s="45" t="inlineStr">
         <is>
@@ -2146,19 +2146,19 @@
         </is>
       </c>
       <c r="F19" s="25" t="n">
-        <v>-0.000266081649054728</v>
+        <v>-0.002720430924946671</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>0.003104845738190587</v>
+        <v>0.0001140430431030293</v>
       </c>
       <c r="H19" s="25" t="n">
+        <v>0.003034033466968733</v>
+      </c>
+      <c r="I19" s="25" t="n">
         <v>0.003586110382227004</v>
       </c>
-      <c r="I19" s="25" t="n">
+      <c r="J19" s="25" t="n">
         <v>0.003340299146002312</v>
-      </c>
-      <c r="J19" s="25" t="n">
-        <v>-0.003808410193644085</v>
       </c>
       <c r="K19" s="46" t="n"/>
       <c r="L19" s="28" t="n"/>
@@ -2167,7 +2167,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="51" t="n">
+      <c r="N19" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O19" s="45" t="inlineStr">
@@ -2204,7 +2204,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="D20" s="45" t="inlineStr">
         <is>
@@ -2217,19 +2217,19 @@
         </is>
       </c>
       <c r="F20" s="25" t="n">
-        <v>0.01301309563112138</v>
+        <v>0.00953129551963138</v>
       </c>
       <c r="G20" s="25" t="n">
-        <v>0.01493573774828597</v>
+        <v>0.01332673049411251</v>
       </c>
       <c r="H20" s="25" t="n">
+        <v>0.01486409029783278</v>
+      </c>
+      <c r="I20" s="25" t="n">
         <v>0.01491547162301134</v>
       </c>
-      <c r="I20" s="25" t="n">
+      <c r="J20" s="25" t="n">
         <v>0.01221779548472771</v>
-      </c>
-      <c r="J20" s="25" t="n">
-        <v>0.002297953282280082</v>
       </c>
       <c r="K20" s="46" t="n"/>
       <c r="L20" s="28" t="inlineStr">
@@ -2242,7 +2242,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="51" t="n">
+      <c r="N20" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O20" s="45" t="inlineStr">
@@ -2283,7 +2283,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="D21" s="45" t="inlineStr">
         <is>
@@ -2296,13 +2296,13 @@
         </is>
       </c>
       <c r="F21" s="45" t="n">
-        <v>4.1</v>
+        <v>3.8</v>
       </c>
       <c r="G21" s="45" t="n">
-        <v>4.6</v>
+        <v>4</v>
       </c>
       <c r="H21" s="45" t="n">
-        <v>4.4</v>
+        <v>4.5</v>
       </c>
       <c r="I21" s="45" t="n">
         <v>4.4</v>
@@ -2317,7 +2317,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="51" t="n">
+      <c r="N21" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O21" s="45" t="inlineStr">
@@ -2357,7 +2357,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="51" t="n">
+      <c r="C22" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="D22" s="45" t="inlineStr">
@@ -2396,7 +2396,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="51" t="n">
+      <c r="N22" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O22" s="45" t="inlineStr">
@@ -2432,7 +2432,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="51" t="n">
+      <c r="C23" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="D23" s="45" t="inlineStr">
@@ -2466,7 +2466,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="51" t="n">
+      <c r="N23" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O23" s="45" t="inlineStr">
@@ -2506,7 +2506,7 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="51" t="n">
+      <c r="C24" s="52" t="n">
         <v>46235</v>
       </c>
       <c r="D24" s="45" t="inlineStr">
@@ -2546,7 +2546,7 @@
         </is>
       </c>
       <c r="N24" s="51" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="O24" s="45" t="inlineStr">
         <is>
@@ -2559,19 +2559,19 @@
         </is>
       </c>
       <c r="Q24" s="38" t="n">
-        <v>0.003102796328484869</v>
+        <v>0.004908404312709447</v>
       </c>
       <c r="R24" s="38" t="n">
-        <v>0.0005034094549449808</v>
+        <v>0.003232027563706552</v>
       </c>
       <c r="S24" s="38" t="n">
+        <v>0.0006178206947051734</v>
+      </c>
+      <c r="T24" s="38" t="n">
         <v>-0.001028641964020527</v>
       </c>
-      <c r="T24" s="38" t="n">
+      <c r="U24" s="23" t="n">
         <v>0.004354414105546933</v>
-      </c>
-      <c r="U24" s="23" t="n">
-        <v>0.004358018523500373</v>
       </c>
     </row>
     <row r="25">
@@ -2585,7 +2585,7 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="51" t="n">
+      <c r="C25" s="52" t="n">
         <v>46235</v>
       </c>
       <c r="D25" s="45" t="inlineStr">
@@ -2621,7 +2621,7 @@
         </is>
       </c>
       <c r="N25" s="51" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="O25" s="45" t="inlineStr">
         <is>
@@ -2634,19 +2634,19 @@
         </is>
       </c>
       <c r="Q25" s="38" t="n">
-        <v>0.03419031824505426</v>
+        <v>0.03648874225123632</v>
       </c>
       <c r="R25" s="38" t="n">
-        <v>0.033615431894473</v>
+        <v>0.03444183322984532</v>
       </c>
       <c r="S25" s="38" t="n">
+        <v>0.03373362961562106</v>
+      </c>
+      <c r="T25" s="38" t="n">
         <v>0.03453010336936787</v>
       </c>
-      <c r="T25" s="38" t="n">
+      <c r="U25" s="23" t="n">
         <v>0.0382333396620468</v>
-      </c>
-      <c r="U25" s="23" t="n">
-        <v>0.03573947987920389</v>
       </c>
     </row>
     <row r="26">
@@ -2661,7 +2661,7 @@
         </is>
       </c>
       <c r="C26" s="51" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="D26" s="45" t="inlineStr">
         <is>
@@ -2674,19 +2674,19 @@
         </is>
       </c>
       <c r="F26" s="38" t="n">
+        <v>0.03040374576676874</v>
+      </c>
+      <c r="G26" s="38" t="n">
         <v>0.02173921402703938</v>
       </c>
-      <c r="G26" s="38" t="n">
+      <c r="H26" s="38" t="n">
         <v>0.02391240953315132</v>
       </c>
-      <c r="H26" s="38" t="n">
+      <c r="I26" s="38" t="n">
         <v>0.005295862445843902</v>
       </c>
-      <c r="I26" s="38" t="n">
+      <c r="J26" s="38" t="n">
         <v>0.009411852445720736</v>
-      </c>
-      <c r="J26" s="38" t="n">
-        <v>0.01849694172720051</v>
       </c>
       <c r="K26" s="46" t="n"/>
       <c r="L26" s="28" t="inlineStr">
@@ -2700,7 +2700,7 @@
         </is>
       </c>
       <c r="N26" s="51" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="O26" s="45" t="inlineStr">
         <is>
@@ -2713,19 +2713,19 @@
         </is>
       </c>
       <c r="Q26" s="38" t="n">
-        <v>0.002474391583994873</v>
+        <v>0.003165017740958787</v>
       </c>
       <c r="R26" s="38" t="n">
-        <v>0.001261839361694106</v>
+        <v>0.002620094046777544</v>
       </c>
       <c r="S26" s="38" t="n">
+        <v>0.001377251498434262</v>
+      </c>
+      <c r="T26" s="38" t="n">
         <v>0.001332860796942947</v>
       </c>
-      <c r="T26" s="38" t="n">
+      <c r="U26" s="23" t="n">
         <v>0.003099037829900508</v>
-      </c>
-      <c r="U26" s="23" t="n">
-        <v>0.002828799503991286</v>
       </c>
     </row>
     <row r="27">
@@ -2740,7 +2740,7 @@
         </is>
       </c>
       <c r="C27" s="51" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="D27" s="45" t="inlineStr">
         <is>
@@ -2753,19 +2753,19 @@
         </is>
       </c>
       <c r="F27" s="38" t="n">
+        <v>-0.008462060110915437</v>
+      </c>
+      <c r="G27" s="38" t="n">
         <v>0.006940517752098252</v>
       </c>
-      <c r="G27" s="38" t="n">
+      <c r="H27" s="38" t="n">
         <v>-0.01948561470458643</v>
       </c>
-      <c r="H27" s="38" t="n">
+      <c r="I27" s="38" t="n">
         <v>-0.004482704112548475</v>
       </c>
-      <c r="I27" s="38" t="n">
+      <c r="J27" s="38" t="n">
         <v>-0.01618651426201678</v>
-      </c>
-      <c r="J27" s="38" t="n">
-        <v>-0.01101732062248628</v>
       </c>
       <c r="K27" s="46" t="n"/>
       <c r="L27" s="28" t="n"/>
@@ -2775,7 +2775,7 @@
         </is>
       </c>
       <c r="N27" s="51" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="O27" s="45" t="inlineStr">
         <is>
@@ -2788,19 +2788,19 @@
         </is>
       </c>
       <c r="Q27" s="38" t="n">
-        <v>0.03007595976185597</v>
+        <v>0.03121159602962021</v>
       </c>
       <c r="R27" s="38" t="n">
-        <v>0.02983468262070393</v>
+        <v>0.03034442461664801</v>
       </c>
       <c r="S27" s="38" t="n">
+        <v>0.0299533882544732</v>
+      </c>
+      <c r="T27" s="38" t="n">
         <v>0.03041234252733225</v>
       </c>
-      <c r="T27" s="38" t="n">
+      <c r="U27" s="23" t="n">
         <v>0.0316170977125689</v>
-      </c>
-      <c r="U27" s="23" t="n">
-        <v>0.03083872406870407</v>
       </c>
     </row>
     <row r="28">
@@ -2814,7 +2814,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="52" t="n">
+      <c r="C28" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="D28" s="45" t="inlineStr">
@@ -2853,7 +2853,7 @@
           <t>MICH</t>
         </is>
       </c>
-      <c r="N28" s="51" t="n">
+      <c r="N28" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O28" s="45" t="inlineStr">
@@ -2889,7 +2889,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="52" t="n">
+      <c r="C29" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="D29" s="45" t="inlineStr">
@@ -2928,8 +2928,8 @@
           <t>T5YIFR</t>
         </is>
       </c>
-      <c r="N29" s="52" t="n">
-        <v>46322</v>
+      <c r="N29" s="51" t="n">
+        <v>46323</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2942,19 +2942,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.25</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.2</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.19</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.34</v>
       </c>
     </row>
     <row r="30">
@@ -2968,7 +2968,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="52" t="n">
+      <c r="C30" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="D30" s="45" t="inlineStr">
@@ -3007,8 +3007,8 @@
           <t>T10YIE</t>
         </is>
       </c>
-      <c r="N30" s="52" t="n">
-        <v>46322</v>
+      <c r="N30" s="51" t="n">
+        <v>46323</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3021,19 +3021,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.35</v>
-      </c>
-      <c r="R30" s="45" t="n">
-        <v>2.34</v>
       </c>
       <c r="S30" s="45" t="n">
         <v>2.34</v>
       </c>
       <c r="T30" s="45" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="U30" s="21" t="n">
         <v>2.32</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.37</v>
       </c>
     </row>
     <row r="31">
@@ -3043,7 +3043,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="52" t="n">
+      <c r="C31" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="D31" s="45" t="inlineStr">
@@ -3082,7 +3082,7 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N31" s="51" t="n">
+      <c r="N31" s="52" t="n">
         <v>46113</v>
       </c>
       <c r="O31" s="45" t="inlineStr">
@@ -3122,7 +3122,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="51" t="n">
+      <c r="C32" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="D32" s="45" t="inlineStr">
@@ -3157,7 +3157,7 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N32" s="51" t="n">
+      <c r="N32" s="52" t="n">
         <v>46113</v>
       </c>
       <c r="O32" s="45" t="inlineStr">
@@ -3193,7 +3193,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="51" t="n">
+      <c r="C33" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="D33" s="45" t="inlineStr">
@@ -3232,7 +3232,7 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="51" t="n">
+      <c r="N33" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O33" s="45" t="inlineStr">
@@ -3272,7 +3272,7 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="51" t="n">
+      <c r="C34" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="D34" s="45" t="inlineStr">
@@ -3307,8 +3307,8 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N34" s="51" t="n">
-        <v>46235</v>
+      <c r="N34" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O34" s="45" t="inlineStr">
         <is>
@@ -3321,19 +3321,19 @@
         </is>
       </c>
       <c r="Q34" s="38" t="n">
-        <v>-0.002958631913215778</v>
+        <v>-0.006023712934928774</v>
       </c>
       <c r="R34" s="38" t="n">
-        <v>-0.001484371505816307</v>
+        <v>-0.003201053320079647</v>
       </c>
       <c r="S34" s="38" t="n">
+        <v>-0.001598542379663732</v>
+      </c>
+      <c r="T34" s="38" t="n">
         <v>-0.0006782988032908383</v>
       </c>
-      <c r="T34" s="38" t="n">
+      <c r="U34" s="23" t="n">
         <v>-0.004701862813512956</v>
-      </c>
-      <c r="U34" s="23" t="n">
-        <v>-2.432480889988557e-05</v>
       </c>
     </row>
     <row r="35" ht="31.5" customHeight="1">
@@ -3347,7 +3347,7 @@
           <t>PRS85006092</t>
         </is>
       </c>
-      <c r="C35" s="51" t="n">
+      <c r="C35" s="52" t="n">
         <v>46113</v>
       </c>
       <c r="D35" s="45" t="inlineStr">
@@ -3386,8 +3386,8 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N35" s="51" t="n">
-        <v>46235</v>
+      <c r="N35" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O35" s="45" t="inlineStr">
         <is>
@@ -3400,19 +3400,19 @@
         </is>
       </c>
       <c r="Q35" s="38" t="n">
-        <v>8.50375855385721e-05</v>
+        <v>-0.003566744745047701</v>
       </c>
       <c r="R35" s="38" t="n">
-        <v>0.0008263155649324005</v>
+        <v>-4.378827047801792e-05</v>
       </c>
       <c r="S35" s="38" t="n">
+        <v>0.0007118804857439986</v>
+      </c>
+      <c r="T35" s="38" t="n">
         <v>0.003699825727481398</v>
       </c>
-      <c r="T35" s="38" t="n">
+      <c r="U35" s="23" t="n">
         <v>-0.002206341131705591</v>
-      </c>
-      <c r="U35" s="23" t="n">
-        <v>-0.002739653360595784</v>
       </c>
     </row>
     <row r="36" ht="31.5" customHeight="1">
@@ -3426,7 +3426,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="51" t="n">
+      <c r="C36" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="D36" s="45" t="inlineStr">
@@ -3461,8 +3461,8 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N36" s="51" t="n">
-        <v>46235</v>
+      <c r="N36" s="52" t="n">
+        <v>46266</v>
       </c>
       <c r="O36" s="45" t="inlineStr">
         <is>
@@ -3475,19 +3475,19 @@
         </is>
       </c>
       <c r="Q36" s="38" t="n">
-        <v>-0.002958631913215778</v>
+        <v>-0.006023712934928774</v>
       </c>
       <c r="R36" s="38" t="n">
-        <v>-0.001484371505816307</v>
+        <v>-0.003201053320079647</v>
       </c>
       <c r="S36" s="38" t="n">
+        <v>-0.001598542379663732</v>
+      </c>
+      <c r="T36" s="38" t="n">
         <v>-0.0006782988032908383</v>
       </c>
-      <c r="T36" s="38" t="n">
+      <c r="U36" s="23" t="n">
         <v>-0.004701862813512956</v>
-      </c>
-      <c r="U36" s="23" t="n">
-        <v>-2.432480889988557e-05</v>
       </c>
     </row>
     <row r="37">
@@ -3497,7 +3497,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="51" t="n">
+      <c r="C37" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="D37" s="45" t="inlineStr">
@@ -3536,7 +3536,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="52" t="n">
+      <c r="N37" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O37" s="45" t="inlineStr">
@@ -3576,7 +3576,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="51" t="n">
+      <c r="C38" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="D38" s="45" t="inlineStr">
@@ -3611,7 +3611,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="52" t="n">
+      <c r="N38" s="51" t="n">
         <v>46235</v>
       </c>
       <c r="O38" s="45" t="inlineStr">
@@ -3647,7 +3647,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="51" t="n">
+      <c r="C39" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="D39" s="45" t="inlineStr">
@@ -3686,7 +3686,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="51" t="n">
+      <c r="N39" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O39" s="45" t="inlineStr">
@@ -3726,7 +3726,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="52" t="n">
+      <c r="C40" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="D40" s="45" t="inlineStr">
@@ -3761,7 +3761,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="51" t="n">
+      <c r="N40" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O40" s="45" t="inlineStr">
@@ -3797,7 +3797,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="52" t="n">
+      <c r="C41" s="51" t="n">
         <v>46266</v>
       </c>
       <c r="D41" s="45" t="inlineStr">
@@ -3836,7 +3836,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="51" t="n">
+      <c r="N41" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O41" s="45" t="inlineStr">
@@ -3876,7 +3876,7 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C42" s="51" t="n">
+      <c r="C42" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="D42" s="45" t="inlineStr">
@@ -3911,7 +3911,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="51" t="n">
+      <c r="N42" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O42" s="45" t="inlineStr">
@@ -3947,7 +3947,7 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C43" s="51" t="n">
+      <c r="C43" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="D43" s="45" t="inlineStr">
@@ -3986,7 +3986,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="51" t="n">
+      <c r="N43" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O43" s="45" t="inlineStr">
@@ -4027,7 +4027,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="D44" s="45" t="inlineStr">
         <is>
@@ -4040,19 +4040,19 @@
         </is>
       </c>
       <c r="F44" s="24" t="n">
+        <v>5772.578</v>
+      </c>
+      <c r="G44" s="24" t="n">
         <v>5626.646</v>
       </c>
-      <c r="G44" s="24" t="n">
+      <c r="H44" s="24" t="n">
         <v>5483.833</v>
       </c>
-      <c r="H44" s="24" t="n">
+      <c r="I44" s="24" t="n">
         <v>5409.276</v>
       </c>
-      <c r="I44" s="24" t="n">
+      <c r="J44" s="24" t="n">
         <v>5404.135</v>
-      </c>
-      <c r="J44" s="24" t="n">
-        <v>5332.951</v>
       </c>
       <c r="K44" s="46" t="n"/>
       <c r="L44" s="28" t="n"/>
@@ -4061,7 +4061,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="51" t="n">
+      <c r="N44" s="52" t="n">
         <v>46266</v>
       </c>
       <c r="O44" s="45" t="inlineStr">
@@ -4098,7 +4098,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="D45" s="45" t="inlineStr">
         <is>
@@ -4111,19 +4111,19 @@
         </is>
       </c>
       <c r="F45" s="38" t="n">
+        <v>0.02593587725262991</v>
+      </c>
+      <c r="G45" s="38" t="n">
         <v>0.0260425508946025</v>
       </c>
-      <c r="G45" s="38" t="n">
+      <c r="H45" s="38" t="n">
         <v>0.0137831754194091</v>
       </c>
-      <c r="H45" s="38" t="n">
+      <c r="I45" s="38" t="n">
         <v>0.0009513085812993261</v>
       </c>
-      <c r="I45" s="38" t="n">
+      <c r="J45" s="38" t="n">
         <v>0.01334795688165902</v>
-      </c>
-      <c r="J45" s="38" t="n">
-        <v>0.0111412368534316</v>
       </c>
       <c r="K45" s="46" t="n"/>
       <c r="L45" s="28" t="n"/>
@@ -4148,7 +4148,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="51" t="n">
+      <c r="C46" s="52" t="n">
         <v>46235</v>
       </c>
       <c r="D46" s="45" t="inlineStr">
@@ -4235,7 +4235,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="51" t="n">
+      <c r="C47" s="52" t="n">
         <v>46235</v>
       </c>
       <c r="D47" s="45" t="inlineStr">
@@ -4274,8 +4274,8 @@
           <t>DFF</t>
         </is>
       </c>
-      <c r="N47" s="52" t="n">
-        <v>46321</v>
+      <c r="N47" s="51" t="n">
+        <v>46322</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4314,7 +4314,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="51" t="n">
+      <c r="C48" s="52" t="n">
         <v>46235</v>
       </c>
       <c r="D48" s="45" t="inlineStr">
@@ -4353,8 +4353,8 @@
           <t>DGS2</t>
         </is>
       </c>
-      <c r="N48" s="52" t="n">
-        <v>46321</v>
+      <c r="N48" s="51" t="n">
+        <v>46322</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4367,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.68</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.69</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.65</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.81</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.79</v>
       </c>
     </row>
     <row r="49">
@@ -4389,7 +4389,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="51" t="n">
+      <c r="C49" s="52" t="n">
         <v>46235</v>
       </c>
       <c r="D49" s="45" t="inlineStr">
@@ -4428,8 +4428,8 @@
           <t>DGS5</t>
         </is>
       </c>
-      <c r="N49" s="52" t="n">
-        <v>46321</v>
+      <c r="N49" s="51" t="n">
+        <v>46322</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4442,19 +4442,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.84</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.82</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.78</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.95</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.94</v>
       </c>
     </row>
     <row r="50">
@@ -4468,7 +4468,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="51" t="n">
+      <c r="C50" s="52" t="n">
         <v>46235</v>
       </c>
       <c r="D50" s="45" t="inlineStr">
@@ -4507,8 +4507,8 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="52" t="n">
-        <v>46321</v>
+      <c r="N50" s="51" t="n">
+        <v>46322</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4521,19 +4521,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="R50" s="45" t="n">
         <v>5</v>
       </c>
       <c r="S50" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="T50" s="45" t="n">
         <v>4.96</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>5.13</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>5.12</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4543,7 +4543,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="51" t="n">
+      <c r="C51" s="52" t="n">
         <v>46235</v>
       </c>
       <c r="D51" s="45" t="inlineStr">
@@ -4582,8 +4582,8 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="52" t="n">
-        <v>46314</v>
+      <c r="N51" s="51" t="n">
+        <v>46321</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
         <is>
@@ -4596,19 +4596,19 @@
         </is>
       </c>
       <c r="Q51" s="45" t="n">
+        <v>7.24</v>
+      </c>
+      <c r="R51" s="45" t="n">
         <v>7.32</v>
-      </c>
-      <c r="R51" s="45" t="n">
-        <v>7.4</v>
       </c>
       <c r="S51" s="45" t="n">
         <v>7.4</v>
       </c>
       <c r="T51" s="45" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="U51" s="21" t="n">
         <v>7.28</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>7.03</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="N52" s="57" t="n">
-        <v>46321</v>
+        <v>46323</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4647,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.48</v>
+      </c>
+      <c r="R52" s="9" t="n">
+        <v>6.44</v>
+      </c>
+      <c r="S52" s="9" t="n">
         <v>6.45</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.47</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.42</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>6.57</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.56</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-10-30
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="N29" s="51" t="n">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2942,19 +2942,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.27</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.25</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.2</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.19</v>
       </c>
     </row>
     <row r="30">
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="N30" s="51" t="n">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3021,19 +3021,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.38</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.35</v>
-      </c>
-      <c r="S30" s="45" t="n">
-        <v>2.34</v>
       </c>
       <c r="T30" s="45" t="n">
         <v>2.34</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.32</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="31">
@@ -3082,8 +3082,8 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N31" s="52" t="n">
-        <v>46113</v>
+      <c r="N31" s="51" t="n">
+        <v>46204</v>
       </c>
       <c r="O31" s="45" t="inlineStr">
         <is>
@@ -3096,19 +3096,19 @@
         </is>
       </c>
       <c r="Q31" s="38" t="n">
+        <v>0.007776101893748999</v>
+      </c>
+      <c r="R31" s="38" t="n">
         <v>0.008518405841192678</v>
       </c>
-      <c r="R31" s="38" t="n">
+      <c r="S31" s="38" t="n">
         <v>0.007177997310378714</v>
       </c>
-      <c r="S31" s="38" t="n">
+      <c r="T31" s="38" t="n">
         <v>0.007345039668930076</v>
       </c>
-      <c r="T31" s="38" t="n">
+      <c r="U31" s="23" t="n">
         <v>0.007979811365325773</v>
-      </c>
-      <c r="U31" s="23" t="n">
-        <v>0.01026193247962737</v>
       </c>
     </row>
     <row r="32">
@@ -3157,8 +3157,8 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N32" s="52" t="n">
-        <v>46113</v>
+      <c r="N32" s="51" t="n">
+        <v>46204</v>
       </c>
       <c r="O32" s="45" t="inlineStr">
         <is>
@@ -3171,19 +3171,19 @@
         </is>
       </c>
       <c r="Q32" s="38" t="n">
+        <v>0.03117497770766159</v>
+      </c>
+      <c r="R32" s="38" t="n">
         <v>0.03138341697251144</v>
       </c>
-      <c r="R32" s="38" t="n">
+      <c r="S32" s="38" t="n">
         <v>0.03316647264260756</v>
       </c>
-      <c r="S32" s="38" t="n">
+      <c r="T32" s="38" t="n">
         <v>0.03362463343108507</v>
       </c>
-      <c r="T32" s="38" t="n">
+      <c r="U32" s="23" t="n">
         <v>0.0358081705150977</v>
-      </c>
-      <c r="U32" s="23" t="n">
-        <v>0.03557875894988063</v>
       </c>
     </row>
     <row r="33" ht="31.5" customHeight="1">
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="N47" s="51" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="N48" s="51" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4367,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.7</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.68</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.69</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.65</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.81</v>
       </c>
     </row>
     <row r="49">
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="N49" s="51" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4442,19 +4442,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.82</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.84</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.82</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.78</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.95</v>
       </c>
     </row>
     <row r="50">
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="N50" s="51" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4521,19 +4521,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.99</v>
-      </c>
-      <c r="R50" s="45" t="n">
-        <v>5</v>
       </c>
       <c r="S50" s="45" t="n">
         <v>5</v>
       </c>
       <c r="T50" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="U50" s="21" t="n">
         <v>4.96</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>5.13</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="N52" s="57" t="n">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4647,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.47</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.48</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.44</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.45</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.47</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.42</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>